<commit_message>
Model bottles from historic actuals; guide now equals blended low case
- New Bottles sheet in the Brand Pro Forma: monthly actuals 2023-Jul 2026
  from management's sales export (R1.03m 2024, R1.95m 2025, R1.54m Jan-Jul
  2026); Aug-Dec 2026 projected at the observed +4.4% YoY, 2027 held to a
  conservative +5% (vs +89% in 2025); gross margin a stated 30% placeholder
  pending cost data
- Combined pro forma: R16.07m revenue to Dec 27, R4.63m EBITDA (28.8%),
  peak funding need R1.51m, blended valuation R15.0m/R21.4m/R29.6m — the
  ~R15m guide now equals the blended low case
- Revenue chart stacked cans + bottles with legend; cash curve updated;
  P&L and valuation tables carry the combined numbers; copy updated
  site-wide (bottles now in the projections)
- All workbook outputs verified by independent formula evaluation

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hyws6xeXfxtGdqZV2paNDe
</commit_message>
<xml_diff>
--- a/site/downloads/Dona-Fuego-Brand-Pro-Forma.xlsx
+++ b/site/downloads/Dona-Fuego-Brand-Pro-Forma.xlsx
@@ -1,17 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P&amp;L" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cashflow" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Assumptions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Bottles" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="P&amp;L" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cashflow" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Valuation" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Summary" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -106,14 +107,14 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="17" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -494,14 +495,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ASSUMPTIONS — Doña Fuego Brand Pro Forma (cans only)</t>
+          <t>ASSUMPTIONS — Doña Fuego Brand Pro Forma (cans + bottles)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Brand entity scope: Doña Fuego cans. Fuego Tequila bottles NOT yet modelled (sales data pending) — upside.</t>
+          <t>Brand entity scope: Doña Fuego cans + Fuego Tequila bottles (Bottles sheet, from historic actuals).</t>
         </is>
       </c>
     </row>
@@ -663,7 +664,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>COGS build (% of revenue)</t>
+          <t>Can COGS build (% of revenue)</t>
         </is>
       </c>
     </row>
@@ -725,7 +726,7 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Total COGS ratio</t>
+          <t>Total can COGS ratio</t>
         </is>
       </c>
       <c r="B21" s="12">
@@ -789,7 +790,426 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:G24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>FUEGO TEQUILA BOTTLES — historic sales &amp; projection</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Historic revenue per management sales export (bottle &amp; mini, 2023–Jul 2026), received Aug 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>2027 (proj)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="n">
+        <v>87354</v>
+      </c>
+      <c r="D4" s="9" t="n">
+        <v>107377.8</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>185865.3</v>
+      </c>
+      <c r="G4" s="14">
+        <f>(D4+E4)/($D$16+$E$16)*$B$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>February</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>7728</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>46920</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>209857.2</v>
+      </c>
+      <c r="G5" s="14">
+        <f>(D5+E5)/($D$16+$E$16)*$B$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>March</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>126617.4</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>260918.59</v>
+      </c>
+      <c r="G6" s="14">
+        <f>(D6+E6)/($D$16+$E$16)*$B$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>April</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>21931.51</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>663918</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>470561.32</v>
+      </c>
+      <c r="G7" s="14">
+        <f>(D7+E7)/($D$16+$E$16)*$B$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>1895.8</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>168670.5</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>167687.8</v>
+      </c>
+      <c r="G8" s="14">
+        <f>(D8+E8)/($D$16+$E$16)*$B$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>June</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>68533.21000000001</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>98574.11</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>60059.82</v>
+      </c>
+      <c r="G9" s="14">
+        <f>(D9+E9)/($D$16+$E$16)*$B$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>July</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>36027.3</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>266641.05</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>188654.34</v>
+      </c>
+      <c r="G10" s="14">
+        <f>(D10+E10)/($D$16+$E$16)*$B$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>August</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>5796</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>44441.56</v>
+      </c>
+      <c r="E11" s="14">
+        <f>D11*$B$19</f>
+        <v/>
+      </c>
+      <c r="G11" s="14">
+        <f>(D11+E11)/($D$16+$E$16)*$B$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>September</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>1334</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>46252.59</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>65847.11</v>
+      </c>
+      <c r="E12" s="14">
+        <f>D12*$B$19</f>
+        <v/>
+      </c>
+      <c r="G12" s="14">
+        <f>(D12+E12)/($D$16+$E$16)*$B$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>October</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>2894</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>530949.8100000001</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>63268.38</v>
+      </c>
+      <c r="E13" s="14">
+        <f>D13*$B$19</f>
+        <v/>
+      </c>
+      <c r="G13" s="14">
+        <f>(D13+E13)/($D$16+$E$16)*$B$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>November</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>81964.75</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>257848.55</v>
+      </c>
+      <c r="E14" s="14">
+        <f>D14*$B$19</f>
+        <v/>
+      </c>
+      <c r="G14" s="14">
+        <f>(D14+E14)/($D$16+$E$16)*$B$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>December</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="n">
+        <v>21919</v>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>138333.09</v>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>35332.6</v>
+      </c>
+      <c r="E15" s="14">
+        <f>D15*$B$19</f>
+        <v/>
+      </c>
+      <c r="G15" s="14">
+        <f>(D15+E15)/($D$16+$E$16)*$B$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Annual total</t>
+        </is>
+      </c>
+      <c r="B16" s="15">
+        <f>SUM(B4:B15)</f>
+        <v/>
+      </c>
+      <c r="C16" s="15">
+        <f>SUM(C4:C15)</f>
+        <v/>
+      </c>
+      <c r="D16" s="15">
+        <f>SUM(D4:D15)</f>
+        <v/>
+      </c>
+      <c r="E16" s="15">
+        <f>SUM(E4:E15)</f>
+        <v/>
+      </c>
+      <c r="G16" s="15">
+        <f>SUM(G4:G15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Projection assumptions</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>YoY growth (Jan-Jul 26 vs Jan-Jul 25)</t>
+        </is>
+      </c>
+      <c r="B19" s="12">
+        <f>SUM(E4:E10)/SUM(D4:D10)</f>
+        <v/>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Applied to 2025 actuals for Aug-Dec 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>2027 growth on 2026</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>CONSERVATIVE vs +89% (2025) and +4.4% YTD (2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>2027 total</t>
+        </is>
+      </c>
+      <c r="B21" s="14">
+        <f>E16*(1+B20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Bottle gross margin %</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER matching cans — awaiting bottle cost data from management</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2026 cells Aug-Dec are projections (2025 month x B19); 2027 monthly = blended 2025+2026 seasonality x B21.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -817,7 +1237,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>P&amp;L (ACCRUAL) — Doña Fuego cans</t>
+          <t>P&amp;L (ACCRUAL) — Doña Fuego cans + Fuego Tequila bottles</t>
         </is>
       </c>
     </row>
@@ -827,61 +1247,61 @@
           <t>Month</t>
         </is>
       </c>
-      <c r="B3" s="14" t="n">
+      <c r="B3" s="16" t="n">
         <v>46174</v>
       </c>
-      <c r="C3" s="14" t="n">
+      <c r="C3" s="16" t="n">
         <v>46204</v>
       </c>
-      <c r="D3" s="14" t="n">
+      <c r="D3" s="16" t="n">
         <v>46235</v>
       </c>
-      <c r="E3" s="14" t="n">
+      <c r="E3" s="16" t="n">
         <v>46266</v>
       </c>
-      <c r="F3" s="14" t="n">
+      <c r="F3" s="16" t="n">
         <v>46296</v>
       </c>
-      <c r="G3" s="14" t="n">
+      <c r="G3" s="16" t="n">
         <v>46327</v>
       </c>
-      <c r="H3" s="14" t="n">
+      <c r="H3" s="16" t="n">
         <v>46357</v>
       </c>
-      <c r="I3" s="14" t="n">
+      <c r="I3" s="16" t="n">
         <v>46388</v>
       </c>
-      <c r="J3" s="14" t="n">
+      <c r="J3" s="16" t="n">
         <v>46419</v>
       </c>
-      <c r="K3" s="14" t="n">
+      <c r="K3" s="16" t="n">
         <v>46447</v>
       </c>
-      <c r="L3" s="14" t="n">
+      <c r="L3" s="16" t="n">
         <v>46478</v>
       </c>
-      <c r="M3" s="14" t="n">
+      <c r="M3" s="16" t="n">
         <v>46508</v>
       </c>
-      <c r="N3" s="14" t="n">
+      <c r="N3" s="16" t="n">
         <v>46539</v>
       </c>
-      <c r="O3" s="14" t="n">
+      <c r="O3" s="16" t="n">
         <v>46569</v>
       </c>
-      <c r="P3" s="14" t="n">
+      <c r="P3" s="16" t="n">
         <v>46600</v>
       </c>
-      <c r="Q3" s="14" t="n">
+      <c r="Q3" s="16" t="n">
         <v>46631</v>
       </c>
-      <c r="R3" s="14" t="n">
+      <c r="R3" s="16" t="n">
         <v>46661</v>
       </c>
-      <c r="S3" s="14" t="n">
+      <c r="S3" s="16" t="n">
         <v>46692</v>
       </c>
-      <c r="T3" s="14" t="n">
+      <c r="T3" s="16" t="n">
         <v>46722</v>
       </c>
       <c r="U3" s="3" t="inlineStr">
@@ -893,83 +1313,83 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Cases delivered</t>
-        </is>
-      </c>
-      <c r="B4" s="15" t="n">
+          <t>Cases delivered (cans)</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="C4" s="15" t="n">
+      <c r="C4" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="16">
+      <c r="D4" s="18">
         <f>Assumptions!B7</f>
         <v/>
       </c>
-      <c r="E4" s="15" t="n">
+      <c r="E4" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="16">
+      <c r="F4" s="18">
         <f>Assumptions!B8</f>
         <v/>
       </c>
-      <c r="G4" s="16">
+      <c r="G4" s="18">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="H4" s="16">
+      <c r="H4" s="18">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="I4" s="16">
+      <c r="I4" s="18">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="J4" s="16">
+      <c r="J4" s="18">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="K4" s="16">
+      <c r="K4" s="18">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="L4" s="16">
+      <c r="L4" s="18">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="M4" s="16">
+      <c r="M4" s="18">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="N4" s="16">
+      <c r="N4" s="18">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="O4" s="16">
+      <c r="O4" s="18">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="P4" s="16">
+      <c r="P4" s="18">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="Q4" s="16">
+      <c r="Q4" s="18">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="R4" s="16">
+      <c r="R4" s="18">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="S4" s="16">
+      <c r="S4" s="18">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="T4" s="16">
+      <c r="T4" s="18">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="U4" s="17">
+      <c r="U4" s="19">
         <f>SUM(B4:T4)</f>
         <v/>
       </c>
@@ -977,86 +1397,86 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Revenue</t>
-        </is>
-      </c>
-      <c r="B5" s="18">
+          <t>Can revenue</t>
+        </is>
+      </c>
+      <c r="B5" s="14">
         <f>B4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="C5" s="18">
+      <c r="C5" s="14">
         <f>C4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="D5" s="18">
+      <c r="D5" s="14">
         <f>D4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="E5" s="18">
+      <c r="E5" s="14">
         <f>E4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="F5" s="18">
+      <c r="F5" s="14">
         <f>F4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="G5" s="18">
+      <c r="G5" s="14">
         <f>G4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="H5" s="18">
+      <c r="H5" s="14">
         <f>H4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="I5" s="18">
+      <c r="I5" s="14">
         <f>I4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="J5" s="18">
+      <c r="J5" s="14">
         <f>J4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="K5" s="18">
+      <c r="K5" s="14">
         <f>K4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="L5" s="18">
+      <c r="L5" s="14">
         <f>L4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="M5" s="18">
+      <c r="M5" s="14">
         <f>M4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="N5" s="18">
+      <c r="N5" s="14">
         <f>N4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="O5" s="18">
+      <c r="O5" s="14">
         <f>O4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="P5" s="18">
+      <c r="P5" s="14">
         <f>P4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="Q5" s="18">
+      <c r="Q5" s="14">
         <f>Q4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="R5" s="18">
+      <c r="R5" s="14">
         <f>R4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="S5" s="18">
+      <c r="S5" s="14">
         <f>S4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="T5" s="18">
+      <c r="T5" s="14">
         <f>T4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="U5" s="19">
+      <c r="U5" s="15">
         <f>SUM(B5:T5)</f>
         <v/>
       </c>
@@ -1064,86 +1484,86 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>COGS (70% of revenue)</t>
-        </is>
-      </c>
-      <c r="B6" s="18">
-        <f>-B5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="C6" s="18">
-        <f>-C5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="D6" s="18">
-        <f>-D5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="E6" s="18">
-        <f>-E5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="F6" s="18">
-        <f>-F5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="G6" s="18">
-        <f>-G5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="H6" s="18">
-        <f>-H5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="I6" s="18">
-        <f>-I5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="J6" s="18">
-        <f>-J5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="K6" s="18">
-        <f>-K5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="L6" s="18">
-        <f>-L5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="M6" s="18">
-        <f>-M5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="N6" s="18">
-        <f>-N5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="O6" s="18">
-        <f>-O5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="P6" s="18">
-        <f>-P5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="Q6" s="18">
-        <f>-Q5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="R6" s="18">
-        <f>-R5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="S6" s="18">
-        <f>-S5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="T6" s="18">
-        <f>-T5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="U6" s="19">
+          <t>Bottle revenue</t>
+        </is>
+      </c>
+      <c r="B6" s="20">
+        <f>Bottles!E9</f>
+        <v/>
+      </c>
+      <c r="C6" s="20">
+        <f>Bottles!E10</f>
+        <v/>
+      </c>
+      <c r="D6" s="20">
+        <f>Bottles!E11</f>
+        <v/>
+      </c>
+      <c r="E6" s="20">
+        <f>Bottles!E12</f>
+        <v/>
+      </c>
+      <c r="F6" s="20">
+        <f>Bottles!E13</f>
+        <v/>
+      </c>
+      <c r="G6" s="20">
+        <f>Bottles!E14</f>
+        <v/>
+      </c>
+      <c r="H6" s="20">
+        <f>Bottles!E15</f>
+        <v/>
+      </c>
+      <c r="I6" s="20">
+        <f>Bottles!G4</f>
+        <v/>
+      </c>
+      <c r="J6" s="20">
+        <f>Bottles!G5</f>
+        <v/>
+      </c>
+      <c r="K6" s="20">
+        <f>Bottles!G6</f>
+        <v/>
+      </c>
+      <c r="L6" s="20">
+        <f>Bottles!G7</f>
+        <v/>
+      </c>
+      <c r="M6" s="20">
+        <f>Bottles!G8</f>
+        <v/>
+      </c>
+      <c r="N6" s="20">
+        <f>Bottles!G9</f>
+        <v/>
+      </c>
+      <c r="O6" s="20">
+        <f>Bottles!G10</f>
+        <v/>
+      </c>
+      <c r="P6" s="20">
+        <f>Bottles!G11</f>
+        <v/>
+      </c>
+      <c r="Q6" s="20">
+        <f>Bottles!G12</f>
+        <v/>
+      </c>
+      <c r="R6" s="20">
+        <f>Bottles!G13</f>
+        <v/>
+      </c>
+      <c r="S6" s="20">
+        <f>Bottles!G14</f>
+        <v/>
+      </c>
+      <c r="T6" s="20">
+        <f>Bottles!G15</f>
+        <v/>
+      </c>
+      <c r="U6" s="15">
         <f>SUM(B6:T6)</f>
         <v/>
       </c>
@@ -1151,86 +1571,86 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Gross margin</t>
-        </is>
-      </c>
-      <c r="B7" s="19">
+          <t>Total revenue</t>
+        </is>
+      </c>
+      <c r="B7" s="15">
         <f>B5+B6</f>
         <v/>
       </c>
-      <c r="C7" s="19">
+      <c r="C7" s="15">
         <f>C5+C6</f>
         <v/>
       </c>
-      <c r="D7" s="19">
+      <c r="D7" s="15">
         <f>D5+D6</f>
         <v/>
       </c>
-      <c r="E7" s="19">
+      <c r="E7" s="15">
         <f>E5+E6</f>
         <v/>
       </c>
-      <c r="F7" s="19">
+      <c r="F7" s="15">
         <f>F5+F6</f>
         <v/>
       </c>
-      <c r="G7" s="19">
+      <c r="G7" s="15">
         <f>G5+G6</f>
         <v/>
       </c>
-      <c r="H7" s="19">
+      <c r="H7" s="15">
         <f>H5+H6</f>
         <v/>
       </c>
-      <c r="I7" s="19">
+      <c r="I7" s="15">
         <f>I5+I6</f>
         <v/>
       </c>
-      <c r="J7" s="19">
+      <c r="J7" s="15">
         <f>J5+J6</f>
         <v/>
       </c>
-      <c r="K7" s="19">
+      <c r="K7" s="15">
         <f>K5+K6</f>
         <v/>
       </c>
-      <c r="L7" s="19">
+      <c r="L7" s="15">
         <f>L5+L6</f>
         <v/>
       </c>
-      <c r="M7" s="19">
+      <c r="M7" s="15">
         <f>M5+M6</f>
         <v/>
       </c>
-      <c r="N7" s="19">
+      <c r="N7" s="15">
         <f>N5+N6</f>
         <v/>
       </c>
-      <c r="O7" s="19">
+      <c r="O7" s="15">
         <f>O5+O6</f>
         <v/>
       </c>
-      <c r="P7" s="19">
+      <c r="P7" s="15">
         <f>P5+P6</f>
         <v/>
       </c>
-      <c r="Q7" s="19">
+      <c r="Q7" s="15">
         <f>Q5+Q6</f>
         <v/>
       </c>
-      <c r="R7" s="19">
+      <c r="R7" s="15">
         <f>R5+R6</f>
         <v/>
       </c>
-      <c r="S7" s="19">
+      <c r="S7" s="15">
         <f>S5+S6</f>
         <v/>
       </c>
-      <c r="T7" s="19">
+      <c r="T7" s="15">
         <f>T5+T6</f>
         <v/>
       </c>
-      <c r="U7" s="19">
+      <c r="U7" s="15">
         <f>SUM(B7:T7)</f>
         <v/>
       </c>
@@ -1238,173 +1658,173 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Gross margin %</t>
-        </is>
-      </c>
-      <c r="B8" s="12">
-        <f>IF(B5=0,0,B7/B5)</f>
-        <v/>
-      </c>
-      <c r="C8" s="12">
-        <f>IF(C5=0,0,C7/C5)</f>
-        <v/>
-      </c>
-      <c r="D8" s="12">
-        <f>IF(D5=0,0,D7/D5)</f>
-        <v/>
-      </c>
-      <c r="E8" s="12">
-        <f>IF(E5=0,0,E7/E5)</f>
-        <v/>
-      </c>
-      <c r="F8" s="12">
-        <f>IF(F5=0,0,F7/F5)</f>
-        <v/>
-      </c>
-      <c r="G8" s="12">
-        <f>IF(G5=0,0,G7/G5)</f>
-        <v/>
-      </c>
-      <c r="H8" s="12">
-        <f>IF(H5=0,0,H7/H5)</f>
-        <v/>
-      </c>
-      <c r="I8" s="12">
-        <f>IF(I5=0,0,I7/I5)</f>
-        <v/>
-      </c>
-      <c r="J8" s="12">
-        <f>IF(J5=0,0,J7/J5)</f>
-        <v/>
-      </c>
-      <c r="K8" s="12">
-        <f>IF(K5=0,0,K7/K5)</f>
-        <v/>
-      </c>
-      <c r="L8" s="12">
-        <f>IF(L5=0,0,L7/L5)</f>
-        <v/>
-      </c>
-      <c r="M8" s="12">
-        <f>IF(M5=0,0,M7/M5)</f>
-        <v/>
-      </c>
-      <c r="N8" s="12">
-        <f>IF(N5=0,0,N7/N5)</f>
-        <v/>
-      </c>
-      <c r="O8" s="12">
-        <f>IF(O5=0,0,O7/O5)</f>
-        <v/>
-      </c>
-      <c r="P8" s="12">
-        <f>IF(P5=0,0,P7/P5)</f>
-        <v/>
-      </c>
-      <c r="Q8" s="12">
-        <f>IF(Q5=0,0,Q7/Q5)</f>
-        <v/>
-      </c>
-      <c r="R8" s="12">
-        <f>IF(R5=0,0,R7/R5)</f>
-        <v/>
-      </c>
-      <c r="S8" s="12">
-        <f>IF(S5=0,0,S7/S5)</f>
-        <v/>
-      </c>
-      <c r="T8" s="12">
-        <f>IF(T5=0,0,T7/T5)</f>
-        <v/>
-      </c>
-      <c r="U8" s="20">
-        <f>U7/U5</f>
+          <t>Can COGS</t>
+        </is>
+      </c>
+      <c r="B8" s="14">
+        <f>-B5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="C8" s="14">
+        <f>-C5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="D8" s="14">
+        <f>-D5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="E8" s="14">
+        <f>-E5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="F8" s="14">
+        <f>-F5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="G8" s="14">
+        <f>-G5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="H8" s="14">
+        <f>-H5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="I8" s="14">
+        <f>-I5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="J8" s="14">
+        <f>-J5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="K8" s="14">
+        <f>-K5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="L8" s="14">
+        <f>-L5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="M8" s="14">
+        <f>-M5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="N8" s="14">
+        <f>-N5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="O8" s="14">
+        <f>-O5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="P8" s="14">
+        <f>-P5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="Q8" s="14">
+        <f>-Q5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="R8" s="14">
+        <f>-R5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="S8" s="14">
+        <f>-S5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="T8" s="14">
+        <f>-T5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="U8" s="15">
+        <f>SUM(B8:T8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Opex (legal &amp; admin)</t>
-        </is>
-      </c>
-      <c r="B9" s="18">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="C9" s="18">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="D9" s="18">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="E9" s="18">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="F9" s="18">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="G9" s="18">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="H9" s="18">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="I9" s="18">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="J9" s="18">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="K9" s="18">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="L9" s="18">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="M9" s="18">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="N9" s="18">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="O9" s="18">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="P9" s="18">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="Q9" s="18">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="R9" s="18">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="S9" s="18">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="T9" s="18">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="U9" s="19">
+          <t>Bottle COGS</t>
+        </is>
+      </c>
+      <c r="B9" s="14">
+        <f>-B6*(1-Bottles!$B$22)</f>
+        <v/>
+      </c>
+      <c r="C9" s="14">
+        <f>-C6*(1-Bottles!$B$22)</f>
+        <v/>
+      </c>
+      <c r="D9" s="14">
+        <f>-D6*(1-Bottles!$B$22)</f>
+        <v/>
+      </c>
+      <c r="E9" s="14">
+        <f>-E6*(1-Bottles!$B$22)</f>
+        <v/>
+      </c>
+      <c r="F9" s="14">
+        <f>-F6*(1-Bottles!$B$22)</f>
+        <v/>
+      </c>
+      <c r="G9" s="14">
+        <f>-G6*(1-Bottles!$B$22)</f>
+        <v/>
+      </c>
+      <c r="H9" s="14">
+        <f>-H6*(1-Bottles!$B$22)</f>
+        <v/>
+      </c>
+      <c r="I9" s="14">
+        <f>-I6*(1-Bottles!$B$22)</f>
+        <v/>
+      </c>
+      <c r="J9" s="14">
+        <f>-J6*(1-Bottles!$B$22)</f>
+        <v/>
+      </c>
+      <c r="K9" s="14">
+        <f>-K6*(1-Bottles!$B$22)</f>
+        <v/>
+      </c>
+      <c r="L9" s="14">
+        <f>-L6*(1-Bottles!$B$22)</f>
+        <v/>
+      </c>
+      <c r="M9" s="14">
+        <f>-M6*(1-Bottles!$B$22)</f>
+        <v/>
+      </c>
+      <c r="N9" s="14">
+        <f>-N6*(1-Bottles!$B$22)</f>
+        <v/>
+      </c>
+      <c r="O9" s="14">
+        <f>-O6*(1-Bottles!$B$22)</f>
+        <v/>
+      </c>
+      <c r="P9" s="14">
+        <f>-P6*(1-Bottles!$B$22)</f>
+        <v/>
+      </c>
+      <c r="Q9" s="14">
+        <f>-Q6*(1-Bottles!$B$22)</f>
+        <v/>
+      </c>
+      <c r="R9" s="14">
+        <f>-R6*(1-Bottles!$B$22)</f>
+        <v/>
+      </c>
+      <c r="S9" s="14">
+        <f>-S6*(1-Bottles!$B$22)</f>
+        <v/>
+      </c>
+      <c r="T9" s="14">
+        <f>-T6*(1-Bottles!$B$22)</f>
+        <v/>
+      </c>
+      <c r="U9" s="15">
         <f>SUM(B9:T9)</f>
         <v/>
       </c>
@@ -1412,86 +1832,86 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>EBITDA</t>
-        </is>
-      </c>
-      <c r="B10" s="19">
-        <f>B7+B9</f>
-        <v/>
-      </c>
-      <c r="C10" s="19">
-        <f>C7+C9</f>
-        <v/>
-      </c>
-      <c r="D10" s="19">
-        <f>D7+D9</f>
-        <v/>
-      </c>
-      <c r="E10" s="19">
-        <f>E7+E9</f>
-        <v/>
-      </c>
-      <c r="F10" s="19">
-        <f>F7+F9</f>
-        <v/>
-      </c>
-      <c r="G10" s="19">
-        <f>G7+G9</f>
-        <v/>
-      </c>
-      <c r="H10" s="19">
-        <f>H7+H9</f>
-        <v/>
-      </c>
-      <c r="I10" s="19">
-        <f>I7+I9</f>
-        <v/>
-      </c>
-      <c r="J10" s="19">
-        <f>J7+J9</f>
-        <v/>
-      </c>
-      <c r="K10" s="19">
-        <f>K7+K9</f>
-        <v/>
-      </c>
-      <c r="L10" s="19">
-        <f>L7+L9</f>
-        <v/>
-      </c>
-      <c r="M10" s="19">
-        <f>M7+M9</f>
-        <v/>
-      </c>
-      <c r="N10" s="19">
-        <f>N7+N9</f>
-        <v/>
-      </c>
-      <c r="O10" s="19">
-        <f>O7+O9</f>
-        <v/>
-      </c>
-      <c r="P10" s="19">
-        <f>P7+P9</f>
-        <v/>
-      </c>
-      <c r="Q10" s="19">
-        <f>Q7+Q9</f>
-        <v/>
-      </c>
-      <c r="R10" s="19">
-        <f>R7+R9</f>
-        <v/>
-      </c>
-      <c r="S10" s="19">
-        <f>S7+S9</f>
-        <v/>
-      </c>
-      <c r="T10" s="19">
-        <f>T7+T9</f>
-        <v/>
-      </c>
-      <c r="U10" s="19">
+          <t>Gross margin</t>
+        </is>
+      </c>
+      <c r="B10" s="15">
+        <f>B7+B8+B9</f>
+        <v/>
+      </c>
+      <c r="C10" s="15">
+        <f>C7+C8+C9</f>
+        <v/>
+      </c>
+      <c r="D10" s="15">
+        <f>D7+D8+D9</f>
+        <v/>
+      </c>
+      <c r="E10" s="15">
+        <f>E7+E8+E9</f>
+        <v/>
+      </c>
+      <c r="F10" s="15">
+        <f>F7+F8+F9</f>
+        <v/>
+      </c>
+      <c r="G10" s="15">
+        <f>G7+G8+G9</f>
+        <v/>
+      </c>
+      <c r="H10" s="15">
+        <f>H7+H8+H9</f>
+        <v/>
+      </c>
+      <c r="I10" s="15">
+        <f>I7+I8+I9</f>
+        <v/>
+      </c>
+      <c r="J10" s="15">
+        <f>J7+J8+J9</f>
+        <v/>
+      </c>
+      <c r="K10" s="15">
+        <f>K7+K8+K9</f>
+        <v/>
+      </c>
+      <c r="L10" s="15">
+        <f>L7+L8+L9</f>
+        <v/>
+      </c>
+      <c r="M10" s="15">
+        <f>M7+M8+M9</f>
+        <v/>
+      </c>
+      <c r="N10" s="15">
+        <f>N7+N8+N9</f>
+        <v/>
+      </c>
+      <c r="O10" s="15">
+        <f>O7+O8+O9</f>
+        <v/>
+      </c>
+      <c r="P10" s="15">
+        <f>P7+P8+P9</f>
+        <v/>
+      </c>
+      <c r="Q10" s="15">
+        <f>Q7+Q8+Q9</f>
+        <v/>
+      </c>
+      <c r="R10" s="15">
+        <f>R7+R8+R9</f>
+        <v/>
+      </c>
+      <c r="S10" s="15">
+        <f>S7+S8+S9</f>
+        <v/>
+      </c>
+      <c r="T10" s="15">
+        <f>T7+T8+T9</f>
+        <v/>
+      </c>
+      <c r="U10" s="15">
         <f>SUM(B10:T10)</f>
         <v/>
       </c>
@@ -1499,87 +1919,348 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
+          <t>Gross margin %</t>
+        </is>
+      </c>
+      <c r="B11" s="12">
+        <f>IF(B7=0,0,B10/B7)</f>
+        <v/>
+      </c>
+      <c r="C11" s="12">
+        <f>IF(C7=0,0,C10/C7)</f>
+        <v/>
+      </c>
+      <c r="D11" s="12">
+        <f>IF(D7=0,0,D10/D7)</f>
+        <v/>
+      </c>
+      <c r="E11" s="12">
+        <f>IF(E7=0,0,E10/E7)</f>
+        <v/>
+      </c>
+      <c r="F11" s="12">
+        <f>IF(F7=0,0,F10/F7)</f>
+        <v/>
+      </c>
+      <c r="G11" s="12">
+        <f>IF(G7=0,0,G10/G7)</f>
+        <v/>
+      </c>
+      <c r="H11" s="12">
+        <f>IF(H7=0,0,H10/H7)</f>
+        <v/>
+      </c>
+      <c r="I11" s="12">
+        <f>IF(I7=0,0,I10/I7)</f>
+        <v/>
+      </c>
+      <c r="J11" s="12">
+        <f>IF(J7=0,0,J10/J7)</f>
+        <v/>
+      </c>
+      <c r="K11" s="12">
+        <f>IF(K7=0,0,K10/K7)</f>
+        <v/>
+      </c>
+      <c r="L11" s="12">
+        <f>IF(L7=0,0,L10/L7)</f>
+        <v/>
+      </c>
+      <c r="M11" s="12">
+        <f>IF(M7=0,0,M10/M7)</f>
+        <v/>
+      </c>
+      <c r="N11" s="12">
+        <f>IF(N7=0,0,N10/N7)</f>
+        <v/>
+      </c>
+      <c r="O11" s="12">
+        <f>IF(O7=0,0,O10/O7)</f>
+        <v/>
+      </c>
+      <c r="P11" s="12">
+        <f>IF(P7=0,0,P10/P7)</f>
+        <v/>
+      </c>
+      <c r="Q11" s="12">
+        <f>IF(Q7=0,0,Q10/Q7)</f>
+        <v/>
+      </c>
+      <c r="R11" s="12">
+        <f>IF(R7=0,0,R10/R7)</f>
+        <v/>
+      </c>
+      <c r="S11" s="12">
+        <f>IF(S7=0,0,S10/S7)</f>
+        <v/>
+      </c>
+      <c r="T11" s="12">
+        <f>IF(T7=0,0,T10/T7)</f>
+        <v/>
+      </c>
+      <c r="U11" s="21">
+        <f>U10/U7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Opex (legal &amp; admin)</t>
+        </is>
+      </c>
+      <c r="B12" s="14">
+        <f>-Assumptions!$B$23</f>
+        <v/>
+      </c>
+      <c r="C12" s="14">
+        <f>-Assumptions!$B$23</f>
+        <v/>
+      </c>
+      <c r="D12" s="14">
+        <f>-Assumptions!$B$23</f>
+        <v/>
+      </c>
+      <c r="E12" s="14">
+        <f>-Assumptions!$B$23</f>
+        <v/>
+      </c>
+      <c r="F12" s="14">
+        <f>-Assumptions!$B$23</f>
+        <v/>
+      </c>
+      <c r="G12" s="14">
+        <f>-Assumptions!$B$23</f>
+        <v/>
+      </c>
+      <c r="H12" s="14">
+        <f>-Assumptions!$B$23</f>
+        <v/>
+      </c>
+      <c r="I12" s="14">
+        <f>-Assumptions!$B$23</f>
+        <v/>
+      </c>
+      <c r="J12" s="14">
+        <f>-Assumptions!$B$23</f>
+        <v/>
+      </c>
+      <c r="K12" s="14">
+        <f>-Assumptions!$B$23</f>
+        <v/>
+      </c>
+      <c r="L12" s="14">
+        <f>-Assumptions!$B$23</f>
+        <v/>
+      </c>
+      <c r="M12" s="14">
+        <f>-Assumptions!$B$23</f>
+        <v/>
+      </c>
+      <c r="N12" s="14">
+        <f>-Assumptions!$B$23</f>
+        <v/>
+      </c>
+      <c r="O12" s="14">
+        <f>-Assumptions!$B$23</f>
+        <v/>
+      </c>
+      <c r="P12" s="14">
+        <f>-Assumptions!$B$23</f>
+        <v/>
+      </c>
+      <c r="Q12" s="14">
+        <f>-Assumptions!$B$23</f>
+        <v/>
+      </c>
+      <c r="R12" s="14">
+        <f>-Assumptions!$B$23</f>
+        <v/>
+      </c>
+      <c r="S12" s="14">
+        <f>-Assumptions!$B$23</f>
+        <v/>
+      </c>
+      <c r="T12" s="14">
+        <f>-Assumptions!$B$23</f>
+        <v/>
+      </c>
+      <c r="U12" s="15">
+        <f>SUM(B12:T12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="B13" s="15">
+        <f>B10+B12</f>
+        <v/>
+      </c>
+      <c r="C13" s="15">
+        <f>C10+C12</f>
+        <v/>
+      </c>
+      <c r="D13" s="15">
+        <f>D10+D12</f>
+        <v/>
+      </c>
+      <c r="E13" s="15">
+        <f>E10+E12</f>
+        <v/>
+      </c>
+      <c r="F13" s="15">
+        <f>F10+F12</f>
+        <v/>
+      </c>
+      <c r="G13" s="15">
+        <f>G10+G12</f>
+        <v/>
+      </c>
+      <c r="H13" s="15">
+        <f>H10+H12</f>
+        <v/>
+      </c>
+      <c r="I13" s="15">
+        <f>I10+I12</f>
+        <v/>
+      </c>
+      <c r="J13" s="15">
+        <f>J10+J12</f>
+        <v/>
+      </c>
+      <c r="K13" s="15">
+        <f>K10+K12</f>
+        <v/>
+      </c>
+      <c r="L13" s="15">
+        <f>L10+L12</f>
+        <v/>
+      </c>
+      <c r="M13" s="15">
+        <f>M10+M12</f>
+        <v/>
+      </c>
+      <c r="N13" s="15">
+        <f>N10+N12</f>
+        <v/>
+      </c>
+      <c r="O13" s="15">
+        <f>O10+O12</f>
+        <v/>
+      </c>
+      <c r="P13" s="15">
+        <f>P10+P12</f>
+        <v/>
+      </c>
+      <c r="Q13" s="15">
+        <f>Q10+Q12</f>
+        <v/>
+      </c>
+      <c r="R13" s="15">
+        <f>R10+R12</f>
+        <v/>
+      </c>
+      <c r="S13" s="15">
+        <f>S10+S12</f>
+        <v/>
+      </c>
+      <c r="T13" s="15">
+        <f>T10+T12</f>
+        <v/>
+      </c>
+      <c r="U13" s="15">
+        <f>SUM(B13:T13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
           <t>EBITDA %</t>
         </is>
       </c>
-      <c r="B11" s="12">
-        <f>IF(B5=0,0,B10/B5)</f>
-        <v/>
-      </c>
-      <c r="C11" s="12">
-        <f>IF(C5=0,0,C10/C5)</f>
-        <v/>
-      </c>
-      <c r="D11" s="12">
-        <f>IF(D5=0,0,D10/D5)</f>
-        <v/>
-      </c>
-      <c r="E11" s="12">
-        <f>IF(E5=0,0,E10/E5)</f>
-        <v/>
-      </c>
-      <c r="F11" s="12">
-        <f>IF(F5=0,0,F10/F5)</f>
-        <v/>
-      </c>
-      <c r="G11" s="12">
-        <f>IF(G5=0,0,G10/G5)</f>
-        <v/>
-      </c>
-      <c r="H11" s="12">
-        <f>IF(H5=0,0,H10/H5)</f>
-        <v/>
-      </c>
-      <c r="I11" s="12">
-        <f>IF(I5=0,0,I10/I5)</f>
-        <v/>
-      </c>
-      <c r="J11" s="12">
-        <f>IF(J5=0,0,J10/J5)</f>
-        <v/>
-      </c>
-      <c r="K11" s="12">
-        <f>IF(K5=0,0,K10/K5)</f>
-        <v/>
-      </c>
-      <c r="L11" s="12">
-        <f>IF(L5=0,0,L10/L5)</f>
-        <v/>
-      </c>
-      <c r="M11" s="12">
-        <f>IF(M5=0,0,M10/M5)</f>
-        <v/>
-      </c>
-      <c r="N11" s="12">
-        <f>IF(N5=0,0,N10/N5)</f>
-        <v/>
-      </c>
-      <c r="O11" s="12">
-        <f>IF(O5=0,0,O10/O5)</f>
-        <v/>
-      </c>
-      <c r="P11" s="12">
-        <f>IF(P5=0,0,P10/P5)</f>
-        <v/>
-      </c>
-      <c r="Q11" s="12">
-        <f>IF(Q5=0,0,Q10/Q5)</f>
-        <v/>
-      </c>
-      <c r="R11" s="12">
-        <f>IF(R5=0,0,R10/R5)</f>
-        <v/>
-      </c>
-      <c r="S11" s="12">
-        <f>IF(S5=0,0,S10/S5)</f>
-        <v/>
-      </c>
-      <c r="T11" s="12">
-        <f>IF(T5=0,0,T10/T5)</f>
-        <v/>
-      </c>
-      <c r="U11" s="20">
-        <f>U10/U5</f>
+      <c r="B14" s="12">
+        <f>IF(B7=0,0,B13/B7)</f>
+        <v/>
+      </c>
+      <c r="C14" s="12">
+        <f>IF(C7=0,0,C13/C7)</f>
+        <v/>
+      </c>
+      <c r="D14" s="12">
+        <f>IF(D7=0,0,D13/D7)</f>
+        <v/>
+      </c>
+      <c r="E14" s="12">
+        <f>IF(E7=0,0,E13/E7)</f>
+        <v/>
+      </c>
+      <c r="F14" s="12">
+        <f>IF(F7=0,0,F13/F7)</f>
+        <v/>
+      </c>
+      <c r="G14" s="12">
+        <f>IF(G7=0,0,G13/G7)</f>
+        <v/>
+      </c>
+      <c r="H14" s="12">
+        <f>IF(H7=0,0,H13/H7)</f>
+        <v/>
+      </c>
+      <c r="I14" s="12">
+        <f>IF(I7=0,0,I13/I7)</f>
+        <v/>
+      </c>
+      <c r="J14" s="12">
+        <f>IF(J7=0,0,J13/J7)</f>
+        <v/>
+      </c>
+      <c r="K14" s="12">
+        <f>IF(K7=0,0,K13/K7)</f>
+        <v/>
+      </c>
+      <c r="L14" s="12">
+        <f>IF(L7=0,0,L13/L7)</f>
+        <v/>
+      </c>
+      <c r="M14" s="12">
+        <f>IF(M7=0,0,M13/M7)</f>
+        <v/>
+      </c>
+      <c r="N14" s="12">
+        <f>IF(N7=0,0,N13/N7)</f>
+        <v/>
+      </c>
+      <c r="O14" s="12">
+        <f>IF(O7=0,0,O13/O7)</f>
+        <v/>
+      </c>
+      <c r="P14" s="12">
+        <f>IF(P7=0,0,P13/P7)</f>
+        <v/>
+      </c>
+      <c r="Q14" s="12">
+        <f>IF(Q7=0,0,Q13/Q7)</f>
+        <v/>
+      </c>
+      <c r="R14" s="12">
+        <f>IF(R7=0,0,R13/R7)</f>
+        <v/>
+      </c>
+      <c r="S14" s="12">
+        <f>IF(S7=0,0,S13/S7)</f>
+        <v/>
+      </c>
+      <c r="T14" s="12">
+        <f>IF(T7=0,0,T13/T7)</f>
+        <v/>
+      </c>
+      <c r="U14" s="21">
+        <f>U13/U7</f>
         <v/>
       </c>
     </row>
@@ -1588,13 +2269,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U18"/>
+  <dimension ref="A1:U19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1622,7 +2303,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CASHFLOW (CASH BASIS) — Doña Fuego cans</t>
+          <t>CASHFLOW (CASH BASIS) — brand entity</t>
         </is>
       </c>
     </row>
@@ -1632,61 +2313,61 @@
           <t>Month</t>
         </is>
       </c>
-      <c r="B3" s="14" t="n">
+      <c r="B3" s="16" t="n">
         <v>46174</v>
       </c>
-      <c r="C3" s="14" t="n">
+      <c r="C3" s="16" t="n">
         <v>46204</v>
       </c>
-      <c r="D3" s="14" t="n">
+      <c r="D3" s="16" t="n">
         <v>46235</v>
       </c>
-      <c r="E3" s="14" t="n">
+      <c r="E3" s="16" t="n">
         <v>46266</v>
       </c>
-      <c r="F3" s="14" t="n">
+      <c r="F3" s="16" t="n">
         <v>46296</v>
       </c>
-      <c r="G3" s="14" t="n">
+      <c r="G3" s="16" t="n">
         <v>46327</v>
       </c>
-      <c r="H3" s="14" t="n">
+      <c r="H3" s="16" t="n">
         <v>46357</v>
       </c>
-      <c r="I3" s="14" t="n">
+      <c r="I3" s="16" t="n">
         <v>46388</v>
       </c>
-      <c r="J3" s="14" t="n">
+      <c r="J3" s="16" t="n">
         <v>46419</v>
       </c>
-      <c r="K3" s="14" t="n">
+      <c r="K3" s="16" t="n">
         <v>46447</v>
       </c>
-      <c r="L3" s="14" t="n">
+      <c r="L3" s="16" t="n">
         <v>46478</v>
       </c>
-      <c r="M3" s="14" t="n">
+      <c r="M3" s="16" t="n">
         <v>46508</v>
       </c>
-      <c r="N3" s="14" t="n">
+      <c r="N3" s="16" t="n">
         <v>46539</v>
       </c>
-      <c r="O3" s="14" t="n">
+      <c r="O3" s="16" t="n">
         <v>46569</v>
       </c>
-      <c r="P3" s="14" t="n">
+      <c r="P3" s="16" t="n">
         <v>46600</v>
       </c>
-      <c r="Q3" s="14" t="n">
+      <c r="Q3" s="16" t="n">
         <v>46631</v>
       </c>
-      <c r="R3" s="14" t="n">
+      <c r="R3" s="16" t="n">
         <v>46661</v>
       </c>
-      <c r="S3" s="14" t="n">
+      <c r="S3" s="16" t="n">
         <v>46692</v>
       </c>
-      <c r="T3" s="14" t="n">
+      <c r="T3" s="16" t="n">
         <v>46722</v>
       </c>
       <c r="U3" s="3" t="inlineStr">
@@ -1698,85 +2379,85 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Receipts (revenue +30 days)</t>
-        </is>
-      </c>
-      <c r="B4" s="18" t="n">
+          <t>Can receipts (revenue +30 days)</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="C4" s="21">
+      <c r="C4" s="20">
         <f>'P&amp;L'!B5</f>
         <v/>
       </c>
-      <c r="D4" s="21">
+      <c r="D4" s="20">
         <f>'P&amp;L'!C5</f>
         <v/>
       </c>
-      <c r="E4" s="21">
+      <c r="E4" s="20">
         <f>'P&amp;L'!D5</f>
         <v/>
       </c>
-      <c r="F4" s="21">
+      <c r="F4" s="20">
         <f>'P&amp;L'!E5</f>
         <v/>
       </c>
-      <c r="G4" s="21">
+      <c r="G4" s="20">
         <f>'P&amp;L'!F5</f>
         <v/>
       </c>
-      <c r="H4" s="21">
+      <c r="H4" s="20">
         <f>'P&amp;L'!G5</f>
         <v/>
       </c>
-      <c r="I4" s="21">
+      <c r="I4" s="20">
         <f>'P&amp;L'!H5</f>
         <v/>
       </c>
-      <c r="J4" s="21">
+      <c r="J4" s="20">
         <f>'P&amp;L'!I5</f>
         <v/>
       </c>
-      <c r="K4" s="21">
+      <c r="K4" s="20">
         <f>'P&amp;L'!J5</f>
         <v/>
       </c>
-      <c r="L4" s="21">
+      <c r="L4" s="20">
         <f>'P&amp;L'!K5</f>
         <v/>
       </c>
-      <c r="M4" s="21">
+      <c r="M4" s="20">
         <f>'P&amp;L'!L5</f>
         <v/>
       </c>
-      <c r="N4" s="21">
+      <c r="N4" s="20">
         <f>'P&amp;L'!M5</f>
         <v/>
       </c>
-      <c r="O4" s="21">
+      <c r="O4" s="20">
         <f>'P&amp;L'!N5</f>
         <v/>
       </c>
-      <c r="P4" s="21">
+      <c r="P4" s="20">
         <f>'P&amp;L'!O5</f>
         <v/>
       </c>
-      <c r="Q4" s="21">
+      <c r="Q4" s="20">
         <f>'P&amp;L'!P5</f>
         <v/>
       </c>
-      <c r="R4" s="21">
+      <c r="R4" s="20">
         <f>'P&amp;L'!Q5</f>
         <v/>
       </c>
-      <c r="S4" s="21">
+      <c r="S4" s="20">
         <f>'P&amp;L'!R5</f>
         <v/>
       </c>
-      <c r="T4" s="21">
+      <c r="T4" s="20">
         <f>'P&amp;L'!S5</f>
         <v/>
       </c>
-      <c r="U4" s="19">
+      <c r="U4" s="15">
         <f>SUM(B4:T4)</f>
         <v/>
       </c>
@@ -1787,15 +2468,15 @@
           <t xml:space="preserve">  Bron Pro (design/brand)</t>
         </is>
       </c>
-      <c r="B5" s="18">
+      <c r="B5" s="14">
         <f>-103500*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="D5" s="18">
+      <c r="D5" s="14">
         <f>-243800*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="U5" s="18">
+      <c r="U5" s="14">
         <f>SUM(B5:T5)</f>
         <v/>
       </c>
@@ -1806,15 +2487,15 @@
           <t xml:space="preserve">  Sullwaldt printing</t>
         </is>
       </c>
-      <c r="C6" s="18">
+      <c r="C6" s="14">
         <f>-91066*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="F6" s="18">
+      <c r="F6" s="14">
         <f>-72400*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="U6" s="18">
+      <c r="U6" s="14">
         <f>SUM(B6:T6)</f>
         <v/>
       </c>
@@ -1825,15 +2506,15 @@
           <t xml:space="preserve">  Tiny Keg cans</t>
         </is>
       </c>
-      <c r="C7" s="18">
+      <c r="C7" s="14">
         <f>-405950*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="E7" s="18">
+      <c r="E7" s="14">
         <f>-319000*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="U7" s="18">
+      <c r="U7" s="14">
         <f>SUM(B7:T7)</f>
         <v/>
       </c>
@@ -1844,11 +2525,11 @@
           <t xml:space="preserve">  Chep pallets</t>
         </is>
       </c>
-      <c r="B8" s="18">
+      <c r="B8" s="14">
         <f>-14375*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="U8" s="18">
+      <c r="U8" s="14">
         <f>SUM(B8:T8)</f>
         <v/>
       </c>
@@ -1859,15 +2540,15 @@
           <t xml:space="preserve">  FAL distribution</t>
         </is>
       </c>
-      <c r="C9" s="18">
+      <c r="C9" s="14">
         <f>-51750*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="14">
         <f>-28000*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="U9" s="18">
+      <c r="U9" s="14">
         <f>SUM(B9:T9)</f>
         <v/>
       </c>
@@ -1878,15 +2559,15 @@
           <t xml:space="preserve">  Tiny Keg production</t>
         </is>
       </c>
-      <c r="D10" s="18">
+      <c r="D10" s="14">
         <f>-373350*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="14">
         <f>-293250*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="U10" s="18">
+      <c r="U10" s="14">
         <f>SUM(B10:T10)</f>
         <v/>
       </c>
@@ -1897,15 +2578,15 @@
           <t xml:space="preserve">  SARS excise (launch)</t>
         </is>
       </c>
-      <c r="E11" s="18">
+      <c r="E11" s="14">
         <f>-630000*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="G11" s="18">
+      <c r="G11" s="14">
         <f>-495571*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="U11" s="18">
+      <c r="U11" s="14">
         <f>SUM(B11:T11)</f>
         <v/>
       </c>
@@ -1916,10 +2597,10 @@
           <t xml:space="preserve">  Legal &amp; admin (2026)</t>
         </is>
       </c>
-      <c r="C12" s="18" t="n">
+      <c r="C12" s="14" t="n">
         <v>-57500</v>
       </c>
-      <c r="U12" s="18">
+      <c r="U12" s="14">
         <f>SUM(B12:T12)</f>
         <v/>
       </c>
@@ -1927,145 +2608,145 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2027 recurring COGS + opex</t>
-        </is>
-      </c>
-      <c r="I13" s="18">
+          <t xml:space="preserve">  Bottles net contribution (GM, cash in month)</t>
+        </is>
+      </c>
+      <c r="B13" s="20">
+        <f>'P&amp;L'!B6*Bottles!$B$22</f>
+        <v/>
+      </c>
+      <c r="C13" s="20">
+        <f>'P&amp;L'!C6*Bottles!$B$22</f>
+        <v/>
+      </c>
+      <c r="D13" s="20">
+        <f>'P&amp;L'!D6*Bottles!$B$22</f>
+        <v/>
+      </c>
+      <c r="E13" s="20">
+        <f>'P&amp;L'!E6*Bottles!$B$22</f>
+        <v/>
+      </c>
+      <c r="F13" s="20">
+        <f>'P&amp;L'!F6*Bottles!$B$22</f>
+        <v/>
+      </c>
+      <c r="G13" s="20">
+        <f>'P&amp;L'!G6*Bottles!$B$22</f>
+        <v/>
+      </c>
+      <c r="H13" s="20">
+        <f>'P&amp;L'!H6*Bottles!$B$22</f>
+        <v/>
+      </c>
+      <c r="I13" s="20">
+        <f>'P&amp;L'!I6*Bottles!$B$22</f>
+        <v/>
+      </c>
+      <c r="J13" s="20">
+        <f>'P&amp;L'!J6*Bottles!$B$22</f>
+        <v/>
+      </c>
+      <c r="K13" s="20">
+        <f>'P&amp;L'!K6*Bottles!$B$22</f>
+        <v/>
+      </c>
+      <c r="L13" s="20">
+        <f>'P&amp;L'!L6*Bottles!$B$22</f>
+        <v/>
+      </c>
+      <c r="M13" s="20">
+        <f>'P&amp;L'!M6*Bottles!$B$22</f>
+        <v/>
+      </c>
+      <c r="N13" s="20">
+        <f>'P&amp;L'!N6*Bottles!$B$22</f>
+        <v/>
+      </c>
+      <c r="O13" s="20">
+        <f>'P&amp;L'!O6*Bottles!$B$22</f>
+        <v/>
+      </c>
+      <c r="P13" s="20">
+        <f>'P&amp;L'!P6*Bottles!$B$22</f>
+        <v/>
+      </c>
+      <c r="Q13" s="20">
+        <f>'P&amp;L'!Q6*Bottles!$B$22</f>
+        <v/>
+      </c>
+      <c r="R13" s="20">
+        <f>'P&amp;L'!R6*Bottles!$B$22</f>
+        <v/>
+      </c>
+      <c r="S13" s="20">
+        <f>'P&amp;L'!S6*Bottles!$B$22</f>
+        <v/>
+      </c>
+      <c r="T13" s="20">
+        <f>'P&amp;L'!T6*Bottles!$B$22</f>
+        <v/>
+      </c>
+      <c r="U13" s="14">
+        <f>SUM(B13:T13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2027 recurring can COGS + opex</t>
+        </is>
+      </c>
+      <c r="I14" s="14">
         <f>-('P&amp;L'!I5*Assumptions!$B$21+Assumptions!$B$23)</f>
         <v/>
       </c>
-      <c r="J13" s="18">
+      <c r="J14" s="14">
         <f>-('P&amp;L'!J5*Assumptions!$B$21+Assumptions!$B$23)</f>
         <v/>
       </c>
-      <c r="K13" s="18">
+      <c r="K14" s="14">
         <f>-('P&amp;L'!K5*Assumptions!$B$21+Assumptions!$B$23)</f>
         <v/>
       </c>
-      <c r="L13" s="18">
+      <c r="L14" s="14">
         <f>-('P&amp;L'!L5*Assumptions!$B$21+Assumptions!$B$23)</f>
         <v/>
       </c>
-      <c r="M13" s="18">
+      <c r="M14" s="14">
         <f>-('P&amp;L'!M5*Assumptions!$B$21+Assumptions!$B$23)</f>
         <v/>
       </c>
-      <c r="N13" s="18">
+      <c r="N14" s="14">
         <f>-('P&amp;L'!N5*Assumptions!$B$21+Assumptions!$B$23)</f>
         <v/>
       </c>
-      <c r="O13" s="18">
+      <c r="O14" s="14">
         <f>-('P&amp;L'!O5*Assumptions!$B$21+Assumptions!$B$23)</f>
         <v/>
       </c>
-      <c r="P13" s="18">
+      <c r="P14" s="14">
         <f>-('P&amp;L'!P5*Assumptions!$B$21+Assumptions!$B$23)</f>
         <v/>
       </c>
-      <c r="Q13" s="18">
+      <c r="Q14" s="14">
         <f>-('P&amp;L'!Q5*Assumptions!$B$21+Assumptions!$B$23)</f>
         <v/>
       </c>
-      <c r="R13" s="18">
+      <c r="R14" s="14">
         <f>-('P&amp;L'!R5*Assumptions!$B$21+Assumptions!$B$23)</f>
         <v/>
       </c>
-      <c r="S13" s="18">
+      <c r="S14" s="14">
         <f>-('P&amp;L'!S5*Assumptions!$B$21+Assumptions!$B$23)</f>
         <v/>
       </c>
-      <c r="T13" s="18">
+      <c r="T14" s="14">
         <f>-('P&amp;L'!T5*Assumptions!$B$21+Assumptions!$B$23)</f>
         <v/>
       </c>
-      <c r="U13" s="18">
-        <f>SUM(B13:T13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Net monthly cashflow</t>
-        </is>
-      </c>
-      <c r="B14" s="19">
-        <f>SUM(B4:B13)</f>
-        <v/>
-      </c>
-      <c r="C14" s="19">
-        <f>SUM(C4:C13)</f>
-        <v/>
-      </c>
-      <c r="D14" s="19">
-        <f>SUM(D4:D13)</f>
-        <v/>
-      </c>
-      <c r="E14" s="19">
-        <f>SUM(E4:E13)</f>
-        <v/>
-      </c>
-      <c r="F14" s="19">
-        <f>SUM(F4:F13)</f>
-        <v/>
-      </c>
-      <c r="G14" s="19">
-        <f>SUM(G4:G13)</f>
-        <v/>
-      </c>
-      <c r="H14" s="19">
-        <f>SUM(H4:H13)</f>
-        <v/>
-      </c>
-      <c r="I14" s="19">
-        <f>SUM(I4:I13)</f>
-        <v/>
-      </c>
-      <c r="J14" s="19">
-        <f>SUM(J4:J13)</f>
-        <v/>
-      </c>
-      <c r="K14" s="19">
-        <f>SUM(K4:K13)</f>
-        <v/>
-      </c>
-      <c r="L14" s="19">
-        <f>SUM(L4:L13)</f>
-        <v/>
-      </c>
-      <c r="M14" s="19">
-        <f>SUM(M4:M13)</f>
-        <v/>
-      </c>
-      <c r="N14" s="19">
-        <f>SUM(N4:N13)</f>
-        <v/>
-      </c>
-      <c r="O14" s="19">
-        <f>SUM(O4:O13)</f>
-        <v/>
-      </c>
-      <c r="P14" s="19">
-        <f>SUM(P4:P13)</f>
-        <v/>
-      </c>
-      <c r="Q14" s="19">
-        <f>SUM(Q4:Q13)</f>
-        <v/>
-      </c>
-      <c r="R14" s="19">
-        <f>SUM(R4:R13)</f>
-        <v/>
-      </c>
-      <c r="S14" s="19">
-        <f>SUM(S4:S13)</f>
-        <v/>
-      </c>
-      <c r="T14" s="19">
-        <f>SUM(T4:T13)</f>
-        <v/>
-      </c>
-      <c r="U14" s="19">
+      <c r="U14" s="14">
         <f>SUM(B14:T14)</f>
         <v/>
       </c>
@@ -2073,97 +2754,184 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>Net monthly cashflow</t>
+        </is>
+      </c>
+      <c r="B15" s="15">
+        <f>SUM(B4:B14)</f>
+        <v/>
+      </c>
+      <c r="C15" s="15">
+        <f>SUM(C4:C14)</f>
+        <v/>
+      </c>
+      <c r="D15" s="15">
+        <f>SUM(D4:D14)</f>
+        <v/>
+      </c>
+      <c r="E15" s="15">
+        <f>SUM(E4:E14)</f>
+        <v/>
+      </c>
+      <c r="F15" s="15">
+        <f>SUM(F4:F14)</f>
+        <v/>
+      </c>
+      <c r="G15" s="15">
+        <f>SUM(G4:G14)</f>
+        <v/>
+      </c>
+      <c r="H15" s="15">
+        <f>SUM(H4:H14)</f>
+        <v/>
+      </c>
+      <c r="I15" s="15">
+        <f>SUM(I4:I14)</f>
+        <v/>
+      </c>
+      <c r="J15" s="15">
+        <f>SUM(J4:J14)</f>
+        <v/>
+      </c>
+      <c r="K15" s="15">
+        <f>SUM(K4:K14)</f>
+        <v/>
+      </c>
+      <c r="L15" s="15">
+        <f>SUM(L4:L14)</f>
+        <v/>
+      </c>
+      <c r="M15" s="15">
+        <f>SUM(M4:M14)</f>
+        <v/>
+      </c>
+      <c r="N15" s="15">
+        <f>SUM(N4:N14)</f>
+        <v/>
+      </c>
+      <c r="O15" s="15">
+        <f>SUM(O4:O14)</f>
+        <v/>
+      </c>
+      <c r="P15" s="15">
+        <f>SUM(P4:P14)</f>
+        <v/>
+      </c>
+      <c r="Q15" s="15">
+        <f>SUM(Q4:Q14)</f>
+        <v/>
+      </c>
+      <c r="R15" s="15">
+        <f>SUM(R4:R14)</f>
+        <v/>
+      </c>
+      <c r="S15" s="15">
+        <f>SUM(S4:S14)</f>
+        <v/>
+      </c>
+      <c r="T15" s="15">
+        <f>SUM(T4:T14)</f>
+        <v/>
+      </c>
+      <c r="U15" s="15">
+        <f>SUM(B15:T15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>Cumulative cash position</t>
         </is>
       </c>
-      <c r="B15" s="19">
-        <f>B14</f>
-        <v/>
-      </c>
-      <c r="C15" s="19">
-        <f>B15+C14</f>
-        <v/>
-      </c>
-      <c r="D15" s="19">
-        <f>C15+D14</f>
-        <v/>
-      </c>
-      <c r="E15" s="19">
-        <f>D15+E14</f>
-        <v/>
-      </c>
-      <c r="F15" s="19">
-        <f>E15+F14</f>
-        <v/>
-      </c>
-      <c r="G15" s="19">
-        <f>F15+G14</f>
-        <v/>
-      </c>
-      <c r="H15" s="19">
-        <f>G15+H14</f>
-        <v/>
-      </c>
-      <c r="I15" s="19">
-        <f>H15+I14</f>
-        <v/>
-      </c>
-      <c r="J15" s="19">
-        <f>I15+J14</f>
-        <v/>
-      </c>
-      <c r="K15" s="19">
-        <f>J15+K14</f>
-        <v/>
-      </c>
-      <c r="L15" s="19">
-        <f>K15+L14</f>
-        <v/>
-      </c>
-      <c r="M15" s="19">
-        <f>L15+M14</f>
-        <v/>
-      </c>
-      <c r="N15" s="19">
-        <f>M15+N14</f>
-        <v/>
-      </c>
-      <c r="O15" s="19">
-        <f>N15+O14</f>
-        <v/>
-      </c>
-      <c r="P15" s="19">
-        <f>O15+P14</f>
-        <v/>
-      </c>
-      <c r="Q15" s="19">
-        <f>P15+Q14</f>
-        <v/>
-      </c>
-      <c r="R15" s="19">
-        <f>Q15+R14</f>
-        <v/>
-      </c>
-      <c r="S15" s="19">
-        <f>R15+S14</f>
-        <v/>
-      </c>
-      <c r="T15" s="19">
-        <f>S15+T14</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Note: 2026 launch costs are the project model's quoted cash costs, scaled by the store factor (Assumptions!B24); legal retainer unscaled.</t>
-        </is>
+      <c r="B16" s="15">
+        <f>B15</f>
+        <v/>
+      </c>
+      <c r="C16" s="15">
+        <f>B16+C15</f>
+        <v/>
+      </c>
+      <c r="D16" s="15">
+        <f>C16+D15</f>
+        <v/>
+      </c>
+      <c r="E16" s="15">
+        <f>D16+E15</f>
+        <v/>
+      </c>
+      <c r="F16" s="15">
+        <f>E16+F15</f>
+        <v/>
+      </c>
+      <c r="G16" s="15">
+        <f>F16+G15</f>
+        <v/>
+      </c>
+      <c r="H16" s="15">
+        <f>G16+H15</f>
+        <v/>
+      </c>
+      <c r="I16" s="15">
+        <f>H16+I15</f>
+        <v/>
+      </c>
+      <c r="J16" s="15">
+        <f>I16+J15</f>
+        <v/>
+      </c>
+      <c r="K16" s="15">
+        <f>J16+K15</f>
+        <v/>
+      </c>
+      <c r="L16" s="15">
+        <f>K16+L15</f>
+        <v/>
+      </c>
+      <c r="M16" s="15">
+        <f>L16+M15</f>
+        <v/>
+      </c>
+      <c r="N16" s="15">
+        <f>M16+N15</f>
+        <v/>
+      </c>
+      <c r="O16" s="15">
+        <f>N16+O15</f>
+        <v/>
+      </c>
+      <c r="P16" s="15">
+        <f>O16+P15</f>
+        <v/>
+      </c>
+      <c r="Q16" s="15">
+        <f>P16+Q15</f>
+        <v/>
+      </c>
+      <c r="R16" s="15">
+        <f>Q16+R15</f>
+        <v/>
+      </c>
+      <c r="S16" s="15">
+        <f>R16+S15</f>
+        <v/>
+      </c>
+      <c r="T16" s="15">
+        <f>S16+T15</f>
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2027 steady-state COGS assumed paid in month of delivery; tequila purchased under the distillery supply agreement.</t>
+          <t>Note: 2026 launch costs are the project model's quoted cash costs, scaled by the store factor (Assumptions!B24); legal retainer unscaled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Bottles assumed cash-in-month at gross margin; 2027 steady-state can COGS paid in month of delivery.</t>
         </is>
       </c>
     </row>
@@ -2172,7 +2940,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2191,7 +2959,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>VALUATION — Doña Fuego brand entity (cans only; bottles not yet modelled)</t>
+          <t>VALUATION — Doña Fuego brand entity (cans + bottles)</t>
         </is>
       </c>
     </row>
@@ -2208,8 +2976,8 @@
           <t>2026 (Jun–Dec) revenue</t>
         </is>
       </c>
-      <c r="B4" s="21">
-        <f>SUM('P&amp;L'!B5:H5)</f>
+      <c r="B4" s="20">
+        <f>SUM('P&amp;L'!B7:H7)</f>
         <v/>
       </c>
     </row>
@@ -2219,8 +2987,8 @@
           <t>2026 (Jun–Dec) EBITDA</t>
         </is>
       </c>
-      <c r="B5" s="21">
-        <f>SUM('P&amp;L'!B10:H10)</f>
+      <c r="B5" s="20">
+        <f>SUM('P&amp;L'!B13:H13)</f>
         <v/>
       </c>
     </row>
@@ -2230,8 +2998,8 @@
           <t>2027 revenue</t>
         </is>
       </c>
-      <c r="B6" s="21">
-        <f>SUM('P&amp;L'!I5:T5)</f>
+      <c r="B6" s="20">
+        <f>SUM('P&amp;L'!I7:T7)</f>
         <v/>
       </c>
     </row>
@@ -2241,8 +3009,8 @@
           <t>2027 EBITDA</t>
         </is>
       </c>
-      <c r="B7" s="21">
-        <f>SUM('P&amp;L'!I10:T10)</f>
+      <c r="B7" s="20">
+        <f>SUM('P&amp;L'!I13:T13)</f>
         <v/>
       </c>
     </row>
@@ -2290,15 +3058,15 @@
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="B11" s="18">
+      <c r="B11" s="14">
         <f>$B$7*B10</f>
         <v/>
       </c>
-      <c r="C11" s="18">
+      <c r="C11" s="14">
         <f>$B$7*C10</f>
         <v/>
       </c>
-      <c r="D11" s="18">
+      <c r="D11" s="14">
         <f>$B$7*D10</f>
         <v/>
       </c>
@@ -2332,15 +3100,15 @@
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="B15" s="18">
+      <c r="B15" s="14">
         <f>$B$6*B14</f>
         <v/>
       </c>
-      <c r="C15" s="18">
+      <c r="C15" s="14">
         <f>$B$6*C14</f>
         <v/>
       </c>
-      <c r="D15" s="18">
+      <c r="D15" s="14">
         <f>$B$6*D14</f>
         <v/>
       </c>
@@ -2390,15 +3158,15 @@
           <t>Enterprise value (DCF)</t>
         </is>
       </c>
-      <c r="B20" s="18">
+      <c r="B20" s="14">
         <f>$B$5/(1+B18)^0.25+$B$7/(1+B18)+$B$7*B19/(1+B18)^1.5</f>
         <v/>
       </c>
-      <c r="C20" s="18">
+      <c r="C20" s="14">
         <f>$B$5/(1+C18)^0.25+$B$7/(1+C18)+$B$7*C19/(1+C18)^1.5</f>
         <v/>
       </c>
-      <c r="D20" s="18">
+      <c r="D20" s="14">
         <f>$B$5/(1+D18)^0.25+$B$7/(1+D18)+$B$7*D19/(1+D18)^1.5</f>
         <v/>
       </c>
@@ -2409,15 +3177,15 @@
           <t>Blended enterprise value (avg of methods)</t>
         </is>
       </c>
-      <c r="B22" s="19">
+      <c r="B22" s="15">
         <f>AVERAGE(B11,B15,B20)</f>
         <v/>
       </c>
-      <c r="C22" s="19">
+      <c r="C22" s="15">
         <f>AVERAGE(C11,C15,C20)</f>
         <v/>
       </c>
-      <c r="D22" s="19">
+      <c r="D22" s="15">
         <f>AVERAGE(D11,D15,D20)</f>
         <v/>
       </c>
@@ -2433,14 +3201,14 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Guide sits between the blended Low and Base; bottles, 360-store actuals vs conservative reorders, export and post-exclusivity retail are upside outside this model.</t>
+          <t>With bottles modelled off three years of actuals, the ~R15m guide equals the blended LOW case; better-than-flat reorders, new retailers and export remain outside the model.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Same three methods and multiples as the tequila project model, applied to brand-only economics.</t>
+          <t>Same three methods and multiples as the tequila project model, applied to brand-entity economics.</t>
         </is>
       </c>
     </row>
@@ -2449,13 +3217,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -2486,7 +3254,7 @@
           <t>Opening order (initial fill revenue)</t>
         </is>
       </c>
-      <c r="B4" s="21">
+      <c r="B4" s="20">
         <f>'P&amp;L'!D5</f>
         <v/>
       </c>
@@ -2494,106 +3262,117 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Total can revenue (Jun 26 – Dec 27)</t>
-        </is>
-      </c>
-      <c r="B5" s="21">
-        <f>'P&amp;L'!U5</f>
+          <t>Bottle revenue (Jun 26 – Dec 27)</t>
+        </is>
+      </c>
+      <c r="B5" s="20">
+        <f>'P&amp;L'!U6</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Total EBITDA (Jun 26 – Dec 27)</t>
-        </is>
-      </c>
-      <c r="B6" s="21">
-        <f>'P&amp;L'!U10</f>
+          <t>Total revenue, cans + bottles (Jun 26 – Dec 27)</t>
+        </is>
+      </c>
+      <c r="B6" s="20">
+        <f>'P&amp;L'!U7</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>EBITDA margin</t>
-        </is>
-      </c>
-      <c r="B7" s="25">
-        <f>'P&amp;L'!U11</f>
+          <t>Total EBITDA (Jun 26 – Dec 27)</t>
+        </is>
+      </c>
+      <c r="B7" s="20">
+        <f>'P&amp;L'!U13</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Peak funding need</t>
-        </is>
-      </c>
-      <c r="B8" s="21">
-        <f>MIN(Cashflow!B15:T15)</f>
+          <t>EBITDA margin</t>
+        </is>
+      </c>
+      <c r="B8" s="25">
+        <f>'P&amp;L'!U14</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Ending cash (Dec 27)</t>
-        </is>
-      </c>
-      <c r="B9" s="21">
-        <f>Cashflow!T15</f>
+          <t>Peak funding need</t>
+        </is>
+      </c>
+      <c r="B9" s="20">
+        <f>MIN(Cashflow!B16:T16)</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Blended valuation — low</t>
-        </is>
-      </c>
-      <c r="B10" s="21">
-        <f>Valuation!B22</f>
+          <t>Ending cash (Dec 27)</t>
+        </is>
+      </c>
+      <c r="B10" s="20">
+        <f>Cashflow!T16</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Blended valuation — base</t>
-        </is>
-      </c>
-      <c r="B11" s="21">
-        <f>Valuation!C22</f>
+          <t>Blended valuation — low</t>
+        </is>
+      </c>
+      <c r="B11" s="20">
+        <f>Valuation!B22</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Blended valuation — high</t>
-        </is>
-      </c>
-      <c r="B12" s="21">
-        <f>Valuation!D22</f>
+          <t>Blended valuation — base</t>
+        </is>
+      </c>
+      <c r="B12" s="20">
+        <f>Valuation!C22</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
+          <t>Blended valuation — high</t>
+        </is>
+      </c>
+      <c r="B13" s="20">
+        <f>Valuation!D22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
           <t>Valuation guide</t>
         </is>
       </c>
-      <c r="B13" s="21">
+      <c r="B14" s="20">
         <f>Valuation!B24</f>
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Not modelled (upside): Fuego Tequila bottled range (sales data pending), post-exclusivity retailers, export.</t>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Not modelled (upside): better-than-flat can reorders, post-exclusivity retailers, export. Bottle margin is a placeholder pending cost data.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Full sales, operations and distribution cost base in the pro forma
- Opex block in Assumptions (management-estimate inputs): sales & key
  accounts R40k, ops & merchandising R18k, trade marketing R25k,
  warehousing & insurance R12k, legal & admin R10k — R105k/month steady
  state, phased from July/August 2026
- P&L opex phased by month; cashflow carries opex explicitly (legal lump
  replaced by the monthly schedule)
- Results: EBITDA R2.96m (18.4%) to Dec 27, peak funding need R1.64m,
  end cash R2.15m; blended valuation R10.5m/R15.1m/R21.4m — the ~R15m
  guide equals the blended base case of the fully costed pro forma
- Dataroom P&L gains an opex row; valuation table, cash chart, stat bands
  and FAQs carry the fully costed numbers

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hyws6xeXfxtGdqZV2paNDe
</commit_message>
<xml_diff>
--- a/site/downloads/Dona-Fuego-Brand-Pro-Forma.xlsx
+++ b/site/downloads/Dona-Fuego-Brand-Pro-Forma.xlsx
@@ -107,6 +107,7 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="17" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -116,7 +117,6 @@
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -737,14 +737,14 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Operating costs</t>
+          <t>Operating costs — sales, operations &amp; distribution (monthly)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Legal &amp; admin (R/month)</t>
+          <t>Legal &amp; admin</t>
         </is>
       </c>
       <c r="B23" s="9" t="n">
@@ -752,7 +752,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Per project model</t>
+          <t>Per project model; from June 2026</t>
         </is>
       </c>
     </row>
@@ -777,6 +777,77 @@
         <is>
           <t>Legend: blue = input (edit these) · black = formula · green = link to another sheet · yellow = key assumptions to sense-check</t>
         </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Sales &amp; key accounts (1 FTE)</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="n">
+        <v>40000</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>MANAGEMENT ESTIMATE, from July 2026 — supports founder-led sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Operations &amp; merchandising coordinator</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="n">
+        <v>18000</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>MANAGEMENT ESTIMATE, from July 2026 — shared resource with distillery</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Trade marketing &amp; promotions</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="n">
+        <v>25000</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>MANAGEMENT ESTIMATE, from August 2026 — always-on consumer &amp; in-store support</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Warehousing &amp; insurance</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="n">
+        <v>12000</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>MANAGEMENT ESTIMATE, from August 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Steady-state opex total</t>
+        </is>
+      </c>
+      <c r="B32" s="15">
+        <f>B23+B28+B29+B30+B31</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -864,7 +935,7 @@
       <c r="E4" s="9" t="n">
         <v>185865.3</v>
       </c>
-      <c r="G4" s="14">
+      <c r="G4" s="15">
         <f>(D4+E4)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
@@ -884,7 +955,7 @@
       <c r="E5" s="9" t="n">
         <v>209857.2</v>
       </c>
-      <c r="G5" s="14">
+      <c r="G5" s="15">
         <f>(D5+E5)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
@@ -901,7 +972,7 @@
       <c r="E6" s="9" t="n">
         <v>260918.59</v>
       </c>
-      <c r="G6" s="14">
+      <c r="G6" s="15">
         <f>(D6+E6)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
@@ -921,7 +992,7 @@
       <c r="E7" s="9" t="n">
         <v>470561.32</v>
       </c>
-      <c r="G7" s="14">
+      <c r="G7" s="15">
         <f>(D7+E7)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
@@ -941,7 +1012,7 @@
       <c r="E8" s="9" t="n">
         <v>167687.8</v>
       </c>
-      <c r="G8" s="14">
+      <c r="G8" s="15">
         <f>(D8+E8)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
@@ -961,7 +1032,7 @@
       <c r="E9" s="9" t="n">
         <v>60059.82</v>
       </c>
-      <c r="G9" s="14">
+      <c r="G9" s="15">
         <f>(D9+E9)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
@@ -981,7 +1052,7 @@
       <c r="E10" s="9" t="n">
         <v>188654.34</v>
       </c>
-      <c r="G10" s="14">
+      <c r="G10" s="15">
         <f>(D10+E10)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
@@ -998,11 +1069,11 @@
       <c r="D11" s="9" t="n">
         <v>44441.56</v>
       </c>
-      <c r="E11" s="14">
+      <c r="E11" s="15">
         <f>D11*$B$19</f>
         <v/>
       </c>
-      <c r="G11" s="14">
+      <c r="G11" s="15">
         <f>(D11+E11)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
@@ -1022,11 +1093,11 @@
       <c r="D12" s="9" t="n">
         <v>65847.11</v>
       </c>
-      <c r="E12" s="14">
+      <c r="E12" s="15">
         <f>D12*$B$19</f>
         <v/>
       </c>
-      <c r="G12" s="14">
+      <c r="G12" s="15">
         <f>(D12+E12)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
@@ -1046,11 +1117,11 @@
       <c r="D13" s="9" t="n">
         <v>63268.38</v>
       </c>
-      <c r="E13" s="14">
+      <c r="E13" s="15">
         <f>D13*$B$19</f>
         <v/>
       </c>
-      <c r="G13" s="14">
+      <c r="G13" s="15">
         <f>(D13+E13)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
@@ -1067,11 +1138,11 @@
       <c r="D14" s="9" t="n">
         <v>257848.55</v>
       </c>
-      <c r="E14" s="14">
+      <c r="E14" s="15">
         <f>D14*$B$19</f>
         <v/>
       </c>
-      <c r="G14" s="14">
+      <c r="G14" s="15">
         <f>(D14+E14)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
@@ -1091,11 +1162,11 @@
       <c r="D15" s="9" t="n">
         <v>35332.6</v>
       </c>
-      <c r="E15" s="14">
+      <c r="E15" s="15">
         <f>D15*$B$19</f>
         <v/>
       </c>
-      <c r="G15" s="14">
+      <c r="G15" s="15">
         <f>(D15+E15)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
@@ -1106,23 +1177,23 @@
           <t>Annual total</t>
         </is>
       </c>
-      <c r="B16" s="15">
+      <c r="B16" s="16">
         <f>SUM(B4:B15)</f>
         <v/>
       </c>
-      <c r="C16" s="15">
+      <c r="C16" s="16">
         <f>SUM(C4:C15)</f>
         <v/>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="16">
         <f>SUM(D4:D15)</f>
         <v/>
       </c>
-      <c r="E16" s="15">
+      <c r="E16" s="16">
         <f>SUM(E4:E15)</f>
         <v/>
       </c>
-      <c r="G16" s="15">
+      <c r="G16" s="16">
         <f>SUM(G4:G15)</f>
         <v/>
       </c>
@@ -1171,7 +1242,7 @@
           <t>2027 total</t>
         </is>
       </c>
-      <c r="B21" s="14">
+      <c r="B21" s="15">
         <f>E16*(1+B20)</f>
         <v/>
       </c>
@@ -1247,61 +1318,61 @@
           <t>Month</t>
         </is>
       </c>
-      <c r="B3" s="16" t="n">
+      <c r="B3" s="17" t="n">
         <v>46174</v>
       </c>
-      <c r="C3" s="16" t="n">
+      <c r="C3" s="17" t="n">
         <v>46204</v>
       </c>
-      <c r="D3" s="16" t="n">
+      <c r="D3" s="17" t="n">
         <v>46235</v>
       </c>
-      <c r="E3" s="16" t="n">
+      <c r="E3" s="17" t="n">
         <v>46266</v>
       </c>
-      <c r="F3" s="16" t="n">
+      <c r="F3" s="17" t="n">
         <v>46296</v>
       </c>
-      <c r="G3" s="16" t="n">
+      <c r="G3" s="17" t="n">
         <v>46327</v>
       </c>
-      <c r="H3" s="16" t="n">
+      <c r="H3" s="17" t="n">
         <v>46357</v>
       </c>
-      <c r="I3" s="16" t="n">
+      <c r="I3" s="17" t="n">
         <v>46388</v>
       </c>
-      <c r="J3" s="16" t="n">
+      <c r="J3" s="17" t="n">
         <v>46419</v>
       </c>
-      <c r="K3" s="16" t="n">
+      <c r="K3" s="17" t="n">
         <v>46447</v>
       </c>
-      <c r="L3" s="16" t="n">
+      <c r="L3" s="17" t="n">
         <v>46478</v>
       </c>
-      <c r="M3" s="16" t="n">
+      <c r="M3" s="17" t="n">
         <v>46508</v>
       </c>
-      <c r="N3" s="16" t="n">
+      <c r="N3" s="17" t="n">
         <v>46539</v>
       </c>
-      <c r="O3" s="16" t="n">
+      <c r="O3" s="17" t="n">
         <v>46569</v>
       </c>
-      <c r="P3" s="16" t="n">
+      <c r="P3" s="17" t="n">
         <v>46600</v>
       </c>
-      <c r="Q3" s="16" t="n">
+      <c r="Q3" s="17" t="n">
         <v>46631</v>
       </c>
-      <c r="R3" s="16" t="n">
+      <c r="R3" s="17" t="n">
         <v>46661</v>
       </c>
-      <c r="S3" s="16" t="n">
+      <c r="S3" s="17" t="n">
         <v>46692</v>
       </c>
-      <c r="T3" s="16" t="n">
+      <c r="T3" s="17" t="n">
         <v>46722</v>
       </c>
       <c r="U3" s="3" t="inlineStr">
@@ -1316,80 +1387,80 @@
           <t>Cases delivered (cans)</t>
         </is>
       </c>
-      <c r="B4" s="17" t="n">
+      <c r="B4" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="C4" s="17" t="n">
+      <c r="C4" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="18">
+      <c r="D4" s="19">
         <f>Assumptions!B7</f>
         <v/>
       </c>
-      <c r="E4" s="17" t="n">
+      <c r="E4" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="18">
+      <c r="F4" s="19">
         <f>Assumptions!B8</f>
         <v/>
       </c>
-      <c r="G4" s="18">
+      <c r="G4" s="19">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="H4" s="18">
+      <c r="H4" s="19">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="I4" s="18">
+      <c r="I4" s="19">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="J4" s="18">
+      <c r="J4" s="19">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="K4" s="18">
+      <c r="K4" s="19">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="L4" s="18">
+      <c r="L4" s="19">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="M4" s="18">
+      <c r="M4" s="19">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="N4" s="18">
+      <c r="N4" s="19">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="O4" s="18">
+      <c r="O4" s="19">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="P4" s="18">
+      <c r="P4" s="19">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="Q4" s="18">
+      <c r="Q4" s="19">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="R4" s="18">
+      <c r="R4" s="19">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="S4" s="18">
+      <c r="S4" s="19">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="T4" s="18">
+      <c r="T4" s="19">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="U4" s="19">
+      <c r="U4" s="20">
         <f>SUM(B4:T4)</f>
         <v/>
       </c>
@@ -1400,83 +1471,83 @@
           <t>Can revenue</t>
         </is>
       </c>
-      <c r="B5" s="14">
+      <c r="B5" s="15">
         <f>B4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="C5" s="14">
+      <c r="C5" s="15">
         <f>C4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="D5" s="14">
+      <c r="D5" s="15">
         <f>D4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="E5" s="14">
+      <c r="E5" s="15">
         <f>E4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="F5" s="14">
+      <c r="F5" s="15">
         <f>F4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="G5" s="14">
+      <c r="G5" s="15">
         <f>G4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="H5" s="14">
+      <c r="H5" s="15">
         <f>H4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="I5" s="14">
+      <c r="I5" s="15">
         <f>I4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="J5" s="14">
+      <c r="J5" s="15">
         <f>J4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="K5" s="14">
+      <c r="K5" s="15">
         <f>K4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="L5" s="14">
+      <c r="L5" s="15">
         <f>L4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="M5" s="14">
+      <c r="M5" s="15">
         <f>M4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="N5" s="14">
+      <c r="N5" s="15">
         <f>N4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="O5" s="14">
+      <c r="O5" s="15">
         <f>O4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="P5" s="14">
+      <c r="P5" s="15">
         <f>P4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="Q5" s="14">
+      <c r="Q5" s="15">
         <f>Q4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="R5" s="14">
+      <c r="R5" s="15">
         <f>R4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="S5" s="14">
+      <c r="S5" s="15">
         <f>S4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="T5" s="14">
+      <c r="T5" s="15">
         <f>T4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="U5" s="15">
+      <c r="U5" s="16">
         <f>SUM(B5:T5)</f>
         <v/>
       </c>
@@ -1487,83 +1558,83 @@
           <t>Bottle revenue</t>
         </is>
       </c>
-      <c r="B6" s="20">
+      <c r="B6" s="21">
         <f>Bottles!E9</f>
         <v/>
       </c>
-      <c r="C6" s="20">
+      <c r="C6" s="21">
         <f>Bottles!E10</f>
         <v/>
       </c>
-      <c r="D6" s="20">
+      <c r="D6" s="21">
         <f>Bottles!E11</f>
         <v/>
       </c>
-      <c r="E6" s="20">
+      <c r="E6" s="21">
         <f>Bottles!E12</f>
         <v/>
       </c>
-      <c r="F6" s="20">
+      <c r="F6" s="21">
         <f>Bottles!E13</f>
         <v/>
       </c>
-      <c r="G6" s="20">
+      <c r="G6" s="21">
         <f>Bottles!E14</f>
         <v/>
       </c>
-      <c r="H6" s="20">
+      <c r="H6" s="21">
         <f>Bottles!E15</f>
         <v/>
       </c>
-      <c r="I6" s="20">
+      <c r="I6" s="21">
         <f>Bottles!G4</f>
         <v/>
       </c>
-      <c r="J6" s="20">
+      <c r="J6" s="21">
         <f>Bottles!G5</f>
         <v/>
       </c>
-      <c r="K6" s="20">
+      <c r="K6" s="21">
         <f>Bottles!G6</f>
         <v/>
       </c>
-      <c r="L6" s="20">
+      <c r="L6" s="21">
         <f>Bottles!G7</f>
         <v/>
       </c>
-      <c r="M6" s="20">
+      <c r="M6" s="21">
         <f>Bottles!G8</f>
         <v/>
       </c>
-      <c r="N6" s="20">
+      <c r="N6" s="21">
         <f>Bottles!G9</f>
         <v/>
       </c>
-      <c r="O6" s="20">
+      <c r="O6" s="21">
         <f>Bottles!G10</f>
         <v/>
       </c>
-      <c r="P6" s="20">
+      <c r="P6" s="21">
         <f>Bottles!G11</f>
         <v/>
       </c>
-      <c r="Q6" s="20">
+      <c r="Q6" s="21">
         <f>Bottles!G12</f>
         <v/>
       </c>
-      <c r="R6" s="20">
+      <c r="R6" s="21">
         <f>Bottles!G13</f>
         <v/>
       </c>
-      <c r="S6" s="20">
+      <c r="S6" s="21">
         <f>Bottles!G14</f>
         <v/>
       </c>
-      <c r="T6" s="20">
+      <c r="T6" s="21">
         <f>Bottles!G15</f>
         <v/>
       </c>
-      <c r="U6" s="15">
+      <c r="U6" s="16">
         <f>SUM(B6:T6)</f>
         <v/>
       </c>
@@ -1574,83 +1645,83 @@
           <t>Total revenue</t>
         </is>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="16">
         <f>B5+B6</f>
         <v/>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="16">
         <f>C5+C6</f>
         <v/>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="16">
         <f>D5+D6</f>
         <v/>
       </c>
-      <c r="E7" s="15">
+      <c r="E7" s="16">
         <f>E5+E6</f>
         <v/>
       </c>
-      <c r="F7" s="15">
+      <c r="F7" s="16">
         <f>F5+F6</f>
         <v/>
       </c>
-      <c r="G7" s="15">
+      <c r="G7" s="16">
         <f>G5+G6</f>
         <v/>
       </c>
-      <c r="H7" s="15">
+      <c r="H7" s="16">
         <f>H5+H6</f>
         <v/>
       </c>
-      <c r="I7" s="15">
+      <c r="I7" s="16">
         <f>I5+I6</f>
         <v/>
       </c>
-      <c r="J7" s="15">
+      <c r="J7" s="16">
         <f>J5+J6</f>
         <v/>
       </c>
-      <c r="K7" s="15">
+      <c r="K7" s="16">
         <f>K5+K6</f>
         <v/>
       </c>
-      <c r="L7" s="15">
+      <c r="L7" s="16">
         <f>L5+L6</f>
         <v/>
       </c>
-      <c r="M7" s="15">
+      <c r="M7" s="16">
         <f>M5+M6</f>
         <v/>
       </c>
-      <c r="N7" s="15">
+      <c r="N7" s="16">
         <f>N5+N6</f>
         <v/>
       </c>
-      <c r="O7" s="15">
+      <c r="O7" s="16">
         <f>O5+O6</f>
         <v/>
       </c>
-      <c r="P7" s="15">
+      <c r="P7" s="16">
         <f>P5+P6</f>
         <v/>
       </c>
-      <c r="Q7" s="15">
+      <c r="Q7" s="16">
         <f>Q5+Q6</f>
         <v/>
       </c>
-      <c r="R7" s="15">
+      <c r="R7" s="16">
         <f>R5+R6</f>
         <v/>
       </c>
-      <c r="S7" s="15">
+      <c r="S7" s="16">
         <f>S5+S6</f>
         <v/>
       </c>
-      <c r="T7" s="15">
+      <c r="T7" s="16">
         <f>T5+T6</f>
         <v/>
       </c>
-      <c r="U7" s="15">
+      <c r="U7" s="16">
         <f>SUM(B7:T7)</f>
         <v/>
       </c>
@@ -1661,83 +1732,83 @@
           <t>Can COGS</t>
         </is>
       </c>
-      <c r="B8" s="14">
+      <c r="B8" s="15">
         <f>-B5*Assumptions!$B$21</f>
         <v/>
       </c>
-      <c r="C8" s="14">
+      <c r="C8" s="15">
         <f>-C5*Assumptions!$B$21</f>
         <v/>
       </c>
-      <c r="D8" s="14">
+      <c r="D8" s="15">
         <f>-D5*Assumptions!$B$21</f>
         <v/>
       </c>
-      <c r="E8" s="14">
+      <c r="E8" s="15">
         <f>-E5*Assumptions!$B$21</f>
         <v/>
       </c>
-      <c r="F8" s="14">
+      <c r="F8" s="15">
         <f>-F5*Assumptions!$B$21</f>
         <v/>
       </c>
-      <c r="G8" s="14">
+      <c r="G8" s="15">
         <f>-G5*Assumptions!$B$21</f>
         <v/>
       </c>
-      <c r="H8" s="14">
+      <c r="H8" s="15">
         <f>-H5*Assumptions!$B$21</f>
         <v/>
       </c>
-      <c r="I8" s="14">
+      <c r="I8" s="15">
         <f>-I5*Assumptions!$B$21</f>
         <v/>
       </c>
-      <c r="J8" s="14">
+      <c r="J8" s="15">
         <f>-J5*Assumptions!$B$21</f>
         <v/>
       </c>
-      <c r="K8" s="14">
+      <c r="K8" s="15">
         <f>-K5*Assumptions!$B$21</f>
         <v/>
       </c>
-      <c r="L8" s="14">
+      <c r="L8" s="15">
         <f>-L5*Assumptions!$B$21</f>
         <v/>
       </c>
-      <c r="M8" s="14">
+      <c r="M8" s="15">
         <f>-M5*Assumptions!$B$21</f>
         <v/>
       </c>
-      <c r="N8" s="14">
+      <c r="N8" s="15">
         <f>-N5*Assumptions!$B$21</f>
         <v/>
       </c>
-      <c r="O8" s="14">
+      <c r="O8" s="15">
         <f>-O5*Assumptions!$B$21</f>
         <v/>
       </c>
-      <c r="P8" s="14">
+      <c r="P8" s="15">
         <f>-P5*Assumptions!$B$21</f>
         <v/>
       </c>
-      <c r="Q8" s="14">
+      <c r="Q8" s="15">
         <f>-Q5*Assumptions!$B$21</f>
         <v/>
       </c>
-      <c r="R8" s="14">
+      <c r="R8" s="15">
         <f>-R5*Assumptions!$B$21</f>
         <v/>
       </c>
-      <c r="S8" s="14">
+      <c r="S8" s="15">
         <f>-S5*Assumptions!$B$21</f>
         <v/>
       </c>
-      <c r="T8" s="14">
+      <c r="T8" s="15">
         <f>-T5*Assumptions!$B$21</f>
         <v/>
       </c>
-      <c r="U8" s="15">
+      <c r="U8" s="16">
         <f>SUM(B8:T8)</f>
         <v/>
       </c>
@@ -1748,83 +1819,83 @@
           <t>Bottle COGS</t>
         </is>
       </c>
-      <c r="B9" s="14">
+      <c r="B9" s="15">
         <f>-B6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="C9" s="14">
+      <c r="C9" s="15">
         <f>-C6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="D9" s="14">
+      <c r="D9" s="15">
         <f>-D6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="E9" s="14">
+      <c r="E9" s="15">
         <f>-E6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="F9" s="14">
+      <c r="F9" s="15">
         <f>-F6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="G9" s="14">
+      <c r="G9" s="15">
         <f>-G6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="H9" s="14">
+      <c r="H9" s="15">
         <f>-H6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="I9" s="14">
+      <c r="I9" s="15">
         <f>-I6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="J9" s="14">
+      <c r="J9" s="15">
         <f>-J6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="K9" s="14">
+      <c r="K9" s="15">
         <f>-K6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="L9" s="14">
+      <c r="L9" s="15">
         <f>-L6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="M9" s="14">
+      <c r="M9" s="15">
         <f>-M6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="N9" s="14">
+      <c r="N9" s="15">
         <f>-N6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="O9" s="14">
+      <c r="O9" s="15">
         <f>-O6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="P9" s="14">
+      <c r="P9" s="15">
         <f>-P6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="Q9" s="14">
+      <c r="Q9" s="15">
         <f>-Q6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="R9" s="14">
+      <c r="R9" s="15">
         <f>-R6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="S9" s="14">
+      <c r="S9" s="15">
         <f>-S6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="T9" s="14">
+      <c r="T9" s="15">
         <f>-T6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="U9" s="15">
+      <c r="U9" s="16">
         <f>SUM(B9:T9)</f>
         <v/>
       </c>
@@ -1835,83 +1906,83 @@
           <t>Gross margin</t>
         </is>
       </c>
-      <c r="B10" s="15">
+      <c r="B10" s="16">
         <f>B7+B8+B9</f>
         <v/>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="16">
         <f>C7+C8+C9</f>
         <v/>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="16">
         <f>D7+D8+D9</f>
         <v/>
       </c>
-      <c r="E10" s="15">
+      <c r="E10" s="16">
         <f>E7+E8+E9</f>
         <v/>
       </c>
-      <c r="F10" s="15">
+      <c r="F10" s="16">
         <f>F7+F8+F9</f>
         <v/>
       </c>
-      <c r="G10" s="15">
+      <c r="G10" s="16">
         <f>G7+G8+G9</f>
         <v/>
       </c>
-      <c r="H10" s="15">
+      <c r="H10" s="16">
         <f>H7+H8+H9</f>
         <v/>
       </c>
-      <c r="I10" s="15">
+      <c r="I10" s="16">
         <f>I7+I8+I9</f>
         <v/>
       </c>
-      <c r="J10" s="15">
+      <c r="J10" s="16">
         <f>J7+J8+J9</f>
         <v/>
       </c>
-      <c r="K10" s="15">
+      <c r="K10" s="16">
         <f>K7+K8+K9</f>
         <v/>
       </c>
-      <c r="L10" s="15">
+      <c r="L10" s="16">
         <f>L7+L8+L9</f>
         <v/>
       </c>
-      <c r="M10" s="15">
+      <c r="M10" s="16">
         <f>M7+M8+M9</f>
         <v/>
       </c>
-      <c r="N10" s="15">
+      <c r="N10" s="16">
         <f>N7+N8+N9</f>
         <v/>
       </c>
-      <c r="O10" s="15">
+      <c r="O10" s="16">
         <f>O7+O8+O9</f>
         <v/>
       </c>
-      <c r="P10" s="15">
+      <c r="P10" s="16">
         <f>P7+P8+P9</f>
         <v/>
       </c>
-      <c r="Q10" s="15">
+      <c r="Q10" s="16">
         <f>Q7+Q8+Q9</f>
         <v/>
       </c>
-      <c r="R10" s="15">
+      <c r="R10" s="16">
         <f>R7+R8+R9</f>
         <v/>
       </c>
-      <c r="S10" s="15">
+      <c r="S10" s="16">
         <f>S7+S8+S9</f>
         <v/>
       </c>
-      <c r="T10" s="15">
+      <c r="T10" s="16">
         <f>T7+T8+T9</f>
         <v/>
       </c>
-      <c r="U10" s="15">
+      <c r="U10" s="16">
         <f>SUM(B10:T10)</f>
         <v/>
       </c>
@@ -1998,7 +2069,7 @@
         <f>IF(T7=0,0,T10/T7)</f>
         <v/>
       </c>
-      <c r="U11" s="21">
+      <c r="U11" s="22">
         <f>U10/U7</f>
         <v/>
       </c>
@@ -2009,83 +2080,83 @@
           <t>Opex (legal &amp; admin)</t>
         </is>
       </c>
-      <c r="B12" s="14">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="C12" s="14">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="D12" s="14">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="E12" s="14">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="F12" s="14">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="G12" s="14">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="H12" s="14">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="I12" s="14">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="J12" s="14">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="K12" s="14">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="L12" s="14">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="M12" s="14">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="N12" s="14">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="O12" s="14">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="P12" s="14">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="Q12" s="14">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="R12" s="14">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="S12" s="14">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="T12" s="14">
-        <f>-Assumptions!$B$23</f>
-        <v/>
-      </c>
-      <c r="U12" s="15">
+      <c r="B12" s="15">
+        <f>-(Assumptions!$B$23+IF(B$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(B$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="C12" s="15">
+        <f>-(Assumptions!$B$23+IF(C$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(C$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="D12" s="15">
+        <f>-(Assumptions!$B$23+IF(D$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(D$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="E12" s="15">
+        <f>-(Assumptions!$B$23+IF(E$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(E$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="F12" s="15">
+        <f>-(Assumptions!$B$23+IF(F$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(F$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="G12" s="15">
+        <f>-(Assumptions!$B$23+IF(G$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(G$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="H12" s="15">
+        <f>-(Assumptions!$B$23+IF(H$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(H$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="I12" s="15">
+        <f>-(Assumptions!$B$23+IF(I$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(I$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="J12" s="15">
+        <f>-(Assumptions!$B$23+IF(J$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(J$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="K12" s="15">
+        <f>-(Assumptions!$B$23+IF(K$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(K$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="L12" s="15">
+        <f>-(Assumptions!$B$23+IF(L$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(L$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="M12" s="15">
+        <f>-(Assumptions!$B$23+IF(M$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(M$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="N12" s="15">
+        <f>-(Assumptions!$B$23+IF(N$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(N$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="O12" s="15">
+        <f>-(Assumptions!$B$23+IF(O$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(O$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="P12" s="15">
+        <f>-(Assumptions!$B$23+IF(P$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(P$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="Q12" s="15">
+        <f>-(Assumptions!$B$23+IF(Q$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(Q$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="R12" s="15">
+        <f>-(Assumptions!$B$23+IF(R$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(R$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="S12" s="15">
+        <f>-(Assumptions!$B$23+IF(S$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(S$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="T12" s="15">
+        <f>-(Assumptions!$B$23+IF(T$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(T$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="U12" s="16">
         <f>SUM(B12:T12)</f>
         <v/>
       </c>
@@ -2096,83 +2167,83 @@
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="B13" s="15">
+      <c r="B13" s="16">
         <f>B10+B12</f>
         <v/>
       </c>
-      <c r="C13" s="15">
+      <c r="C13" s="16">
         <f>C10+C12</f>
         <v/>
       </c>
-      <c r="D13" s="15">
+      <c r="D13" s="16">
         <f>D10+D12</f>
         <v/>
       </c>
-      <c r="E13" s="15">
+      <c r="E13" s="16">
         <f>E10+E12</f>
         <v/>
       </c>
-      <c r="F13" s="15">
+      <c r="F13" s="16">
         <f>F10+F12</f>
         <v/>
       </c>
-      <c r="G13" s="15">
+      <c r="G13" s="16">
         <f>G10+G12</f>
         <v/>
       </c>
-      <c r="H13" s="15">
+      <c r="H13" s="16">
         <f>H10+H12</f>
         <v/>
       </c>
-      <c r="I13" s="15">
+      <c r="I13" s="16">
         <f>I10+I12</f>
         <v/>
       </c>
-      <c r="J13" s="15">
+      <c r="J13" s="16">
         <f>J10+J12</f>
         <v/>
       </c>
-      <c r="K13" s="15">
+      <c r="K13" s="16">
         <f>K10+K12</f>
         <v/>
       </c>
-      <c r="L13" s="15">
+      <c r="L13" s="16">
         <f>L10+L12</f>
         <v/>
       </c>
-      <c r="M13" s="15">
+      <c r="M13" s="16">
         <f>M10+M12</f>
         <v/>
       </c>
-      <c r="N13" s="15">
+      <c r="N13" s="16">
         <f>N10+N12</f>
         <v/>
       </c>
-      <c r="O13" s="15">
+      <c r="O13" s="16">
         <f>O10+O12</f>
         <v/>
       </c>
-      <c r="P13" s="15">
+      <c r="P13" s="16">
         <f>P10+P12</f>
         <v/>
       </c>
-      <c r="Q13" s="15">
+      <c r="Q13" s="16">
         <f>Q10+Q12</f>
         <v/>
       </c>
-      <c r="R13" s="15">
+      <c r="R13" s="16">
         <f>R10+R12</f>
         <v/>
       </c>
-      <c r="S13" s="15">
+      <c r="S13" s="16">
         <f>S10+S12</f>
         <v/>
       </c>
-      <c r="T13" s="15">
+      <c r="T13" s="16">
         <f>T10+T12</f>
         <v/>
       </c>
-      <c r="U13" s="15">
+      <c r="U13" s="16">
         <f>SUM(B13:T13)</f>
         <v/>
       </c>
@@ -2259,7 +2330,7 @@
         <f>IF(T7=0,0,T13/T7)</f>
         <v/>
       </c>
-      <c r="U14" s="21">
+      <c r="U14" s="22">
         <f>U13/U7</f>
         <v/>
       </c>
@@ -2313,61 +2384,61 @@
           <t>Month</t>
         </is>
       </c>
-      <c r="B3" s="16" t="n">
+      <c r="B3" s="17" t="n">
         <v>46174</v>
       </c>
-      <c r="C3" s="16" t="n">
+      <c r="C3" s="17" t="n">
         <v>46204</v>
       </c>
-      <c r="D3" s="16" t="n">
+      <c r="D3" s="17" t="n">
         <v>46235</v>
       </c>
-      <c r="E3" s="16" t="n">
+      <c r="E3" s="17" t="n">
         <v>46266</v>
       </c>
-      <c r="F3" s="16" t="n">
+      <c r="F3" s="17" t="n">
         <v>46296</v>
       </c>
-      <c r="G3" s="16" t="n">
+      <c r="G3" s="17" t="n">
         <v>46327</v>
       </c>
-      <c r="H3" s="16" t="n">
+      <c r="H3" s="17" t="n">
         <v>46357</v>
       </c>
-      <c r="I3" s="16" t="n">
+      <c r="I3" s="17" t="n">
         <v>46388</v>
       </c>
-      <c r="J3" s="16" t="n">
+      <c r="J3" s="17" t="n">
         <v>46419</v>
       </c>
-      <c r="K3" s="16" t="n">
+      <c r="K3" s="17" t="n">
         <v>46447</v>
       </c>
-      <c r="L3" s="16" t="n">
+      <c r="L3" s="17" t="n">
         <v>46478</v>
       </c>
-      <c r="M3" s="16" t="n">
+      <c r="M3" s="17" t="n">
         <v>46508</v>
       </c>
-      <c r="N3" s="16" t="n">
+      <c r="N3" s="17" t="n">
         <v>46539</v>
       </c>
-      <c r="O3" s="16" t="n">
+      <c r="O3" s="17" t="n">
         <v>46569</v>
       </c>
-      <c r="P3" s="16" t="n">
+      <c r="P3" s="17" t="n">
         <v>46600</v>
       </c>
-      <c r="Q3" s="16" t="n">
+      <c r="Q3" s="17" t="n">
         <v>46631</v>
       </c>
-      <c r="R3" s="16" t="n">
+      <c r="R3" s="17" t="n">
         <v>46661</v>
       </c>
-      <c r="S3" s="16" t="n">
+      <c r="S3" s="17" t="n">
         <v>46692</v>
       </c>
-      <c r="T3" s="16" t="n">
+      <c r="T3" s="17" t="n">
         <v>46722</v>
       </c>
       <c r="U3" s="3" t="inlineStr">
@@ -2382,82 +2453,82 @@
           <t>Can receipts (revenue +30 days)</t>
         </is>
       </c>
-      <c r="B4" s="14" t="n">
+      <c r="B4" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="C4" s="20">
+      <c r="C4" s="21">
         <f>'P&amp;L'!B5</f>
         <v/>
       </c>
-      <c r="D4" s="20">
+      <c r="D4" s="21">
         <f>'P&amp;L'!C5</f>
         <v/>
       </c>
-      <c r="E4" s="20">
+      <c r="E4" s="21">
         <f>'P&amp;L'!D5</f>
         <v/>
       </c>
-      <c r="F4" s="20">
+      <c r="F4" s="21">
         <f>'P&amp;L'!E5</f>
         <v/>
       </c>
-      <c r="G4" s="20">
+      <c r="G4" s="21">
         <f>'P&amp;L'!F5</f>
         <v/>
       </c>
-      <c r="H4" s="20">
+      <c r="H4" s="21">
         <f>'P&amp;L'!G5</f>
         <v/>
       </c>
-      <c r="I4" s="20">
+      <c r="I4" s="21">
         <f>'P&amp;L'!H5</f>
         <v/>
       </c>
-      <c r="J4" s="20">
+      <c r="J4" s="21">
         <f>'P&amp;L'!I5</f>
         <v/>
       </c>
-      <c r="K4" s="20">
+      <c r="K4" s="21">
         <f>'P&amp;L'!J5</f>
         <v/>
       </c>
-      <c r="L4" s="20">
+      <c r="L4" s="21">
         <f>'P&amp;L'!K5</f>
         <v/>
       </c>
-      <c r="M4" s="20">
+      <c r="M4" s="21">
         <f>'P&amp;L'!L5</f>
         <v/>
       </c>
-      <c r="N4" s="20">
+      <c r="N4" s="21">
         <f>'P&amp;L'!M5</f>
         <v/>
       </c>
-      <c r="O4" s="20">
+      <c r="O4" s="21">
         <f>'P&amp;L'!N5</f>
         <v/>
       </c>
-      <c r="P4" s="20">
+      <c r="P4" s="21">
         <f>'P&amp;L'!O5</f>
         <v/>
       </c>
-      <c r="Q4" s="20">
+      <c r="Q4" s="21">
         <f>'P&amp;L'!P5</f>
         <v/>
       </c>
-      <c r="R4" s="20">
+      <c r="R4" s="21">
         <f>'P&amp;L'!Q5</f>
         <v/>
       </c>
-      <c r="S4" s="20">
+      <c r="S4" s="21">
         <f>'P&amp;L'!R5</f>
         <v/>
       </c>
-      <c r="T4" s="20">
+      <c r="T4" s="21">
         <f>'P&amp;L'!S5</f>
         <v/>
       </c>
-      <c r="U4" s="15">
+      <c r="U4" s="16">
         <f>SUM(B4:T4)</f>
         <v/>
       </c>
@@ -2468,15 +2539,15 @@
           <t xml:space="preserve">  Bron Pro (design/brand)</t>
         </is>
       </c>
-      <c r="B5" s="14">
+      <c r="B5" s="15">
         <f>-103500*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="D5" s="14">
+      <c r="D5" s="15">
         <f>-243800*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="U5" s="14">
+      <c r="U5" s="15">
         <f>SUM(B5:T5)</f>
         <v/>
       </c>
@@ -2487,15 +2558,15 @@
           <t xml:space="preserve">  Sullwaldt printing</t>
         </is>
       </c>
-      <c r="C6" s="14">
+      <c r="C6" s="15">
         <f>-91066*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="F6" s="14">
+      <c r="F6" s="15">
         <f>-72400*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="U6" s="14">
+      <c r="U6" s="15">
         <f>SUM(B6:T6)</f>
         <v/>
       </c>
@@ -2506,15 +2577,15 @@
           <t xml:space="preserve">  Tiny Keg cans</t>
         </is>
       </c>
-      <c r="C7" s="14">
+      <c r="C7" s="15">
         <f>-405950*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="E7" s="14">
+      <c r="E7" s="15">
         <f>-319000*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="U7" s="14">
+      <c r="U7" s="15">
         <f>SUM(B7:T7)</f>
         <v/>
       </c>
@@ -2525,11 +2596,11 @@
           <t xml:space="preserve">  Chep pallets</t>
         </is>
       </c>
-      <c r="B8" s="14">
+      <c r="B8" s="15">
         <f>-14375*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="U8" s="14">
+      <c r="U8" s="15">
         <f>SUM(B8:T8)</f>
         <v/>
       </c>
@@ -2540,15 +2611,15 @@
           <t xml:space="preserve">  FAL distribution</t>
         </is>
       </c>
-      <c r="C9" s="14">
+      <c r="C9" s="15">
         <f>-51750*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="F9" s="14">
+      <c r="F9" s="15">
         <f>-28000*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="U9" s="14">
+      <c r="U9" s="15">
         <f>SUM(B9:T9)</f>
         <v/>
       </c>
@@ -2559,15 +2630,15 @@
           <t xml:space="preserve">  Tiny Keg production</t>
         </is>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="15">
         <f>-373350*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="E10" s="14">
+      <c r="E10" s="15">
         <f>-293250*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="U10" s="14">
+      <c r="U10" s="15">
         <f>SUM(B10:T10)</f>
         <v/>
       </c>
@@ -2578,15 +2649,15 @@
           <t xml:space="preserve">  SARS excise (launch)</t>
         </is>
       </c>
-      <c r="E11" s="14">
+      <c r="E11" s="15">
         <f>-630000*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="G11" s="14">
+      <c r="G11" s="15">
         <f>-495571*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="U11" s="14">
+      <c r="U11" s="15">
         <f>SUM(B11:T11)</f>
         <v/>
       </c>
@@ -2594,13 +2665,86 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Legal &amp; admin (2026)</t>
-        </is>
-      </c>
-      <c r="C12" s="14" t="n">
-        <v>-57500</v>
-      </c>
-      <c r="U12" s="14">
+          <t xml:space="preserve">  Opex (sales, ops, marketing, admin — paid monthly)</t>
+        </is>
+      </c>
+      <c r="B12" s="21">
+        <f>'P&amp;L'!B12</f>
+        <v/>
+      </c>
+      <c r="C12" s="21">
+        <f>'P&amp;L'!C12</f>
+        <v/>
+      </c>
+      <c r="D12" s="21">
+        <f>'P&amp;L'!D12</f>
+        <v/>
+      </c>
+      <c r="E12" s="21">
+        <f>'P&amp;L'!E12</f>
+        <v/>
+      </c>
+      <c r="F12" s="21">
+        <f>'P&amp;L'!F12</f>
+        <v/>
+      </c>
+      <c r="G12" s="21">
+        <f>'P&amp;L'!G12</f>
+        <v/>
+      </c>
+      <c r="H12" s="21">
+        <f>'P&amp;L'!H12</f>
+        <v/>
+      </c>
+      <c r="I12" s="21">
+        <f>'P&amp;L'!I12</f>
+        <v/>
+      </c>
+      <c r="J12" s="21">
+        <f>'P&amp;L'!J12</f>
+        <v/>
+      </c>
+      <c r="K12" s="21">
+        <f>'P&amp;L'!K12</f>
+        <v/>
+      </c>
+      <c r="L12" s="21">
+        <f>'P&amp;L'!L12</f>
+        <v/>
+      </c>
+      <c r="M12" s="21">
+        <f>'P&amp;L'!M12</f>
+        <v/>
+      </c>
+      <c r="N12" s="21">
+        <f>'P&amp;L'!N12</f>
+        <v/>
+      </c>
+      <c r="O12" s="21">
+        <f>'P&amp;L'!O12</f>
+        <v/>
+      </c>
+      <c r="P12" s="21">
+        <f>'P&amp;L'!P12</f>
+        <v/>
+      </c>
+      <c r="Q12" s="21">
+        <f>'P&amp;L'!Q12</f>
+        <v/>
+      </c>
+      <c r="R12" s="21">
+        <f>'P&amp;L'!R12</f>
+        <v/>
+      </c>
+      <c r="S12" s="21">
+        <f>'P&amp;L'!S12</f>
+        <v/>
+      </c>
+      <c r="T12" s="21">
+        <f>'P&amp;L'!T12</f>
+        <v/>
+      </c>
+      <c r="U12" s="15">
         <f>SUM(B12:T12)</f>
         <v/>
       </c>
@@ -2611,83 +2755,83 @@
           <t xml:space="preserve">  Bottles net contribution (GM, cash in month)</t>
         </is>
       </c>
-      <c r="B13" s="20">
+      <c r="B13" s="21">
         <f>'P&amp;L'!B6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="C13" s="20">
+      <c r="C13" s="21">
         <f>'P&amp;L'!C6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="D13" s="20">
+      <c r="D13" s="21">
         <f>'P&amp;L'!D6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="E13" s="20">
+      <c r="E13" s="21">
         <f>'P&amp;L'!E6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="F13" s="20">
+      <c r="F13" s="21">
         <f>'P&amp;L'!F6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="G13" s="20">
+      <c r="G13" s="21">
         <f>'P&amp;L'!G6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="H13" s="20">
+      <c r="H13" s="21">
         <f>'P&amp;L'!H6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="I13" s="20">
+      <c r="I13" s="21">
         <f>'P&amp;L'!I6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="J13" s="20">
+      <c r="J13" s="21">
         <f>'P&amp;L'!J6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="K13" s="20">
+      <c r="K13" s="21">
         <f>'P&amp;L'!K6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="L13" s="20">
+      <c r="L13" s="21">
         <f>'P&amp;L'!L6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="M13" s="20">
+      <c r="M13" s="21">
         <f>'P&amp;L'!M6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="N13" s="20">
+      <c r="N13" s="21">
         <f>'P&amp;L'!N6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="O13" s="20">
+      <c r="O13" s="21">
         <f>'P&amp;L'!O6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="P13" s="20">
+      <c r="P13" s="21">
         <f>'P&amp;L'!P6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="Q13" s="20">
+      <c r="Q13" s="21">
         <f>'P&amp;L'!Q6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="R13" s="20">
+      <c r="R13" s="21">
         <f>'P&amp;L'!R6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="S13" s="20">
+      <c r="S13" s="21">
         <f>'P&amp;L'!S6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="T13" s="20">
+      <c r="T13" s="21">
         <f>'P&amp;L'!T6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="U13" s="14">
+      <c r="U13" s="15">
         <f>SUM(B13:T13)</f>
         <v/>
       </c>
@@ -2695,58 +2839,58 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2027 recurring can COGS + opex</t>
-        </is>
-      </c>
-      <c r="I14" s="14">
-        <f>-('P&amp;L'!I5*Assumptions!$B$21+Assumptions!$B$23)</f>
-        <v/>
-      </c>
-      <c r="J14" s="14">
-        <f>-('P&amp;L'!J5*Assumptions!$B$21+Assumptions!$B$23)</f>
-        <v/>
-      </c>
-      <c r="K14" s="14">
-        <f>-('P&amp;L'!K5*Assumptions!$B$21+Assumptions!$B$23)</f>
-        <v/>
-      </c>
-      <c r="L14" s="14">
-        <f>-('P&amp;L'!L5*Assumptions!$B$21+Assumptions!$B$23)</f>
-        <v/>
-      </c>
-      <c r="M14" s="14">
-        <f>-('P&amp;L'!M5*Assumptions!$B$21+Assumptions!$B$23)</f>
-        <v/>
-      </c>
-      <c r="N14" s="14">
-        <f>-('P&amp;L'!N5*Assumptions!$B$21+Assumptions!$B$23)</f>
-        <v/>
-      </c>
-      <c r="O14" s="14">
-        <f>-('P&amp;L'!O5*Assumptions!$B$21+Assumptions!$B$23)</f>
-        <v/>
-      </c>
-      <c r="P14" s="14">
-        <f>-('P&amp;L'!P5*Assumptions!$B$21+Assumptions!$B$23)</f>
-        <v/>
-      </c>
-      <c r="Q14" s="14">
-        <f>-('P&amp;L'!Q5*Assumptions!$B$21+Assumptions!$B$23)</f>
-        <v/>
-      </c>
-      <c r="R14" s="14">
-        <f>-('P&amp;L'!R5*Assumptions!$B$21+Assumptions!$B$23)</f>
-        <v/>
-      </c>
-      <c r="S14" s="14">
-        <f>-('P&amp;L'!S5*Assumptions!$B$21+Assumptions!$B$23)</f>
-        <v/>
-      </c>
-      <c r="T14" s="14">
-        <f>-('P&amp;L'!T5*Assumptions!$B$21+Assumptions!$B$23)</f>
-        <v/>
-      </c>
-      <c r="U14" s="14">
+          <t xml:space="preserve">  2027 recurring can COGS</t>
+        </is>
+      </c>
+      <c r="I14" s="15">
+        <f>-'P&amp;L'!I5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="J14" s="15">
+        <f>-'P&amp;L'!J5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="K14" s="15">
+        <f>-'P&amp;L'!K5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="L14" s="15">
+        <f>-'P&amp;L'!L5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="M14" s="15">
+        <f>-'P&amp;L'!M5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="N14" s="15">
+        <f>-'P&amp;L'!N5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="O14" s="15">
+        <f>-'P&amp;L'!O5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="P14" s="15">
+        <f>-'P&amp;L'!P5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="Q14" s="15">
+        <f>-'P&amp;L'!Q5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="R14" s="15">
+        <f>-'P&amp;L'!R5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="S14" s="15">
+        <f>-'P&amp;L'!S5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="T14" s="15">
+        <f>-'P&amp;L'!T5*Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="U14" s="15">
         <f>SUM(B14:T14)</f>
         <v/>
       </c>
@@ -2757,83 +2901,83 @@
           <t>Net monthly cashflow</t>
         </is>
       </c>
-      <c r="B15" s="15">
+      <c r="B15" s="16">
         <f>SUM(B4:B14)</f>
         <v/>
       </c>
-      <c r="C15" s="15">
+      <c r="C15" s="16">
         <f>SUM(C4:C14)</f>
         <v/>
       </c>
-      <c r="D15" s="15">
+      <c r="D15" s="16">
         <f>SUM(D4:D14)</f>
         <v/>
       </c>
-      <c r="E15" s="15">
+      <c r="E15" s="16">
         <f>SUM(E4:E14)</f>
         <v/>
       </c>
-      <c r="F15" s="15">
+      <c r="F15" s="16">
         <f>SUM(F4:F14)</f>
         <v/>
       </c>
-      <c r="G15" s="15">
+      <c r="G15" s="16">
         <f>SUM(G4:G14)</f>
         <v/>
       </c>
-      <c r="H15" s="15">
+      <c r="H15" s="16">
         <f>SUM(H4:H14)</f>
         <v/>
       </c>
-      <c r="I15" s="15">
+      <c r="I15" s="16">
         <f>SUM(I4:I14)</f>
         <v/>
       </c>
-      <c r="J15" s="15">
+      <c r="J15" s="16">
         <f>SUM(J4:J14)</f>
         <v/>
       </c>
-      <c r="K15" s="15">
+      <c r="K15" s="16">
         <f>SUM(K4:K14)</f>
         <v/>
       </c>
-      <c r="L15" s="15">
+      <c r="L15" s="16">
         <f>SUM(L4:L14)</f>
         <v/>
       </c>
-      <c r="M15" s="15">
+      <c r="M15" s="16">
         <f>SUM(M4:M14)</f>
         <v/>
       </c>
-      <c r="N15" s="15">
+      <c r="N15" s="16">
         <f>SUM(N4:N14)</f>
         <v/>
       </c>
-      <c r="O15" s="15">
+      <c r="O15" s="16">
         <f>SUM(O4:O14)</f>
         <v/>
       </c>
-      <c r="P15" s="15">
+      <c r="P15" s="16">
         <f>SUM(P4:P14)</f>
         <v/>
       </c>
-      <c r="Q15" s="15">
+      <c r="Q15" s="16">
         <f>SUM(Q4:Q14)</f>
         <v/>
       </c>
-      <c r="R15" s="15">
+      <c r="R15" s="16">
         <f>SUM(R4:R14)</f>
         <v/>
       </c>
-      <c r="S15" s="15">
+      <c r="S15" s="16">
         <f>SUM(S4:S14)</f>
         <v/>
       </c>
-      <c r="T15" s="15">
+      <c r="T15" s="16">
         <f>SUM(T4:T14)</f>
         <v/>
       </c>
-      <c r="U15" s="15">
+      <c r="U15" s="16">
         <f>SUM(B15:T15)</f>
         <v/>
       </c>
@@ -2844,79 +2988,79 @@
           <t>Cumulative cash position</t>
         </is>
       </c>
-      <c r="B16" s="15">
+      <c r="B16" s="16">
         <f>B15</f>
         <v/>
       </c>
-      <c r="C16" s="15">
+      <c r="C16" s="16">
         <f>B16+C15</f>
         <v/>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="16">
         <f>C16+D15</f>
         <v/>
       </c>
-      <c r="E16" s="15">
+      <c r="E16" s="16">
         <f>D16+E15</f>
         <v/>
       </c>
-      <c r="F16" s="15">
+      <c r="F16" s="16">
         <f>E16+F15</f>
         <v/>
       </c>
-      <c r="G16" s="15">
+      <c r="G16" s="16">
         <f>F16+G15</f>
         <v/>
       </c>
-      <c r="H16" s="15">
+      <c r="H16" s="16">
         <f>G16+H15</f>
         <v/>
       </c>
-      <c r="I16" s="15">
+      <c r="I16" s="16">
         <f>H16+I15</f>
         <v/>
       </c>
-      <c r="J16" s="15">
+      <c r="J16" s="16">
         <f>I16+J15</f>
         <v/>
       </c>
-      <c r="K16" s="15">
+      <c r="K16" s="16">
         <f>J16+K15</f>
         <v/>
       </c>
-      <c r="L16" s="15">
+      <c r="L16" s="16">
         <f>K16+L15</f>
         <v/>
       </c>
-      <c r="M16" s="15">
+      <c r="M16" s="16">
         <f>L16+M15</f>
         <v/>
       </c>
-      <c r="N16" s="15">
+      <c r="N16" s="16">
         <f>M16+N15</f>
         <v/>
       </c>
-      <c r="O16" s="15">
+      <c r="O16" s="16">
         <f>N16+O15</f>
         <v/>
       </c>
-      <c r="P16" s="15">
+      <c r="P16" s="16">
         <f>O16+P15</f>
         <v/>
       </c>
-      <c r="Q16" s="15">
+      <c r="Q16" s="16">
         <f>P16+Q15</f>
         <v/>
       </c>
-      <c r="R16" s="15">
+      <c r="R16" s="16">
         <f>Q16+R15</f>
         <v/>
       </c>
-      <c r="S16" s="15">
+      <c r="S16" s="16">
         <f>R16+S15</f>
         <v/>
       </c>
-      <c r="T16" s="15">
+      <c r="T16" s="16">
         <f>S16+T15</f>
         <v/>
       </c>
@@ -2976,7 +3120,7 @@
           <t>2026 (Jun–Dec) revenue</t>
         </is>
       </c>
-      <c r="B4" s="20">
+      <c r="B4" s="21">
         <f>SUM('P&amp;L'!B7:H7)</f>
         <v/>
       </c>
@@ -2987,7 +3131,7 @@
           <t>2026 (Jun–Dec) EBITDA</t>
         </is>
       </c>
-      <c r="B5" s="20">
+      <c r="B5" s="21">
         <f>SUM('P&amp;L'!B13:H13)</f>
         <v/>
       </c>
@@ -2998,7 +3142,7 @@
           <t>2027 revenue</t>
         </is>
       </c>
-      <c r="B6" s="20">
+      <c r="B6" s="21">
         <f>SUM('P&amp;L'!I7:T7)</f>
         <v/>
       </c>
@@ -3009,7 +3153,7 @@
           <t>2027 EBITDA</t>
         </is>
       </c>
-      <c r="B7" s="20">
+      <c r="B7" s="21">
         <f>SUM('P&amp;L'!I13:T13)</f>
         <v/>
       </c>
@@ -3042,13 +3186,13 @@
           <t>Multiple</t>
         </is>
       </c>
-      <c r="B10" s="22" t="n">
+      <c r="B10" s="23" t="n">
         <v>6</v>
       </c>
-      <c r="C10" s="22" t="n">
+      <c r="C10" s="23" t="n">
         <v>9</v>
       </c>
-      <c r="D10" s="22" t="n">
+      <c r="D10" s="23" t="n">
         <v>12</v>
       </c>
     </row>
@@ -3058,15 +3202,15 @@
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="B11" s="14">
+      <c r="B11" s="15">
         <f>$B$7*B10</f>
         <v/>
       </c>
-      <c r="C11" s="14">
+      <c r="C11" s="15">
         <f>$B$7*C10</f>
         <v/>
       </c>
-      <c r="D11" s="14">
+      <c r="D11" s="15">
         <f>$B$7*D10</f>
         <v/>
       </c>
@@ -3084,13 +3228,13 @@
           <t>Multiple</t>
         </is>
       </c>
-      <c r="B14" s="22" t="n">
+      <c r="B14" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="C14" s="22" t="n">
+      <c r="C14" s="23" t="n">
         <v>1.5</v>
       </c>
-      <c r="D14" s="22" t="n">
+      <c r="D14" s="23" t="n">
         <v>2.5</v>
       </c>
     </row>
@@ -3100,15 +3244,15 @@
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="B15" s="14">
+      <c r="B15" s="15">
         <f>$B$6*B14</f>
         <v/>
       </c>
-      <c r="C15" s="14">
+      <c r="C15" s="15">
         <f>$B$6*C14</f>
         <v/>
       </c>
-      <c r="D15" s="14">
+      <c r="D15" s="15">
         <f>$B$6*D14</f>
         <v/>
       </c>
@@ -3142,13 +3286,13 @@
           <t>Exit multiple (2027 EBITDA)</t>
         </is>
       </c>
-      <c r="B19" s="22" t="n">
+      <c r="B19" s="23" t="n">
         <v>6</v>
       </c>
-      <c r="C19" s="22" t="n">
+      <c r="C19" s="23" t="n">
         <v>8</v>
       </c>
-      <c r="D19" s="22" t="n">
+      <c r="D19" s="23" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3158,15 +3302,15 @@
           <t>Enterprise value (DCF)</t>
         </is>
       </c>
-      <c r="B20" s="14">
+      <c r="B20" s="15">
         <f>$B$5/(1+B18)^0.25+$B$7/(1+B18)+$B$7*B19/(1+B18)^1.5</f>
         <v/>
       </c>
-      <c r="C20" s="14">
+      <c r="C20" s="15">
         <f>$B$5/(1+C18)^0.25+$B$7/(1+C18)+$B$7*C19/(1+C18)^1.5</f>
         <v/>
       </c>
-      <c r="D20" s="14">
+      <c r="D20" s="15">
         <f>$B$5/(1+D18)^0.25+$B$7/(1+D18)+$B$7*D19/(1+D18)^1.5</f>
         <v/>
       </c>
@@ -3177,15 +3321,15 @@
           <t>Blended enterprise value (avg of methods)</t>
         </is>
       </c>
-      <c r="B22" s="15">
+      <c r="B22" s="16">
         <f>AVERAGE(B11,B15,B20)</f>
         <v/>
       </c>
-      <c r="C22" s="15">
+      <c r="C22" s="16">
         <f>AVERAGE(C11,C15,C20)</f>
         <v/>
       </c>
-      <c r="D22" s="15">
+      <c r="D22" s="16">
         <f>AVERAGE(D11,D15,D20)</f>
         <v/>
       </c>
@@ -3196,7 +3340,7 @@
           <t>Valuation guide for the raise</t>
         </is>
       </c>
-      <c r="B24" s="23" t="n">
+      <c r="B24" s="14" t="n">
         <v>15000000</v>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -3254,7 +3398,7 @@
           <t>Opening order (initial fill revenue)</t>
         </is>
       </c>
-      <c r="B4" s="20">
+      <c r="B4" s="21">
         <f>'P&amp;L'!D5</f>
         <v/>
       </c>
@@ -3265,7 +3409,7 @@
           <t>Bottle revenue (Jun 26 – Dec 27)</t>
         </is>
       </c>
-      <c r="B5" s="20">
+      <c r="B5" s="21">
         <f>'P&amp;L'!U6</f>
         <v/>
       </c>
@@ -3276,7 +3420,7 @@
           <t>Total revenue, cans + bottles (Jun 26 – Dec 27)</t>
         </is>
       </c>
-      <c r="B6" s="20">
+      <c r="B6" s="21">
         <f>'P&amp;L'!U7</f>
         <v/>
       </c>
@@ -3287,7 +3431,7 @@
           <t>Total EBITDA (Jun 26 – Dec 27)</t>
         </is>
       </c>
-      <c r="B7" s="20">
+      <c r="B7" s="21">
         <f>'P&amp;L'!U13</f>
         <v/>
       </c>
@@ -3309,7 +3453,7 @@
           <t>Peak funding need</t>
         </is>
       </c>
-      <c r="B9" s="20">
+      <c r="B9" s="21">
         <f>MIN(Cashflow!B16:T16)</f>
         <v/>
       </c>
@@ -3320,7 +3464,7 @@
           <t>Ending cash (Dec 27)</t>
         </is>
       </c>
-      <c r="B10" s="20">
+      <c r="B10" s="21">
         <f>Cashflow!T16</f>
         <v/>
       </c>
@@ -3331,7 +3475,7 @@
           <t>Blended valuation — low</t>
         </is>
       </c>
-      <c r="B11" s="20">
+      <c r="B11" s="21">
         <f>Valuation!B22</f>
         <v/>
       </c>
@@ -3342,7 +3486,7 @@
           <t>Blended valuation — base</t>
         </is>
       </c>
-      <c r="B12" s="20">
+      <c r="B12" s="21">
         <f>Valuation!C22</f>
         <v/>
       </c>
@@ -3353,7 +3497,7 @@
           <t>Blended valuation — high</t>
         </is>
       </c>
-      <c r="B13" s="20">
+      <c r="B13" s="21">
         <f>Valuation!D22</f>
         <v/>
       </c>
@@ -3364,7 +3508,7 @@
           <t>Valuation guide</t>
         </is>
       </c>
-      <c r="B14" s="20">
+      <c r="B14" s="21">
         <f>Valuation!B24</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Style the Brand Pro Forma to match the house workbook look
Forest banner titles with cream text, chilli section headers, cream label
cells, blue inputs / green cross-sheet links, forest tab colours — per the
Tequila Project Model's styling. Also corrects the P&L opex row label and
a stale cashflow note.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hyws6xeXfxtGdqZV2paNDe
</commit_message>
<xml_diff>
--- a/site/downloads/Dona-Fuego-Brand-Pro-Forma.xlsx
+++ b/site/downloads/Dona-Fuego-Brand-Pro-Forma.xlsx
@@ -21,15 +21,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="&quot;R&quot;#,##0;(&quot;R&quot;#,##0);-"/>
     <numFmt numFmtId="166" formatCode="0.0&quot;x&quot;"/>
-    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="168" formatCode="#,##0;-#,##0;-"/>
-    <numFmt numFmtId="169" formatCode="0.0x"/>
+    <numFmt numFmtId="167" formatCode="#,##0;-#,##0;-"/>
+    <numFmt numFmtId="168" formatCode="0.0x"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -66,8 +65,42 @@
       <color rgb="00008000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF0070C0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFEFE6CF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFEFE6CF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFEFE6CF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF2E2620"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF2E2620"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -77,6 +110,26 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4A6B47"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC13B2D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF7F1E1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8DCBE"/>
       </patternFill>
     </fill>
   </fills>
@@ -92,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -111,14 +164,38 @@
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="17" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="7" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="12" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="17" fontId="10" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="12" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="12" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -481,6 +558,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="FF4A6B47"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -493,11 +571,13 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>ASSUMPTIONS — Doña Fuego Brand Pro Forma (cans + bottles)</t>
         </is>
       </c>
+      <c r="B1" s="27" t="n"/>
+      <c r="C1" s="27" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -507,19 +587,21 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="28" t="inlineStr">
         <is>
           <t>Checkers listing</t>
         </is>
       </c>
+      <c r="B3" s="29" t="n"/>
+      <c r="C3" s="29" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="30" t="inlineStr">
         <is>
           <t>Stores in Checkers listing</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="31" t="n">
         <v>360</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -529,12 +611,12 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="30" t="inlineStr">
         <is>
           <t>SKUs in listing</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="32" t="n">
         <v>3</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -544,12 +626,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="30" t="inlineStr">
         <is>
           <t>Cases per store per SKU (initial fill)</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="32" t="n">
         <v>3</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -559,7 +641,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="33" t="inlineStr">
         <is>
           <t>Initial fill (cases)</t>
         </is>
@@ -570,7 +652,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="30" t="inlineStr">
         <is>
           <t>October restock (cases)</t>
         </is>
@@ -586,14 +668,16 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>Reorders</t>
         </is>
       </c>
+      <c r="B9" s="29" t="n"/>
+      <c r="C9" s="29" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="30" t="inlineStr">
         <is>
           <t>Steady-state store reorder (cases/month)</t>
         </is>
@@ -609,12 +693,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="30" t="inlineStr">
         <is>
           <t>Sixty60 uplift on steady-state reorders</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n">
+      <c r="B11" s="34" t="n">
         <v>0.1</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -624,7 +708,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="33" t="inlineStr">
         <is>
           <t>Steady-state incl. Sixty60 (cases/month)</t>
         </is>
@@ -635,12 +719,12 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="30" t="inlineStr">
         <is>
           <t>Wholesale price per case (R)</t>
         </is>
       </c>
-      <c r="B13" s="9" t="n">
+      <c r="B13" s="35" t="n">
         <v>847.04</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -650,31 +734,33 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="30" t="inlineStr">
         <is>
           <t>Payment terms</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="36" t="inlineStr">
         <is>
           <t>30 days from statement</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="28" t="inlineStr">
         <is>
           <t>Can COGS build (% of revenue)</t>
         </is>
       </c>
+      <c r="B15" s="29" t="n"/>
+      <c r="C15" s="29" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">  Tequila (supply agreement)</t>
         </is>
       </c>
-      <c r="B16" s="11" t="n">
+      <c r="B16" s="37" t="n">
         <v>0.18</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -684,47 +770,47 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">  Packaging (cans, printing, pallets)</t>
         </is>
       </c>
-      <c r="B17" s="11" t="n">
+      <c r="B17" s="37" t="n">
         <v>0.16</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">  Co-pack production</t>
         </is>
       </c>
-      <c r="B18" s="11" t="n">
+      <c r="B18" s="37" t="n">
         <v>0.12</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">  Distribution (FAL)</t>
         </is>
       </c>
-      <c r="B19" s="11" t="n">
+      <c r="B19" s="37" t="n">
         <v>0.04</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">  SARS Excise</t>
         </is>
       </c>
-      <c r="B20" s="11" t="n">
+      <c r="B20" s="37" t="n">
         <v>0.2</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="A21" s="33" t="inlineStr">
         <is>
           <t>Total can COGS ratio</t>
         </is>
@@ -735,19 +821,21 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" s="28" t="inlineStr">
         <is>
           <t>Operating costs — sales, operations &amp; distribution (monthly)</t>
         </is>
       </c>
+      <c r="B22" s="29" t="n"/>
+      <c r="C22" s="29" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="A23" s="30" t="inlineStr">
         <is>
           <t>Legal &amp; admin</t>
         </is>
       </c>
-      <c r="B23" s="9" t="n">
+      <c r="B23" s="35" t="n">
         <v>10000</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -757,7 +845,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="A24" s="30" t="inlineStr">
         <is>
           <t>Launch cost scaling vs project model</t>
         </is>
@@ -772,6 +860,7 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
@@ -779,13 +868,14 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="A28" s="30" t="inlineStr">
         <is>
           <t>Sales &amp; key accounts (1 FTE)</t>
         </is>
       </c>
-      <c r="B28" s="14" t="n">
+      <c r="B28" s="38" t="n">
         <v>40000</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -795,12 +885,12 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="A29" s="30" t="inlineStr">
         <is>
           <t>Operations &amp; merchandising coordinator</t>
         </is>
       </c>
-      <c r="B29" s="14" t="n">
+      <c r="B29" s="38" t="n">
         <v>18000</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -810,12 +900,12 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="A30" s="30" t="inlineStr">
         <is>
           <t>Trade marketing &amp; promotions</t>
         </is>
       </c>
-      <c r="B30" s="14" t="n">
+      <c r="B30" s="38" t="n">
         <v>25000</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -825,12 +915,12 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="A31" s="30" t="inlineStr">
         <is>
           <t>Warehousing &amp; insurance</t>
         </is>
       </c>
-      <c r="B31" s="14" t="n">
+      <c r="B31" s="38" t="n">
         <v>12000</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -840,7 +930,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+      <c r="A32" s="33" t="inlineStr">
         <is>
           <t>Steady-state opex total</t>
         </is>
@@ -858,6 +948,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="FF4A6B47"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -874,11 +965,17 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>FUEGO TEQUILA BOTTLES — historic sales &amp; projection</t>
         </is>
       </c>
+      <c r="B1" s="27" t="n"/>
+      <c r="C1" s="27" t="n"/>
+      <c r="D1" s="27" t="n"/>
+      <c r="E1" s="27" t="n"/>
+      <c r="F1" s="27" t="n"/>
+      <c r="G1" s="27" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -888,51 +985,51 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="39" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="39" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="39" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="39" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="39" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr"/>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="39" t="inlineStr">
         <is>
           <t>2027 (proj)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="30" t="inlineStr">
         <is>
           <t>January</t>
         </is>
       </c>
-      <c r="C4" s="9" t="n">
+      <c r="C4" s="35" t="n">
         <v>87354</v>
       </c>
-      <c r="D4" s="9" t="n">
+      <c r="D4" s="35" t="n">
         <v>107377.8</v>
       </c>
-      <c r="E4" s="9" t="n">
+      <c r="E4" s="35" t="n">
         <v>185865.3</v>
       </c>
       <c r="G4" s="15">
@@ -941,18 +1038,18 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="30" t="inlineStr">
         <is>
           <t>February</t>
         </is>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5" s="35" t="n">
         <v>7728</v>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D5" s="35" t="n">
         <v>46920</v>
       </c>
-      <c r="E5" s="9" t="n">
+      <c r="E5" s="35" t="n">
         <v>209857.2</v>
       </c>
       <c r="G5" s="15">
@@ -961,15 +1058,15 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="30" t="inlineStr">
         <is>
           <t>March</t>
         </is>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="D6" s="35" t="n">
         <v>126617.4</v>
       </c>
-      <c r="E6" s="9" t="n">
+      <c r="E6" s="35" t="n">
         <v>260918.59</v>
       </c>
       <c r="G6" s="15">
@@ -978,18 +1075,18 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="30" t="inlineStr">
         <is>
           <t>April</t>
         </is>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="35" t="n">
         <v>21931.51</v>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="35" t="n">
         <v>663918</v>
       </c>
-      <c r="E7" s="9" t="n">
+      <c r="E7" s="35" t="n">
         <v>470561.32</v>
       </c>
       <c r="G7" s="15">
@@ -998,18 +1095,18 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="30" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="C8" s="9" t="n">
+      <c r="C8" s="35" t="n">
         <v>1895.8</v>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D8" s="35" t="n">
         <v>168670.5</v>
       </c>
-      <c r="E8" s="9" t="n">
+      <c r="E8" s="35" t="n">
         <v>167687.8</v>
       </c>
       <c r="G8" s="15">
@@ -1018,18 +1115,18 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="30" t="inlineStr">
         <is>
           <t>June</t>
         </is>
       </c>
-      <c r="C9" s="9" t="n">
+      <c r="C9" s="35" t="n">
         <v>68533.21000000001</v>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="D9" s="35" t="n">
         <v>98574.11</v>
       </c>
-      <c r="E9" s="9" t="n">
+      <c r="E9" s="35" t="n">
         <v>60059.82</v>
       </c>
       <c r="G9" s="15">
@@ -1038,18 +1135,18 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="30" t="inlineStr">
         <is>
           <t>July</t>
         </is>
       </c>
-      <c r="C10" s="9" t="n">
+      <c r="C10" s="35" t="n">
         <v>36027.3</v>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D10" s="35" t="n">
         <v>266641.05</v>
       </c>
-      <c r="E10" s="9" t="n">
+      <c r="E10" s="35" t="n">
         <v>188654.34</v>
       </c>
       <c r="G10" s="15">
@@ -1058,15 +1155,15 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="30" t="inlineStr">
         <is>
           <t>August</t>
         </is>
       </c>
-      <c r="C11" s="9" t="n">
+      <c r="C11" s="35" t="n">
         <v>5796</v>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D11" s="35" t="n">
         <v>44441.56</v>
       </c>
       <c r="E11" s="15">
@@ -1079,18 +1176,18 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="30" t="inlineStr">
         <is>
           <t>September</t>
         </is>
       </c>
-      <c r="B12" s="9" t="n">
+      <c r="B12" s="35" t="n">
         <v>1334</v>
       </c>
-      <c r="C12" s="9" t="n">
+      <c r="C12" s="35" t="n">
         <v>46252.59</v>
       </c>
-      <c r="D12" s="9" t="n">
+      <c r="D12" s="35" t="n">
         <v>65847.11</v>
       </c>
       <c r="E12" s="15">
@@ -1103,18 +1200,18 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="30" t="inlineStr">
         <is>
           <t>October</t>
         </is>
       </c>
-      <c r="B13" s="9" t="n">
+      <c r="B13" s="35" t="n">
         <v>2894</v>
       </c>
-      <c r="C13" s="9" t="n">
+      <c r="C13" s="35" t="n">
         <v>530949.8100000001</v>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="D13" s="35" t="n">
         <v>63268.38</v>
       </c>
       <c r="E13" s="15">
@@ -1127,15 +1224,15 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="30" t="inlineStr">
         <is>
           <t>November</t>
         </is>
       </c>
-      <c r="C14" s="9" t="n">
+      <c r="C14" s="35" t="n">
         <v>81964.75</v>
       </c>
-      <c r="D14" s="9" t="n">
+      <c r="D14" s="35" t="n">
         <v>257848.55</v>
       </c>
       <c r="E14" s="15">
@@ -1148,18 +1245,18 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="30" t="inlineStr">
         <is>
           <t>December</t>
         </is>
       </c>
-      <c r="B15" s="9" t="n">
+      <c r="B15" s="35" t="n">
         <v>21919</v>
       </c>
-      <c r="C15" s="9" t="n">
+      <c r="C15" s="35" t="n">
         <v>138333.09</v>
       </c>
-      <c r="D15" s="9" t="n">
+      <c r="D15" s="35" t="n">
         <v>35332.6</v>
       </c>
       <c r="E15" s="15">
@@ -1172,41 +1269,44 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="33" t="inlineStr">
         <is>
           <t>Annual total</t>
         </is>
       </c>
-      <c r="B16" s="16">
+      <c r="B16" s="40">
         <f>SUM(B4:B15)</f>
         <v/>
       </c>
-      <c r="C16" s="16">
+      <c r="C16" s="40">
         <f>SUM(C4:C15)</f>
         <v/>
       </c>
-      <c r="D16" s="16">
+      <c r="D16" s="40">
         <f>SUM(D4:D15)</f>
         <v/>
       </c>
-      <c r="E16" s="16">
+      <c r="E16" s="40">
         <f>SUM(E4:E15)</f>
         <v/>
       </c>
-      <c r="G16" s="16">
+      <c r="G16" s="40">
         <f>SUM(G4:G15)</f>
         <v/>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="28" t="inlineStr">
         <is>
           <t>Projection assumptions</t>
         </is>
       </c>
+      <c r="B18" s="29" t="n"/>
+      <c r="C18" s="29" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="30" t="inlineStr">
         <is>
           <t>YoY growth (Jan-Jul 26 vs Jan-Jul 25)</t>
         </is>
@@ -1222,12 +1322,12 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="30" t="inlineStr">
         <is>
           <t>2027 growth on 2026</t>
         </is>
       </c>
-      <c r="B20" s="8" t="n">
+      <c r="B20" s="34" t="n">
         <v>0.05</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1237,7 +1337,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="A21" s="30" t="inlineStr">
         <is>
           <t>2027 total</t>
         </is>
@@ -1248,12 +1348,12 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="A22" s="30" t="inlineStr">
         <is>
           <t>Bottle gross margin %</t>
         </is>
       </c>
-      <c r="B22" s="8" t="n">
+      <c r="B22" s="34" t="n">
         <v>0.3</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1262,6 +1362,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
@@ -1277,6 +1378,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="FF4A6B47"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -1306,167 +1408,188 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>P&amp;L (ACCRUAL) — Doña Fuego cans + Fuego Tequila bottles</t>
         </is>
       </c>
-    </row>
+      <c r="B1" s="27" t="n"/>
+      <c r="C1" s="27" t="n"/>
+      <c r="D1" s="27" t="n"/>
+      <c r="E1" s="27" t="n"/>
+      <c r="F1" s="27" t="n"/>
+      <c r="G1" s="27" t="n"/>
+      <c r="H1" s="27" t="n"/>
+      <c r="I1" s="27" t="n"/>
+      <c r="J1" s="27" t="n"/>
+      <c r="K1" s="27" t="n"/>
+      <c r="L1" s="27" t="n"/>
+      <c r="M1" s="27" t="n"/>
+      <c r="N1" s="27" t="n"/>
+      <c r="O1" s="27" t="n"/>
+      <c r="P1" s="27" t="n"/>
+      <c r="Q1" s="27" t="n"/>
+      <c r="R1" s="27" t="n"/>
+      <c r="S1" s="27" t="n"/>
+      <c r="T1" s="27" t="n"/>
+      <c r="U1" s="27" t="n"/>
+    </row>
+    <row r="2"/>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="39" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B3" s="17" t="n">
+      <c r="B3" s="41" t="n">
         <v>46174</v>
       </c>
-      <c r="C3" s="17" t="n">
+      <c r="C3" s="41" t="n">
         <v>46204</v>
       </c>
-      <c r="D3" s="17" t="n">
+      <c r="D3" s="41" t="n">
         <v>46235</v>
       </c>
-      <c r="E3" s="17" t="n">
+      <c r="E3" s="41" t="n">
         <v>46266</v>
       </c>
-      <c r="F3" s="17" t="n">
+      <c r="F3" s="41" t="n">
         <v>46296</v>
       </c>
-      <c r="G3" s="17" t="n">
+      <c r="G3" s="41" t="n">
         <v>46327</v>
       </c>
-      <c r="H3" s="17" t="n">
+      <c r="H3" s="41" t="n">
         <v>46357</v>
       </c>
-      <c r="I3" s="17" t="n">
+      <c r="I3" s="41" t="n">
         <v>46388</v>
       </c>
-      <c r="J3" s="17" t="n">
+      <c r="J3" s="41" t="n">
         <v>46419</v>
       </c>
-      <c r="K3" s="17" t="n">
+      <c r="K3" s="41" t="n">
         <v>46447</v>
       </c>
-      <c r="L3" s="17" t="n">
+      <c r="L3" s="41" t="n">
         <v>46478</v>
       </c>
-      <c r="M3" s="17" t="n">
+      <c r="M3" s="41" t="n">
         <v>46508</v>
       </c>
-      <c r="N3" s="17" t="n">
+      <c r="N3" s="41" t="n">
         <v>46539</v>
       </c>
-      <c r="O3" s="17" t="n">
+      <c r="O3" s="41" t="n">
         <v>46569</v>
       </c>
-      <c r="P3" s="17" t="n">
+      <c r="P3" s="41" t="n">
         <v>46600</v>
       </c>
-      <c r="Q3" s="17" t="n">
+      <c r="Q3" s="41" t="n">
         <v>46631</v>
       </c>
-      <c r="R3" s="17" t="n">
+      <c r="R3" s="41" t="n">
         <v>46661</v>
       </c>
-      <c r="S3" s="17" t="n">
+      <c r="S3" s="41" t="n">
         <v>46692</v>
       </c>
-      <c r="T3" s="17" t="n">
+      <c r="T3" s="41" t="n">
         <v>46722</v>
       </c>
-      <c r="U3" s="3" t="inlineStr">
+      <c r="U3" s="39" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="30" t="inlineStr">
         <is>
           <t>Cases delivered (cans)</t>
         </is>
       </c>
-      <c r="B4" s="18" t="n">
+      <c r="B4" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="C4" s="18" t="n">
+      <c r="C4" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="19">
+      <c r="D4" s="43">
         <f>Assumptions!B7</f>
         <v/>
       </c>
-      <c r="E4" s="18" t="n">
+      <c r="E4" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="19">
+      <c r="F4" s="43">
         <f>Assumptions!B8</f>
         <v/>
       </c>
-      <c r="G4" s="19">
+      <c r="G4" s="43">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="H4" s="19">
+      <c r="H4" s="43">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="I4" s="19">
+      <c r="I4" s="43">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="J4" s="19">
+      <c r="J4" s="43">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="K4" s="19">
+      <c r="K4" s="43">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="L4" s="19">
+      <c r="L4" s="43">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="M4" s="19">
+      <c r="M4" s="43">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="N4" s="19">
+      <c r="N4" s="43">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="O4" s="19">
+      <c r="O4" s="43">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="P4" s="19">
+      <c r="P4" s="43">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="Q4" s="19">
+      <c r="Q4" s="43">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="R4" s="19">
+      <c r="R4" s="43">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="S4" s="19">
+      <c r="S4" s="43">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="T4" s="19">
+      <c r="T4" s="43">
         <f>Assumptions!B12</f>
         <v/>
       </c>
-      <c r="U4" s="20">
+      <c r="U4" s="44">
         <f>SUM(B4:T4)</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="30" t="inlineStr">
         <is>
           <t>Can revenue</t>
         </is>
@@ -1547,13 +1670,13 @@
         <f>T4*Assumptions!$B$13</f>
         <v/>
       </c>
-      <c r="U5" s="16">
+      <c r="U5" s="45">
         <f>SUM(B5:T5)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="30" t="inlineStr">
         <is>
           <t>Bottle revenue</t>
         </is>
@@ -1634,13 +1757,13 @@
         <f>Bottles!G15</f>
         <v/>
       </c>
-      <c r="U6" s="16">
+      <c r="U6" s="45">
         <f>SUM(B6:T6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="33" t="inlineStr">
         <is>
           <t>Total revenue</t>
         </is>
@@ -1721,13 +1844,13 @@
         <f>T5+T6</f>
         <v/>
       </c>
-      <c r="U7" s="16">
+      <c r="U7" s="45">
         <f>SUM(B7:T7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="30" t="inlineStr">
         <is>
           <t>Can COGS</t>
         </is>
@@ -1808,13 +1931,13 @@
         <f>-T5*Assumptions!$B$21</f>
         <v/>
       </c>
-      <c r="U8" s="16">
+      <c r="U8" s="45">
         <f>SUM(B8:T8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="30" t="inlineStr">
         <is>
           <t>Bottle COGS</t>
         </is>
@@ -1895,13 +2018,13 @@
         <f>-T6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="U9" s="16">
+      <c r="U9" s="45">
         <f>SUM(B9:T9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="33" t="inlineStr">
         <is>
           <t>Gross margin</t>
         </is>
@@ -1982,13 +2105,13 @@
         <f>T7+T8+T9</f>
         <v/>
       </c>
-      <c r="U10" s="16">
+      <c r="U10" s="45">
         <f>SUM(B10:T10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="30" t="inlineStr">
         <is>
           <t>Gross margin %</t>
         </is>
@@ -2069,15 +2192,15 @@
         <f>IF(T7=0,0,T10/T7)</f>
         <v/>
       </c>
-      <c r="U11" s="22">
+      <c r="U11" s="46">
         <f>U10/U7</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Opex (legal &amp; admin)</t>
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>Opex (sales, ops &amp; distribution)</t>
         </is>
       </c>
       <c r="B12" s="15">
@@ -2156,13 +2279,13 @@
         <f>-(Assumptions!$B$23+IF(T$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(T$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
         <v/>
       </c>
-      <c r="U12" s="16">
+      <c r="U12" s="45">
         <f>SUM(B12:T12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="33" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
@@ -2243,13 +2366,13 @@
         <f>T10+T12</f>
         <v/>
       </c>
-      <c r="U13" s="16">
+      <c r="U13" s="45">
         <f>SUM(B13:T13)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="30" t="inlineStr">
         <is>
           <t>EBITDA %</t>
         </is>
@@ -2330,7 +2453,7 @@
         <f>IF(T7=0,0,T13/T7)</f>
         <v/>
       </c>
-      <c r="U14" s="22">
+      <c r="U14" s="46">
         <f>U13/U7</f>
         <v/>
       </c>
@@ -2343,6 +2466,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="FF4A6B47"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2372,83 +2496,104 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>CASHFLOW (CASH BASIS) — brand entity</t>
         </is>
       </c>
-    </row>
+      <c r="B1" s="27" t="n"/>
+      <c r="C1" s="27" t="n"/>
+      <c r="D1" s="27" t="n"/>
+      <c r="E1" s="27" t="n"/>
+      <c r="F1" s="27" t="n"/>
+      <c r="G1" s="27" t="n"/>
+      <c r="H1" s="27" t="n"/>
+      <c r="I1" s="27" t="n"/>
+      <c r="J1" s="27" t="n"/>
+      <c r="K1" s="27" t="n"/>
+      <c r="L1" s="27" t="n"/>
+      <c r="M1" s="27" t="n"/>
+      <c r="N1" s="27" t="n"/>
+      <c r="O1" s="27" t="n"/>
+      <c r="P1" s="27" t="n"/>
+      <c r="Q1" s="27" t="n"/>
+      <c r="R1" s="27" t="n"/>
+      <c r="S1" s="27" t="n"/>
+      <c r="T1" s="27" t="n"/>
+      <c r="U1" s="27" t="n"/>
+    </row>
+    <row r="2"/>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="39" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B3" s="17" t="n">
+      <c r="B3" s="41" t="n">
         <v>46174</v>
       </c>
-      <c r="C3" s="17" t="n">
+      <c r="C3" s="41" t="n">
         <v>46204</v>
       </c>
-      <c r="D3" s="17" t="n">
+      <c r="D3" s="41" t="n">
         <v>46235</v>
       </c>
-      <c r="E3" s="17" t="n">
+      <c r="E3" s="41" t="n">
         <v>46266</v>
       </c>
-      <c r="F3" s="17" t="n">
+      <c r="F3" s="41" t="n">
         <v>46296</v>
       </c>
-      <c r="G3" s="17" t="n">
+      <c r="G3" s="41" t="n">
         <v>46327</v>
       </c>
-      <c r="H3" s="17" t="n">
+      <c r="H3" s="41" t="n">
         <v>46357</v>
       </c>
-      <c r="I3" s="17" t="n">
+      <c r="I3" s="41" t="n">
         <v>46388</v>
       </c>
-      <c r="J3" s="17" t="n">
+      <c r="J3" s="41" t="n">
         <v>46419</v>
       </c>
-      <c r="K3" s="17" t="n">
+      <c r="K3" s="41" t="n">
         <v>46447</v>
       </c>
-      <c r="L3" s="17" t="n">
+      <c r="L3" s="41" t="n">
         <v>46478</v>
       </c>
-      <c r="M3" s="17" t="n">
+      <c r="M3" s="41" t="n">
         <v>46508</v>
       </c>
-      <c r="N3" s="17" t="n">
+      <c r="N3" s="41" t="n">
         <v>46539</v>
       </c>
-      <c r="O3" s="17" t="n">
+      <c r="O3" s="41" t="n">
         <v>46569</v>
       </c>
-      <c r="P3" s="17" t="n">
+      <c r="P3" s="41" t="n">
         <v>46600</v>
       </c>
-      <c r="Q3" s="17" t="n">
+      <c r="Q3" s="41" t="n">
         <v>46631</v>
       </c>
-      <c r="R3" s="17" t="n">
+      <c r="R3" s="41" t="n">
         <v>46661</v>
       </c>
-      <c r="S3" s="17" t="n">
+      <c r="S3" s="41" t="n">
         <v>46692</v>
       </c>
-      <c r="T3" s="17" t="n">
+      <c r="T3" s="41" t="n">
         <v>46722</v>
       </c>
-      <c r="U3" s="3" t="inlineStr">
+      <c r="U3" s="39" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="30" t="inlineStr">
         <is>
           <t>Can receipts (revenue +30 days)</t>
         </is>
@@ -2528,13 +2673,13 @@
         <f>'P&amp;L'!S5</f>
         <v/>
       </c>
-      <c r="U4" s="16">
+      <c r="U4" s="45">
         <f>SUM(B4:T4)</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">  Bron Pro (design/brand)</t>
         </is>
@@ -2547,13 +2692,13 @@
         <f>-243800*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="U5" s="15">
+      <c r="U5" s="45">
         <f>SUM(B5:T5)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">  Sullwaldt printing</t>
         </is>
@@ -2566,13 +2711,13 @@
         <f>-72400*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="U6" s="15">
+      <c r="U6" s="45">
         <f>SUM(B6:T6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">  Tiny Keg cans</t>
         </is>
@@ -2585,13 +2730,13 @@
         <f>-319000*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="U7" s="15">
+      <c r="U7" s="45">
         <f>SUM(B7:T7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">  Chep pallets</t>
         </is>
@@ -2600,13 +2745,13 @@
         <f>-14375*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="U8" s="15">
+      <c r="U8" s="45">
         <f>SUM(B8:T8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">  FAL distribution</t>
         </is>
@@ -2619,13 +2764,13 @@
         <f>-28000*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="U9" s="15">
+      <c r="U9" s="45">
         <f>SUM(B9:T9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">  Tiny Keg production</t>
         </is>
@@ -2638,13 +2783,13 @@
         <f>-293250*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="U10" s="15">
+      <c r="U10" s="45">
         <f>SUM(B10:T10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">  SARS excise (launch)</t>
         </is>
@@ -2657,13 +2802,13 @@
         <f>-495571*Assumptions!$B$24</f>
         <v/>
       </c>
-      <c r="U11" s="15">
+      <c r="U11" s="45">
         <f>SUM(B11:T11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">  Opex (sales, ops, marketing, admin — paid monthly)</t>
         </is>
@@ -2744,13 +2889,13 @@
         <f>'P&amp;L'!T12</f>
         <v/>
       </c>
-      <c r="U12" s="15">
+      <c r="U12" s="45">
         <f>SUM(B12:T12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">  Bottles net contribution (GM, cash in month)</t>
         </is>
@@ -2831,13 +2976,13 @@
         <f>'P&amp;L'!T6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="U13" s="15">
+      <c r="U13" s="45">
         <f>SUM(B13:T13)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">  2027 recurring can COGS</t>
         </is>
@@ -2890,13 +3035,13 @@
         <f>-'P&amp;L'!T5*Assumptions!$B$21</f>
         <v/>
       </c>
-      <c r="U14" s="15">
+      <c r="U14" s="45">
         <f>SUM(B14:T14)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="33" t="inlineStr">
         <is>
           <t>Net monthly cashflow</t>
         </is>
@@ -2977,13 +3122,13 @@
         <f>SUM(T4:T14)</f>
         <v/>
       </c>
-      <c r="U15" s="16">
+      <c r="U15" s="45">
         <f>SUM(B15:T15)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="33" t="inlineStr">
         <is>
           <t>Cumulative cash position</t>
         </is>
@@ -3065,10 +3210,11 @@
         <v/>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Note: 2026 launch costs are the project model's quoted cash costs, scaled by the store factor (Assumptions!B24); legal retainer unscaled.</t>
+          <t>Note: 2026 launch costs are the project model's quoted cash costs, scaled by the store factor (Assumptions!B24).</t>
         </is>
       </c>
     </row>
@@ -3087,6 +3233,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="FF4A6B47"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -3101,21 +3248,29 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>VALUATION — Doña Fuego brand entity (cans + bottles)</t>
         </is>
       </c>
-    </row>
+      <c r="B1" s="27" t="n"/>
+      <c r="C1" s="27" t="n"/>
+      <c r="D1" s="27" t="n"/>
+      <c r="E1" s="27" t="n"/>
+    </row>
+    <row r="2"/>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="28" t="inlineStr">
         <is>
           <t>Key metrics (linked to P&amp;L)</t>
         </is>
       </c>
+      <c r="B3" s="29" t="n"/>
+      <c r="C3" s="29" t="n"/>
+      <c r="D3" s="29" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="30" t="inlineStr">
         <is>
           <t>2026 (Jun–Dec) revenue</t>
         </is>
@@ -3126,7 +3281,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="30" t="inlineStr">
         <is>
           <t>2026 (Jun–Dec) EBITDA</t>
         </is>
@@ -3137,7 +3292,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="30" t="inlineStr">
         <is>
           <t>2027 revenue</t>
         </is>
@@ -3148,7 +3303,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="30" t="inlineStr">
         <is>
           <t>2027 EBITDA</t>
         </is>
@@ -3158,46 +3313,47 @@
         <v/>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>Method 1: EV/EBITDA on 2027 EBITDA</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="29" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="29" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="29" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="30" t="inlineStr">
         <is>
           <t>Multiple</t>
         </is>
       </c>
-      <c r="B10" s="23" t="n">
+      <c r="B10" s="47" t="n">
         <v>6</v>
       </c>
-      <c r="C10" s="23" t="n">
+      <c r="C10" s="47" t="n">
         <v>9</v>
       </c>
-      <c r="D10" s="23" t="n">
+      <c r="D10" s="47" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="30" t="inlineStr">
         <is>
           <t>Enterprise value</t>
         </is>
@@ -3215,31 +3371,35 @@
         <v/>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="28" t="inlineStr">
         <is>
           <t>Method 2: EV/Revenue on 2027 revenue</t>
         </is>
       </c>
+      <c r="B13" s="29" t="n"/>
+      <c r="C13" s="29" t="n"/>
+      <c r="D13" s="29" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="30" t="inlineStr">
         <is>
           <t>Multiple</t>
         </is>
       </c>
-      <c r="B14" s="23" t="n">
+      <c r="B14" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="C14" s="23" t="n">
+      <c r="C14" s="47" t="n">
         <v>1.5</v>
       </c>
-      <c r="D14" s="23" t="n">
+      <c r="D14" s="47" t="n">
         <v>2.5</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="30" t="inlineStr">
         <is>
           <t>Enterprise value</t>
         </is>
@@ -3257,47 +3417,51 @@
         <v/>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="28" t="inlineStr">
         <is>
           <t>Method 3: simplified DCF (EBITDA as cash proxy)</t>
         </is>
       </c>
+      <c r="B17" s="29" t="n"/>
+      <c r="C17" s="29" t="n"/>
+      <c r="D17" s="29" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="30" t="inlineStr">
         <is>
           <t>WACC</t>
         </is>
       </c>
-      <c r="B18" s="11" t="n">
+      <c r="B18" s="37" t="n">
         <v>0.22</v>
       </c>
-      <c r="C18" s="11" t="n">
+      <c r="C18" s="37" t="n">
         <v>0.18</v>
       </c>
-      <c r="D18" s="11" t="n">
+      <c r="D18" s="37" t="n">
         <v>0.15</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="30" t="inlineStr">
         <is>
           <t>Exit multiple (2027 EBITDA)</t>
         </is>
       </c>
-      <c r="B19" s="23" t="n">
+      <c r="B19" s="47" t="n">
         <v>6</v>
       </c>
-      <c r="C19" s="23" t="n">
+      <c r="C19" s="47" t="n">
         <v>8</v>
       </c>
-      <c r="D19" s="23" t="n">
+      <c r="D19" s="47" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="30" t="inlineStr">
         <is>
           <t>Enterprise value (DCF)</t>
         </is>
@@ -3315,40 +3479,45 @@
         <v/>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" s="33" t="inlineStr">
         <is>
           <t>Blended enterprise value (avg of methods)</t>
         </is>
       </c>
-      <c r="B22" s="16">
+      <c r="B22" s="40">
         <f>AVERAGE(B11,B15,B20)</f>
         <v/>
       </c>
-      <c r="C22" s="16">
+      <c r="C22" s="40">
         <f>AVERAGE(C11,C15,C20)</f>
         <v/>
       </c>
-      <c r="D22" s="16">
+      <c r="D22" s="40">
         <f>AVERAGE(D11,D15,D20)</f>
         <v/>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" s="39" t="inlineStr">
         <is>
           <t>Valuation guide for the raise</t>
         </is>
       </c>
-      <c r="B24" s="14" t="n">
+      <c r="B24" s="48" t="n">
         <v>15000000</v>
       </c>
+      <c r="C24" s="27" t="n"/>
+      <c r="D24" s="27" t="n"/>
       <c r="E24" s="2" t="inlineStr">
         <is>
           <t>With bottles modelled off three years of actuals, the ~R15m guide equals the blended LOW case; better-than-flat reorders, new retailers and export remain outside the model.</t>
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
@@ -3364,6 +3533,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="FF4A6B47"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -3375,14 +3545,16 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>SUMMARY — Doña Fuego Brand Pro Forma</t>
         </is>
       </c>
-    </row>
+      <c r="B1" s="27" t="n"/>
+    </row>
+    <row r="2"/>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="49" t="inlineStr">
         <is>
           <t>Checkers listing</t>
         </is>
@@ -3393,7 +3565,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="49" t="inlineStr">
         <is>
           <t>Opening order (initial fill revenue)</t>
         </is>
@@ -3404,7 +3576,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="49" t="inlineStr">
         <is>
           <t>Bottle revenue (Jun 26 – Dec 27)</t>
         </is>
@@ -3415,29 +3587,29 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="39" t="inlineStr">
         <is>
           <t>Total revenue, cans + bottles (Jun 26 – Dec 27)</t>
         </is>
       </c>
-      <c r="B6" s="21">
+      <c r="B6" s="45">
         <f>'P&amp;L'!U7</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="39" t="inlineStr">
         <is>
           <t>Total EBITDA (Jun 26 – Dec 27)</t>
         </is>
       </c>
-      <c r="B7" s="21">
+      <c r="B7" s="45">
         <f>'P&amp;L'!U13</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="49" t="inlineStr">
         <is>
           <t>EBITDA margin</t>
         </is>
@@ -3448,18 +3620,18 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>Peak funding need</t>
         </is>
       </c>
-      <c r="B9" s="21">
+      <c r="B9" s="45">
         <f>MIN(Cashflow!B16:T16)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="49" t="inlineStr">
         <is>
           <t>Ending cash (Dec 27)</t>
         </is>
@@ -3470,7 +3642,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="49" t="inlineStr">
         <is>
           <t>Blended valuation — low</t>
         </is>
@@ -3481,7 +3653,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="49" t="inlineStr">
         <is>
           <t>Blended valuation — base</t>
         </is>
@@ -3492,7 +3664,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="49" t="inlineStr">
         <is>
           <t>Blended valuation — high</t>
         </is>
@@ -3503,16 +3675,17 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="39" t="inlineStr">
         <is>
           <t>Valuation guide</t>
         </is>
       </c>
-      <c r="B14" s="21">
+      <c r="B14" s="45">
         <f>Valuation!B24</f>
         <v/>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Brand marketing line, seasonal can volumes, 360-store basis throughout
- Opex gains R25k/month brand marketing (steady state R130k/month)
- Can sales seasonally shaped: 70% of annual volume Oct-Mar, 30% Apr-Sep,
  same annual total; workbook inputs for summer share and monthly rates
- Workbook restated on the 360-store listing directly (restock 1,260
  cases, replenishment 720/month, launch costs per supplier quotes)
- Results: revenue R16.61m, EBITDA R2.69m (16.2%), peak funding R1.66m,
  end cash R1.99m; blended valuation R9.4m/R13.5m/R19.3m with the ~R15m
  guide between base and high, premium carried by unmodelled upside
- Charts, tables, stats and FAQs updated; stale valuation note corrected

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hyws6xeXfxtGdqZV2paNDe
</commit_message>
<xml_diff>
--- a/site/downloads/Dona-Fuego-Brand-Pro-Forma.xlsx
+++ b/site/downloads/Dona-Fuego-Brand-Pro-Forma.xlsx
@@ -21,12 +21,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="&quot;R&quot;#,##0;(&quot;R&quot;#,##0);-"/>
-    <numFmt numFmtId="166" formatCode="0.0&quot;x&quot;"/>
-    <numFmt numFmtId="167" formatCode="#,##0;-#,##0;-"/>
-    <numFmt numFmtId="168" formatCode="0.0x"/>
+    <numFmt numFmtId="166" formatCode="#,##0;-#,##0;-"/>
+    <numFmt numFmtId="167" formatCode="0.0x"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -145,7 +144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -159,17 +158,16 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="17" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -188,12 +186,12 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="12" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="17" fontId="10" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="12" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="12" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="12" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -562,7 +560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -571,13 +569,13 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>ASSUMPTIONS — Doña Fuego Brand Pro Forma (cans + bottles)</t>
         </is>
       </c>
-      <c r="B1" s="27" t="n"/>
-      <c r="C1" s="27" t="n"/>
+      <c r="B1" s="26" t="n"/>
+      <c r="C1" s="26" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -587,21 +585,21 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="inlineStr">
+      <c r="A3" s="27" t="inlineStr">
         <is>
           <t>Checkers listing</t>
         </is>
       </c>
-      <c r="B3" s="29" t="n"/>
-      <c r="C3" s="29" t="n"/>
+      <c r="B3" s="28" t="n"/>
+      <c r="C3" s="28" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="30" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>Stores in Checkers listing</t>
         </is>
       </c>
-      <c r="B4" s="31" t="n">
+      <c r="B4" s="30" t="n">
         <v>360</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -611,12 +609,12 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>SKUs in listing</t>
         </is>
       </c>
-      <c r="B5" s="32" t="n">
+      <c r="B5" s="31" t="n">
         <v>3</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -626,22 +624,22 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="30" t="inlineStr">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>Cases per store per SKU (initial fill)</t>
         </is>
       </c>
-      <c r="B6" s="32" t="n">
+      <c r="B6" s="31" t="n">
         <v>3</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Per project model</t>
+          <t>Per Checkers opening order</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="33" t="inlineStr">
+      <c r="A7" s="32" t="inlineStr">
         <is>
           <t>Initial fill (cases)</t>
         </is>
@@ -652,65 +650,63 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="30" t="inlineStr">
+      <c r="A8" s="29" t="inlineStr">
         <is>
           <t>October restock (cases)</t>
         </is>
       </c>
-      <c r="B8" s="7">
-        <f>1050*B4/300</f>
-        <v/>
+      <c r="B8" s="31" t="n">
+        <v>1260</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Scaled from 1,050 cases at 300 stores (project model)</t>
+          <t>Restock order ahead of the summer season</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="28" t="inlineStr">
-        <is>
-          <t>Reorders</t>
-        </is>
-      </c>
-      <c r="B9" s="29" t="n"/>
-      <c r="C9" s="29" t="n"/>
+      <c r="A9" s="27" t="inlineStr">
+        <is>
+          <t>Reorders &amp; seasonality</t>
+        </is>
+      </c>
+      <c r="B9" s="28" t="n"/>
+      <c r="C9" s="28" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="30" t="inlineStr">
-        <is>
-          <t>Steady-state store reorder (cases/month)</t>
-        </is>
-      </c>
-      <c r="B10" s="7">
-        <f>600*B4/300</f>
-        <v/>
+      <c r="A10" s="29" t="inlineStr">
+        <is>
+          <t>Store replenishment (cases/month, annual average)</t>
+        </is>
+      </c>
+      <c r="B10" s="31" t="n">
+        <v>720</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Scaled from 600 cases/month at 300 stores (project model)</t>
+          <t>Baseline replenishment across the 360-store listing</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="30" t="inlineStr">
-        <is>
-          <t>Sixty60 uplift on steady-state reorders</t>
-        </is>
-      </c>
-      <c r="B11" s="34" t="n">
+      <c r="A11" s="29" t="inlineStr">
+        <is>
+          <t>Sixty60 uplift on replenishment</t>
+        </is>
+      </c>
+      <c r="B11" s="33" t="n">
         <v>0.1</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>MANAGEMENT ESTIMATE (conservative): on-demand delivery adds 10% to monthly reorders</t>
+          <t>MANAGEMENT ESTIMATE (conservative): on-demand delivery adds 10%</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="33" t="inlineStr">
-        <is>
-          <t>Steady-state incl. Sixty60 (cases/month)</t>
+      <c r="A12" s="32" t="inlineStr">
+        <is>
+          <t>Average incl. Sixty60 (cases/month)</t>
         </is>
       </c>
       <c r="B12" s="7">
@@ -719,225 +715,260 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="30" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>Summer share of annual can volume</t>
+        </is>
+      </c>
+      <c r="B13" s="33" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Summer = Oct-Mar (incl. festive season); winter = Apr-Sep</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="32" t="inlineStr">
+        <is>
+          <t>Summer months (cases/month)</t>
+        </is>
+      </c>
+      <c r="B14" s="7">
+        <f>ROUND(B12*12*B13/6,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="32" t="inlineStr">
+        <is>
+          <t>Winter months (cases/month)</t>
+        </is>
+      </c>
+      <c r="B15" s="7">
+        <f>ROUND(B12*12*(1-B13)/6,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>Wholesale price per case (R)</t>
         </is>
       </c>
-      <c r="B13" s="35" t="n">
+      <c r="B16" s="34" t="n">
         <v>847.04</v>
       </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Per project model (R169 4-pack / R49 unit retail)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="30" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>R169 4-pack / R49 unit retail</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="29" t="inlineStr">
         <is>
           <t>Payment terms</t>
         </is>
       </c>
-      <c r="B14" s="36" t="inlineStr">
+      <c r="B17" s="35" t="inlineStr">
         <is>
           <t>30 days from statement</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="28" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="27" t="inlineStr">
         <is>
           <t>Can COGS build (% of revenue)</t>
         </is>
       </c>
-      <c r="B15" s="29" t="n"/>
-      <c r="C15" s="29" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="30" t="inlineStr">
+      <c r="B18" s="28" t="n"/>
+      <c r="C18" s="28" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  Tequila (supply agreement)</t>
         </is>
       </c>
-      <c r="B16" s="37" t="n">
+      <c r="B19" s="36" t="n">
         <v>0.18</v>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Bulk tequila from Doña Distillery under special supply agreement</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="30" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Bulk tequila from Dona Distillery under special supply agreement</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  Packaging (cans, printing, pallets)</t>
         </is>
       </c>
-      <c r="B17" s="37" t="n">
+      <c r="B20" s="36" t="n">
         <v>0.16</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="30" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  Co-pack production</t>
         </is>
       </c>
-      <c r="B18" s="37" t="n">
+      <c r="B21" s="36" t="n">
         <v>0.12</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="30" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  Distribution (FAL)</t>
         </is>
       </c>
-      <c r="B19" s="37" t="n">
+      <c r="B22" s="36" t="n">
         <v>0.04</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="30" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  SARS Excise</t>
         </is>
       </c>
-      <c r="B20" s="37" t="n">
+      <c r="B23" s="36" t="n">
         <v>0.2</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="33" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="32" t="inlineStr">
         <is>
           <t>Total can COGS ratio</t>
         </is>
       </c>
-      <c r="B21" s="12">
-        <f>SUM(B16:B20)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="28" t="inlineStr">
+      <c r="B24" s="12">
+        <f>SUM(B19:B23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="27" t="inlineStr">
         <is>
           <t>Operating costs — sales, operations &amp; distribution (monthly)</t>
         </is>
       </c>
-      <c r="B22" s="29" t="n"/>
-      <c r="C22" s="29" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="30" t="inlineStr">
+      <c r="B25" s="28" t="n"/>
+      <c r="C25" s="28" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="29" t="inlineStr">
         <is>
           <t>Legal &amp; admin</t>
         </is>
       </c>
-      <c r="B23" s="35" t="n">
+      <c r="B26" s="34" t="n">
         <v>10000</v>
       </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Per project model; from June 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="30" t="inlineStr">
-        <is>
-          <t>Launch cost scaling vs project model</t>
-        </is>
-      </c>
-      <c r="B24" s="13">
-        <f>B4/300</f>
-        <v/>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Applied to 2026 launch cash costs quoted at 300-store scale</t>
-        </is>
-      </c>
-    </row>
-    <row r="25"/>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>From June 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="29" t="inlineStr">
+        <is>
+          <t>Sales &amp; key accounts (1 FTE)</t>
+        </is>
+      </c>
+      <c r="B27" s="37" t="n">
+        <v>40000</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>MANAGEMENT ESTIMATE, from July 2026 — supports founder-led sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="29" t="inlineStr">
+        <is>
+          <t>Operations &amp; merchandising coordinator</t>
+        </is>
+      </c>
+      <c r="B28" s="37" t="n">
+        <v>18000</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>MANAGEMENT ESTIMATE, from July 2026 — shared resource with distillery</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="29" t="inlineStr">
+        <is>
+          <t>Trade marketing &amp; promotions</t>
+        </is>
+      </c>
+      <c r="B29" s="37" t="n">
+        <v>25000</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>MANAGEMENT ESTIMATE, from August 2026 — in-store support</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="29" t="inlineStr">
+        <is>
+          <t>Brand marketing</t>
+        </is>
+      </c>
+      <c r="B30" s="37" t="n">
+        <v>25000</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>MANAGEMENT ESTIMATE, from August 2026 — always-on consumer brand building</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="29" t="inlineStr">
+        <is>
+          <t>Warehousing &amp; insurance</t>
+        </is>
+      </c>
+      <c r="B31" s="37" t="n">
+        <v>12000</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>MANAGEMENT ESTIMATE, from August 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="32" t="inlineStr">
+        <is>
+          <t>Steady-state opex total</t>
+        </is>
+      </c>
+      <c r="B32" s="14">
+        <f>SUM(B26:B31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33"/>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>Legend: blue = input (edit these) · black = formula · green = link to another sheet · yellow = key assumptions to sense-check</t>
         </is>
-      </c>
-    </row>
-    <row r="27"/>
-    <row r="28">
-      <c r="A28" s="30" t="inlineStr">
-        <is>
-          <t>Sales &amp; key accounts (1 FTE)</t>
-        </is>
-      </c>
-      <c r="B28" s="38" t="n">
-        <v>40000</v>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>MANAGEMENT ESTIMATE, from July 2026 — supports founder-led sales</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="30" t="inlineStr">
-        <is>
-          <t>Operations &amp; merchandising coordinator</t>
-        </is>
-      </c>
-      <c r="B29" s="38" t="n">
-        <v>18000</v>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>MANAGEMENT ESTIMATE, from July 2026 — shared resource with distillery</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="30" t="inlineStr">
-        <is>
-          <t>Trade marketing &amp; promotions</t>
-        </is>
-      </c>
-      <c r="B30" s="38" t="n">
-        <v>25000</v>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>MANAGEMENT ESTIMATE, from August 2026 — always-on consumer &amp; in-store support</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="30" t="inlineStr">
-        <is>
-          <t>Warehousing &amp; insurance</t>
-        </is>
-      </c>
-      <c r="B31" s="38" t="n">
-        <v>12000</v>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>MANAGEMENT ESTIMATE, from August 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="33" t="inlineStr">
-        <is>
-          <t>Steady-state opex total</t>
-        </is>
-      </c>
-      <c r="B32" s="15">
-        <f>B23+B28+B29+B30+B31</f>
-        <v/>
       </c>
     </row>
   </sheetData>
@@ -965,17 +996,17 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>FUEGO TEQUILA BOTTLES — historic sales &amp; projection</t>
         </is>
       </c>
-      <c r="B1" s="27" t="n"/>
-      <c r="C1" s="27" t="n"/>
-      <c r="D1" s="27" t="n"/>
-      <c r="E1" s="27" t="n"/>
-      <c r="F1" s="27" t="n"/>
-      <c r="G1" s="27" t="n"/>
+      <c r="B1" s="26" t="n"/>
+      <c r="C1" s="26" t="n"/>
+      <c r="D1" s="26" t="n"/>
+      <c r="E1" s="26" t="n"/>
+      <c r="F1" s="26" t="n"/>
+      <c r="G1" s="26" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -985,328 +1016,328 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="39" t="inlineStr">
+      <c r="A3" s="38" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B3" s="39" t="inlineStr">
+      <c r="B3" s="38" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="C3" s="39" t="inlineStr">
+      <c r="C3" s="38" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D3" s="39" t="inlineStr">
+      <c r="D3" s="38" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="E3" s="39" t="inlineStr">
+      <c r="E3" s="38" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr"/>
-      <c r="G3" s="39" t="inlineStr">
+      <c r="G3" s="38" t="inlineStr">
         <is>
           <t>2027 (proj)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="30" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>January</t>
         </is>
       </c>
-      <c r="C4" s="35" t="n">
+      <c r="C4" s="34" t="n">
         <v>87354</v>
       </c>
-      <c r="D4" s="35" t="n">
+      <c r="D4" s="34" t="n">
         <v>107377.8</v>
       </c>
-      <c r="E4" s="35" t="n">
+      <c r="E4" s="34" t="n">
         <v>185865.3</v>
       </c>
-      <c r="G4" s="15">
+      <c r="G4" s="14">
         <f>(D4+E4)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>February</t>
         </is>
       </c>
-      <c r="C5" s="35" t="n">
+      <c r="C5" s="34" t="n">
         <v>7728</v>
       </c>
-      <c r="D5" s="35" t="n">
+      <c r="D5" s="34" t="n">
         <v>46920</v>
       </c>
-      <c r="E5" s="35" t="n">
+      <c r="E5" s="34" t="n">
         <v>209857.2</v>
       </c>
-      <c r="G5" s="15">
+      <c r="G5" s="14">
         <f>(D5+E5)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="30" t="inlineStr">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>March</t>
         </is>
       </c>
-      <c r="D6" s="35" t="n">
+      <c r="D6" s="34" t="n">
         <v>126617.4</v>
       </c>
-      <c r="E6" s="35" t="n">
+      <c r="E6" s="34" t="n">
         <v>260918.59</v>
       </c>
-      <c r="G6" s="15">
+      <c r="G6" s="14">
         <f>(D6+E6)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="30" t="inlineStr">
+      <c r="A7" s="29" t="inlineStr">
         <is>
           <t>April</t>
         </is>
       </c>
-      <c r="C7" s="35" t="n">
+      <c r="C7" s="34" t="n">
         <v>21931.51</v>
       </c>
-      <c r="D7" s="35" t="n">
+      <c r="D7" s="34" t="n">
         <v>663918</v>
       </c>
-      <c r="E7" s="35" t="n">
+      <c r="E7" s="34" t="n">
         <v>470561.32</v>
       </c>
-      <c r="G7" s="15">
+      <c r="G7" s="14">
         <f>(D7+E7)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="30" t="inlineStr">
+      <c r="A8" s="29" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="C8" s="35" t="n">
+      <c r="C8" s="34" t="n">
         <v>1895.8</v>
       </c>
-      <c r="D8" s="35" t="n">
+      <c r="D8" s="34" t="n">
         <v>168670.5</v>
       </c>
-      <c r="E8" s="35" t="n">
+      <c r="E8" s="34" t="n">
         <v>167687.8</v>
       </c>
-      <c r="G8" s="15">
+      <c r="G8" s="14">
         <f>(D8+E8)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>June</t>
         </is>
       </c>
-      <c r="C9" s="35" t="n">
+      <c r="C9" s="34" t="n">
         <v>68533.21000000001</v>
       </c>
-      <c r="D9" s="35" t="n">
+      <c r="D9" s="34" t="n">
         <v>98574.11</v>
       </c>
-      <c r="E9" s="35" t="n">
+      <c r="E9" s="34" t="n">
         <v>60059.82</v>
       </c>
-      <c r="G9" s="15">
+      <c r="G9" s="14">
         <f>(D9+E9)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="30" t="inlineStr">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t>July</t>
         </is>
       </c>
-      <c r="C10" s="35" t="n">
+      <c r="C10" s="34" t="n">
         <v>36027.3</v>
       </c>
-      <c r="D10" s="35" t="n">
+      <c r="D10" s="34" t="n">
         <v>266641.05</v>
       </c>
-      <c r="E10" s="35" t="n">
+      <c r="E10" s="34" t="n">
         <v>188654.34</v>
       </c>
-      <c r="G10" s="15">
+      <c r="G10" s="14">
         <f>(D10+E10)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="30" t="inlineStr">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t>August</t>
         </is>
       </c>
-      <c r="C11" s="35" t="n">
+      <c r="C11" s="34" t="n">
         <v>5796</v>
       </c>
-      <c r="D11" s="35" t="n">
+      <c r="D11" s="34" t="n">
         <v>44441.56</v>
       </c>
-      <c r="E11" s="15">
+      <c r="E11" s="14">
         <f>D11*$B$19</f>
         <v/>
       </c>
-      <c r="G11" s="15">
+      <c r="G11" s="14">
         <f>(D11+E11)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="A12" s="29" t="inlineStr">
         <is>
           <t>September</t>
         </is>
       </c>
-      <c r="B12" s="35" t="n">
+      <c r="B12" s="34" t="n">
         <v>1334</v>
       </c>
-      <c r="C12" s="35" t="n">
+      <c r="C12" s="34" t="n">
         <v>46252.59</v>
       </c>
-      <c r="D12" s="35" t="n">
+      <c r="D12" s="34" t="n">
         <v>65847.11</v>
       </c>
-      <c r="E12" s="15">
+      <c r="E12" s="14">
         <f>D12*$B$19</f>
         <v/>
       </c>
-      <c r="G12" s="15">
+      <c r="G12" s="14">
         <f>(D12+E12)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="30" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>October</t>
         </is>
       </c>
-      <c r="B13" s="35" t="n">
+      <c r="B13" s="34" t="n">
         <v>2894</v>
       </c>
-      <c r="C13" s="35" t="n">
+      <c r="C13" s="34" t="n">
         <v>530949.8100000001</v>
       </c>
-      <c r="D13" s="35" t="n">
+      <c r="D13" s="34" t="n">
         <v>63268.38</v>
       </c>
-      <c r="E13" s="15">
+      <c r="E13" s="14">
         <f>D13*$B$19</f>
         <v/>
       </c>
-      <c r="G13" s="15">
+      <c r="G13" s="14">
         <f>(D13+E13)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="30" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>November</t>
         </is>
       </c>
-      <c r="C14" s="35" t="n">
+      <c r="C14" s="34" t="n">
         <v>81964.75</v>
       </c>
-      <c r="D14" s="35" t="n">
+      <c r="D14" s="34" t="n">
         <v>257848.55</v>
       </c>
-      <c r="E14" s="15">
+      <c r="E14" s="14">
         <f>D14*$B$19</f>
         <v/>
       </c>
-      <c r="G14" s="15">
+      <c r="G14" s="14">
         <f>(D14+E14)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="30" t="inlineStr">
+      <c r="A15" s="29" t="inlineStr">
         <is>
           <t>December</t>
         </is>
       </c>
-      <c r="B15" s="35" t="n">
+      <c r="B15" s="34" t="n">
         <v>21919</v>
       </c>
-      <c r="C15" s="35" t="n">
+      <c r="C15" s="34" t="n">
         <v>138333.09</v>
       </c>
-      <c r="D15" s="35" t="n">
+      <c r="D15" s="34" t="n">
         <v>35332.6</v>
       </c>
-      <c r="E15" s="15">
+      <c r="E15" s="14">
         <f>D15*$B$19</f>
         <v/>
       </c>
-      <c r="G15" s="15">
+      <c r="G15" s="14">
         <f>(D15+E15)/($D$16+$E$16)*$B$21</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="33" t="inlineStr">
+      <c r="A16" s="32" t="inlineStr">
         <is>
           <t>Annual total</t>
         </is>
       </c>
-      <c r="B16" s="40">
+      <c r="B16" s="39">
         <f>SUM(B4:B15)</f>
         <v/>
       </c>
-      <c r="C16" s="40">
+      <c r="C16" s="39">
         <f>SUM(C4:C15)</f>
         <v/>
       </c>
-      <c r="D16" s="40">
+      <c r="D16" s="39">
         <f>SUM(D4:D15)</f>
         <v/>
       </c>
-      <c r="E16" s="40">
+      <c r="E16" s="39">
         <f>SUM(E4:E15)</f>
         <v/>
       </c>
-      <c r="G16" s="40">
+      <c r="G16" s="39">
         <f>SUM(G4:G15)</f>
         <v/>
       </c>
     </row>
     <row r="17"/>
     <row r="18">
-      <c r="A18" s="28" t="inlineStr">
+      <c r="A18" s="27" t="inlineStr">
         <is>
           <t>Projection assumptions</t>
         </is>
       </c>
-      <c r="B18" s="29" t="n"/>
-      <c r="C18" s="29" t="n"/>
+      <c r="B18" s="28" t="n"/>
+      <c r="C18" s="28" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="30" t="inlineStr">
+      <c r="A19" s="29" t="inlineStr">
         <is>
           <t>YoY growth (Jan-Jul 26 vs Jan-Jul 25)</t>
         </is>
@@ -1322,12 +1353,12 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="30" t="inlineStr">
+      <c r="A20" s="29" t="inlineStr">
         <is>
           <t>2027 growth on 2026</t>
         </is>
       </c>
-      <c r="B20" s="34" t="n">
+      <c r="B20" s="33" t="n">
         <v>0.05</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1337,23 +1368,23 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="30" t="inlineStr">
+      <c r="A21" s="29" t="inlineStr">
         <is>
           <t>2027 total</t>
         </is>
       </c>
-      <c r="B21" s="15">
+      <c r="B21" s="14">
         <f>E16*(1+B20)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="30" t="inlineStr">
+      <c r="A22" s="29" t="inlineStr">
         <is>
           <t>Bottle gross margin %</t>
         </is>
       </c>
-      <c r="B22" s="34" t="n">
+      <c r="B22" s="33" t="n">
         <v>0.3</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1408,710 +1439,710 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>P&amp;L (ACCRUAL) — Doña Fuego cans + Fuego Tequila bottles</t>
         </is>
       </c>
-      <c r="B1" s="27" t="n"/>
-      <c r="C1" s="27" t="n"/>
-      <c r="D1" s="27" t="n"/>
-      <c r="E1" s="27" t="n"/>
-      <c r="F1" s="27" t="n"/>
-      <c r="G1" s="27" t="n"/>
-      <c r="H1" s="27" t="n"/>
-      <c r="I1" s="27" t="n"/>
-      <c r="J1" s="27" t="n"/>
-      <c r="K1" s="27" t="n"/>
-      <c r="L1" s="27" t="n"/>
-      <c r="M1" s="27" t="n"/>
-      <c r="N1" s="27" t="n"/>
-      <c r="O1" s="27" t="n"/>
-      <c r="P1" s="27" t="n"/>
-      <c r="Q1" s="27" t="n"/>
-      <c r="R1" s="27" t="n"/>
-      <c r="S1" s="27" t="n"/>
-      <c r="T1" s="27" t="n"/>
-      <c r="U1" s="27" t="n"/>
+      <c r="B1" s="26" t="n"/>
+      <c r="C1" s="26" t="n"/>
+      <c r="D1" s="26" t="n"/>
+      <c r="E1" s="26" t="n"/>
+      <c r="F1" s="26" t="n"/>
+      <c r="G1" s="26" t="n"/>
+      <c r="H1" s="26" t="n"/>
+      <c r="I1" s="26" t="n"/>
+      <c r="J1" s="26" t="n"/>
+      <c r="K1" s="26" t="n"/>
+      <c r="L1" s="26" t="n"/>
+      <c r="M1" s="26" t="n"/>
+      <c r="N1" s="26" t="n"/>
+      <c r="O1" s="26" t="n"/>
+      <c r="P1" s="26" t="n"/>
+      <c r="Q1" s="26" t="n"/>
+      <c r="R1" s="26" t="n"/>
+      <c r="S1" s="26" t="n"/>
+      <c r="T1" s="26" t="n"/>
+      <c r="U1" s="26" t="n"/>
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="39" t="inlineStr">
+      <c r="A3" s="38" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B3" s="41" t="n">
+      <c r="B3" s="40" t="n">
         <v>46174</v>
       </c>
-      <c r="C3" s="41" t="n">
+      <c r="C3" s="40" t="n">
         <v>46204</v>
       </c>
-      <c r="D3" s="41" t="n">
+      <c r="D3" s="40" t="n">
         <v>46235</v>
       </c>
-      <c r="E3" s="41" t="n">
+      <c r="E3" s="40" t="n">
         <v>46266</v>
       </c>
-      <c r="F3" s="41" t="n">
+      <c r="F3" s="40" t="n">
         <v>46296</v>
       </c>
-      <c r="G3" s="41" t="n">
+      <c r="G3" s="40" t="n">
         <v>46327</v>
       </c>
-      <c r="H3" s="41" t="n">
+      <c r="H3" s="40" t="n">
         <v>46357</v>
       </c>
-      <c r="I3" s="41" t="n">
+      <c r="I3" s="40" t="n">
         <v>46388</v>
       </c>
-      <c r="J3" s="41" t="n">
+      <c r="J3" s="40" t="n">
         <v>46419</v>
       </c>
-      <c r="K3" s="41" t="n">
+      <c r="K3" s="40" t="n">
         <v>46447</v>
       </c>
-      <c r="L3" s="41" t="n">
+      <c r="L3" s="40" t="n">
         <v>46478</v>
       </c>
-      <c r="M3" s="41" t="n">
+      <c r="M3" s="40" t="n">
         <v>46508</v>
       </c>
-      <c r="N3" s="41" t="n">
+      <c r="N3" s="40" t="n">
         <v>46539</v>
       </c>
-      <c r="O3" s="41" t="n">
+      <c r="O3" s="40" t="n">
         <v>46569</v>
       </c>
-      <c r="P3" s="41" t="n">
+      <c r="P3" s="40" t="n">
         <v>46600</v>
       </c>
-      <c r="Q3" s="41" t="n">
+      <c r="Q3" s="40" t="n">
         <v>46631</v>
       </c>
-      <c r="R3" s="41" t="n">
+      <c r="R3" s="40" t="n">
         <v>46661</v>
       </c>
-      <c r="S3" s="41" t="n">
+      <c r="S3" s="40" t="n">
         <v>46692</v>
       </c>
-      <c r="T3" s="41" t="n">
+      <c r="T3" s="40" t="n">
         <v>46722</v>
       </c>
-      <c r="U3" s="39" t="inlineStr">
+      <c r="U3" s="38" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="30" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>Cases delivered (cans)</t>
         </is>
       </c>
-      <c r="B4" s="42" t="n">
+      <c r="B4" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="C4" s="42" t="n">
+      <c r="C4" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="43">
+      <c r="D4" s="42">
         <f>Assumptions!B7</f>
         <v/>
       </c>
-      <c r="E4" s="42" t="n">
+      <c r="E4" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="43">
+      <c r="F4" s="42">
         <f>Assumptions!B8</f>
         <v/>
       </c>
-      <c r="G4" s="43">
-        <f>Assumptions!B12</f>
-        <v/>
-      </c>
-      <c r="H4" s="43">
-        <f>Assumptions!B12</f>
-        <v/>
-      </c>
-      <c r="I4" s="43">
-        <f>Assumptions!B12</f>
-        <v/>
-      </c>
-      <c r="J4" s="43">
-        <f>Assumptions!B12</f>
-        <v/>
-      </c>
-      <c r="K4" s="43">
-        <f>Assumptions!B12</f>
-        <v/>
-      </c>
-      <c r="L4" s="43">
-        <f>Assumptions!B12</f>
-        <v/>
-      </c>
-      <c r="M4" s="43">
-        <f>Assumptions!B12</f>
-        <v/>
-      </c>
-      <c r="N4" s="43">
-        <f>Assumptions!B12</f>
-        <v/>
-      </c>
-      <c r="O4" s="43">
-        <f>Assumptions!B12</f>
-        <v/>
-      </c>
-      <c r="P4" s="43">
-        <f>Assumptions!B12</f>
-        <v/>
-      </c>
-      <c r="Q4" s="43">
-        <f>Assumptions!B12</f>
-        <v/>
-      </c>
-      <c r="R4" s="43">
-        <f>Assumptions!B12</f>
-        <v/>
-      </c>
-      <c r="S4" s="43">
-        <f>Assumptions!B12</f>
-        <v/>
-      </c>
-      <c r="T4" s="43">
-        <f>Assumptions!B12</f>
-        <v/>
-      </c>
-      <c r="U4" s="44">
+      <c r="G4" s="42">
+        <f>IF(OR(MONTH(G3)&gt;=10,MONTH(G3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
+        <v/>
+      </c>
+      <c r="H4" s="42">
+        <f>IF(OR(MONTH(H3)&gt;=10,MONTH(H3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
+        <v/>
+      </c>
+      <c r="I4" s="42">
+        <f>IF(OR(MONTH(I3)&gt;=10,MONTH(I3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
+        <v/>
+      </c>
+      <c r="J4" s="42">
+        <f>IF(OR(MONTH(J3)&gt;=10,MONTH(J3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
+        <v/>
+      </c>
+      <c r="K4" s="42">
+        <f>IF(OR(MONTH(K3)&gt;=10,MONTH(K3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
+        <v/>
+      </c>
+      <c r="L4" s="42">
+        <f>IF(OR(MONTH(L3)&gt;=10,MONTH(L3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
+        <v/>
+      </c>
+      <c r="M4" s="42">
+        <f>IF(OR(MONTH(M3)&gt;=10,MONTH(M3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
+        <v/>
+      </c>
+      <c r="N4" s="42">
+        <f>IF(OR(MONTH(N3)&gt;=10,MONTH(N3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
+        <v/>
+      </c>
+      <c r="O4" s="42">
+        <f>IF(OR(MONTH(O3)&gt;=10,MONTH(O3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
+        <v/>
+      </c>
+      <c r="P4" s="42">
+        <f>IF(OR(MONTH(P3)&gt;=10,MONTH(P3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
+        <v/>
+      </c>
+      <c r="Q4" s="42">
+        <f>IF(OR(MONTH(Q3)&gt;=10,MONTH(Q3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
+        <v/>
+      </c>
+      <c r="R4" s="42">
+        <f>IF(OR(MONTH(R3)&gt;=10,MONTH(R3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
+        <v/>
+      </c>
+      <c r="S4" s="42">
+        <f>IF(OR(MONTH(S3)&gt;=10,MONTH(S3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
+        <v/>
+      </c>
+      <c r="T4" s="42">
+        <f>IF(OR(MONTH(T3)&gt;=10,MONTH(T3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
+        <v/>
+      </c>
+      <c r="U4" s="43">
         <f>SUM(B4:T4)</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>Can revenue</t>
         </is>
       </c>
-      <c r="B5" s="15">
-        <f>B4*Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="C5" s="15">
-        <f>C4*Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="D5" s="15">
-        <f>D4*Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="E5" s="15">
-        <f>E4*Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="F5" s="15">
-        <f>F4*Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="G5" s="15">
-        <f>G4*Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="H5" s="15">
-        <f>H4*Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="I5" s="15">
-        <f>I4*Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="J5" s="15">
-        <f>J4*Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="K5" s="15">
-        <f>K4*Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="L5" s="15">
-        <f>L4*Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="M5" s="15">
-        <f>M4*Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="N5" s="15">
-        <f>N4*Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="O5" s="15">
-        <f>O4*Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="P5" s="15">
-        <f>P4*Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="Q5" s="15">
-        <f>Q4*Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="R5" s="15">
-        <f>R4*Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="S5" s="15">
-        <f>S4*Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="T5" s="15">
-        <f>T4*Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="U5" s="45">
+      <c r="B5" s="14">
+        <f>B4*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="C5" s="14">
+        <f>C4*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="D5" s="14">
+        <f>D4*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="E5" s="14">
+        <f>E4*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="F5" s="14">
+        <f>F4*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="G5" s="14">
+        <f>G4*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="H5" s="14">
+        <f>H4*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="I5" s="14">
+        <f>I4*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="J5" s="14">
+        <f>J4*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="K5" s="14">
+        <f>K4*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="L5" s="14">
+        <f>L4*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="M5" s="14">
+        <f>M4*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="N5" s="14">
+        <f>N4*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="O5" s="14">
+        <f>O4*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="P5" s="14">
+        <f>P4*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="Q5" s="14">
+        <f>Q4*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="R5" s="14">
+        <f>R4*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="S5" s="14">
+        <f>S4*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="T5" s="14">
+        <f>T4*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="U5" s="44">
         <f>SUM(B5:T5)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="30" t="inlineStr">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>Bottle revenue</t>
         </is>
       </c>
-      <c r="B6" s="21">
+      <c r="B6" s="20">
         <f>Bottles!E9</f>
         <v/>
       </c>
-      <c r="C6" s="21">
+      <c r="C6" s="20">
         <f>Bottles!E10</f>
         <v/>
       </c>
-      <c r="D6" s="21">
+      <c r="D6" s="20">
         <f>Bottles!E11</f>
         <v/>
       </c>
-      <c r="E6" s="21">
+      <c r="E6" s="20">
         <f>Bottles!E12</f>
         <v/>
       </c>
-      <c r="F6" s="21">
+      <c r="F6" s="20">
         <f>Bottles!E13</f>
         <v/>
       </c>
-      <c r="G6" s="21">
+      <c r="G6" s="20">
         <f>Bottles!E14</f>
         <v/>
       </c>
-      <c r="H6" s="21">
+      <c r="H6" s="20">
         <f>Bottles!E15</f>
         <v/>
       </c>
-      <c r="I6" s="21">
+      <c r="I6" s="20">
         <f>Bottles!G4</f>
         <v/>
       </c>
-      <c r="J6" s="21">
+      <c r="J6" s="20">
         <f>Bottles!G5</f>
         <v/>
       </c>
-      <c r="K6" s="21">
+      <c r="K6" s="20">
         <f>Bottles!G6</f>
         <v/>
       </c>
-      <c r="L6" s="21">
+      <c r="L6" s="20">
         <f>Bottles!G7</f>
         <v/>
       </c>
-      <c r="M6" s="21">
+      <c r="M6" s="20">
         <f>Bottles!G8</f>
         <v/>
       </c>
-      <c r="N6" s="21">
+      <c r="N6" s="20">
         <f>Bottles!G9</f>
         <v/>
       </c>
-      <c r="O6" s="21">
+      <c r="O6" s="20">
         <f>Bottles!G10</f>
         <v/>
       </c>
-      <c r="P6" s="21">
+      <c r="P6" s="20">
         <f>Bottles!G11</f>
         <v/>
       </c>
-      <c r="Q6" s="21">
+      <c r="Q6" s="20">
         <f>Bottles!G12</f>
         <v/>
       </c>
-      <c r="R6" s="21">
+      <c r="R6" s="20">
         <f>Bottles!G13</f>
         <v/>
       </c>
-      <c r="S6" s="21">
+      <c r="S6" s="20">
         <f>Bottles!G14</f>
         <v/>
       </c>
-      <c r="T6" s="21">
+      <c r="T6" s="20">
         <f>Bottles!G15</f>
         <v/>
       </c>
-      <c r="U6" s="45">
+      <c r="U6" s="44">
         <f>SUM(B6:T6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="33" t="inlineStr">
+      <c r="A7" s="32" t="inlineStr">
         <is>
           <t>Total revenue</t>
         </is>
       </c>
-      <c r="B7" s="16">
+      <c r="B7" s="15">
         <f>B5+B6</f>
         <v/>
       </c>
-      <c r="C7" s="16">
+      <c r="C7" s="15">
         <f>C5+C6</f>
         <v/>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="15">
         <f>D5+D6</f>
         <v/>
       </c>
-      <c r="E7" s="16">
+      <c r="E7" s="15">
         <f>E5+E6</f>
         <v/>
       </c>
-      <c r="F7" s="16">
+      <c r="F7" s="15">
         <f>F5+F6</f>
         <v/>
       </c>
-      <c r="G7" s="16">
+      <c r="G7" s="15">
         <f>G5+G6</f>
         <v/>
       </c>
-      <c r="H7" s="16">
+      <c r="H7" s="15">
         <f>H5+H6</f>
         <v/>
       </c>
-      <c r="I7" s="16">
+      <c r="I7" s="15">
         <f>I5+I6</f>
         <v/>
       </c>
-      <c r="J7" s="16">
+      <c r="J7" s="15">
         <f>J5+J6</f>
         <v/>
       </c>
-      <c r="K7" s="16">
+      <c r="K7" s="15">
         <f>K5+K6</f>
         <v/>
       </c>
-      <c r="L7" s="16">
+      <c r="L7" s="15">
         <f>L5+L6</f>
         <v/>
       </c>
-      <c r="M7" s="16">
+      <c r="M7" s="15">
         <f>M5+M6</f>
         <v/>
       </c>
-      <c r="N7" s="16">
+      <c r="N7" s="15">
         <f>N5+N6</f>
         <v/>
       </c>
-      <c r="O7" s="16">
+      <c r="O7" s="15">
         <f>O5+O6</f>
         <v/>
       </c>
-      <c r="P7" s="16">
+      <c r="P7" s="15">
         <f>P5+P6</f>
         <v/>
       </c>
-      <c r="Q7" s="16">
+      <c r="Q7" s="15">
         <f>Q5+Q6</f>
         <v/>
       </c>
-      <c r="R7" s="16">
+      <c r="R7" s="15">
         <f>R5+R6</f>
         <v/>
       </c>
-      <c r="S7" s="16">
+      <c r="S7" s="15">
         <f>S5+S6</f>
         <v/>
       </c>
-      <c r="T7" s="16">
+      <c r="T7" s="15">
         <f>T5+T6</f>
         <v/>
       </c>
-      <c r="U7" s="45">
+      <c r="U7" s="44">
         <f>SUM(B7:T7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="30" t="inlineStr">
+      <c r="A8" s="29" t="inlineStr">
         <is>
           <t>Can COGS</t>
         </is>
       </c>
-      <c r="B8" s="15">
-        <f>-B5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="C8" s="15">
-        <f>-C5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="D8" s="15">
-        <f>-D5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="E8" s="15">
-        <f>-E5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="F8" s="15">
-        <f>-F5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="G8" s="15">
-        <f>-G5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="H8" s="15">
-        <f>-H5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="I8" s="15">
-        <f>-I5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="J8" s="15">
-        <f>-J5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="K8" s="15">
-        <f>-K5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="L8" s="15">
-        <f>-L5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="M8" s="15">
-        <f>-M5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="N8" s="15">
-        <f>-N5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="O8" s="15">
-        <f>-O5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="P8" s="15">
-        <f>-P5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="Q8" s="15">
-        <f>-Q5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="R8" s="15">
-        <f>-R5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="S8" s="15">
-        <f>-S5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="T8" s="15">
-        <f>-T5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="U8" s="45">
+      <c r="B8" s="14">
+        <f>-B5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="C8" s="14">
+        <f>-C5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="D8" s="14">
+        <f>-D5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="E8" s="14">
+        <f>-E5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="F8" s="14">
+        <f>-F5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="G8" s="14">
+        <f>-G5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="H8" s="14">
+        <f>-H5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="I8" s="14">
+        <f>-I5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="J8" s="14">
+        <f>-J5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="K8" s="14">
+        <f>-K5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="L8" s="14">
+        <f>-L5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="M8" s="14">
+        <f>-M5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="N8" s="14">
+        <f>-N5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="O8" s="14">
+        <f>-O5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="P8" s="14">
+        <f>-P5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="Q8" s="14">
+        <f>-Q5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="R8" s="14">
+        <f>-R5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="S8" s="14">
+        <f>-S5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="T8" s="14">
+        <f>-T5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="U8" s="44">
         <f>SUM(B8:T8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>Bottle COGS</t>
         </is>
       </c>
-      <c r="B9" s="15">
+      <c r="B9" s="14">
         <f>-B6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="14">
         <f>-C6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="D9" s="15">
+      <c r="D9" s="14">
         <f>-D6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="E9" s="15">
+      <c r="E9" s="14">
         <f>-E6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="F9" s="15">
+      <c r="F9" s="14">
         <f>-F6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="G9" s="15">
+      <c r="G9" s="14">
         <f>-G6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="H9" s="15">
+      <c r="H9" s="14">
         <f>-H6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="I9" s="15">
+      <c r="I9" s="14">
         <f>-I6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="J9" s="15">
+      <c r="J9" s="14">
         <f>-J6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="K9" s="15">
+      <c r="K9" s="14">
         <f>-K6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="L9" s="15">
+      <c r="L9" s="14">
         <f>-L6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="M9" s="15">
+      <c r="M9" s="14">
         <f>-M6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="N9" s="15">
+      <c r="N9" s="14">
         <f>-N6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="O9" s="15">
+      <c r="O9" s="14">
         <f>-O6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="P9" s="15">
+      <c r="P9" s="14">
         <f>-P6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="Q9" s="15">
+      <c r="Q9" s="14">
         <f>-Q6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="R9" s="15">
+      <c r="R9" s="14">
         <f>-R6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="S9" s="15">
+      <c r="S9" s="14">
         <f>-S6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="T9" s="15">
+      <c r="T9" s="14">
         <f>-T6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="U9" s="45">
+      <c r="U9" s="44">
         <f>SUM(B9:T9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="33" t="inlineStr">
+      <c r="A10" s="32" t="inlineStr">
         <is>
           <t>Gross margin</t>
         </is>
       </c>
-      <c r="B10" s="16">
+      <c r="B10" s="15">
         <f>B7+B8+B9</f>
         <v/>
       </c>
-      <c r="C10" s="16">
+      <c r="C10" s="15">
         <f>C7+C8+C9</f>
         <v/>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="15">
         <f>D7+D8+D9</f>
         <v/>
       </c>
-      <c r="E10" s="16">
+      <c r="E10" s="15">
         <f>E7+E8+E9</f>
         <v/>
       </c>
-      <c r="F10" s="16">
+      <c r="F10" s="15">
         <f>F7+F8+F9</f>
         <v/>
       </c>
-      <c r="G10" s="16">
+      <c r="G10" s="15">
         <f>G7+G8+G9</f>
         <v/>
       </c>
-      <c r="H10" s="16">
+      <c r="H10" s="15">
         <f>H7+H8+H9</f>
         <v/>
       </c>
-      <c r="I10" s="16">
+      <c r="I10" s="15">
         <f>I7+I8+I9</f>
         <v/>
       </c>
-      <c r="J10" s="16">
+      <c r="J10" s="15">
         <f>J7+J8+J9</f>
         <v/>
       </c>
-      <c r="K10" s="16">
+      <c r="K10" s="15">
         <f>K7+K8+K9</f>
         <v/>
       </c>
-      <c r="L10" s="16">
+      <c r="L10" s="15">
         <f>L7+L8+L9</f>
         <v/>
       </c>
-      <c r="M10" s="16">
+      <c r="M10" s="15">
         <f>M7+M8+M9</f>
         <v/>
       </c>
-      <c r="N10" s="16">
+      <c r="N10" s="15">
         <f>N7+N8+N9</f>
         <v/>
       </c>
-      <c r="O10" s="16">
+      <c r="O10" s="15">
         <f>O7+O8+O9</f>
         <v/>
       </c>
-      <c r="P10" s="16">
+      <c r="P10" s="15">
         <f>P7+P8+P9</f>
         <v/>
       </c>
-      <c r="Q10" s="16">
+      <c r="Q10" s="15">
         <f>Q7+Q8+Q9</f>
         <v/>
       </c>
-      <c r="R10" s="16">
+      <c r="R10" s="15">
         <f>R7+R8+R9</f>
         <v/>
       </c>
-      <c r="S10" s="16">
+      <c r="S10" s="15">
         <f>S7+S8+S9</f>
         <v/>
       </c>
-      <c r="T10" s="16">
+      <c r="T10" s="15">
         <f>T7+T8+T9</f>
         <v/>
       </c>
-      <c r="U10" s="45">
+      <c r="U10" s="44">
         <f>SUM(B10:T10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="30" t="inlineStr">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t>Gross margin %</t>
         </is>
@@ -2192,187 +2223,187 @@
         <f>IF(T7=0,0,T10/T7)</f>
         <v/>
       </c>
-      <c r="U11" s="46">
+      <c r="U11" s="45">
         <f>U10/U7</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="A12" s="29" t="inlineStr">
         <is>
           <t>Opex (sales, ops &amp; distribution)</t>
         </is>
       </c>
-      <c r="B12" s="15">
-        <f>-(Assumptions!$B$23+IF(B$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(B$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
-        <v/>
-      </c>
-      <c r="C12" s="15">
-        <f>-(Assumptions!$B$23+IF(C$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(C$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
-        <v/>
-      </c>
-      <c r="D12" s="15">
-        <f>-(Assumptions!$B$23+IF(D$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(D$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
-        <v/>
-      </c>
-      <c r="E12" s="15">
-        <f>-(Assumptions!$B$23+IF(E$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(E$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
-        <v/>
-      </c>
-      <c r="F12" s="15">
-        <f>-(Assumptions!$B$23+IF(F$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(F$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
-        <v/>
-      </c>
-      <c r="G12" s="15">
-        <f>-(Assumptions!$B$23+IF(G$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(G$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
-        <v/>
-      </c>
-      <c r="H12" s="15">
-        <f>-(Assumptions!$B$23+IF(H$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(H$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
-        <v/>
-      </c>
-      <c r="I12" s="15">
-        <f>-(Assumptions!$B$23+IF(I$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(I$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
-        <v/>
-      </c>
-      <c r="J12" s="15">
-        <f>-(Assumptions!$B$23+IF(J$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(J$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
-        <v/>
-      </c>
-      <c r="K12" s="15">
-        <f>-(Assumptions!$B$23+IF(K$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(K$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
-        <v/>
-      </c>
-      <c r="L12" s="15">
-        <f>-(Assumptions!$B$23+IF(L$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(L$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
-        <v/>
-      </c>
-      <c r="M12" s="15">
-        <f>-(Assumptions!$B$23+IF(M$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(M$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
-        <v/>
-      </c>
-      <c r="N12" s="15">
-        <f>-(Assumptions!$B$23+IF(N$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(N$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
-        <v/>
-      </c>
-      <c r="O12" s="15">
-        <f>-(Assumptions!$B$23+IF(O$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(O$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
-        <v/>
-      </c>
-      <c r="P12" s="15">
-        <f>-(Assumptions!$B$23+IF(P$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(P$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
-        <v/>
-      </c>
-      <c r="Q12" s="15">
-        <f>-(Assumptions!$B$23+IF(Q$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(Q$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
-        <v/>
-      </c>
-      <c r="R12" s="15">
-        <f>-(Assumptions!$B$23+IF(R$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(R$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
-        <v/>
-      </c>
-      <c r="S12" s="15">
-        <f>-(Assumptions!$B$23+IF(S$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(S$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
-        <v/>
-      </c>
-      <c r="T12" s="15">
-        <f>-(Assumptions!$B$23+IF(T$3&gt;=DATE(2026,7,1),Assumptions!$B$28+Assumptions!$B$29,0)+IF(T$3&gt;=DATE(2026,8,1),Assumptions!$B$30+Assumptions!$B$31,0))</f>
-        <v/>
-      </c>
-      <c r="U12" s="45">
+      <c r="B12" s="14">
+        <f>-(Assumptions!$B$26+IF(B$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(B$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="C12" s="14">
+        <f>-(Assumptions!$B$26+IF(C$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(C$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="D12" s="14">
+        <f>-(Assumptions!$B$26+IF(D$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(D$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="E12" s="14">
+        <f>-(Assumptions!$B$26+IF(E$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(E$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="F12" s="14">
+        <f>-(Assumptions!$B$26+IF(F$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(F$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="G12" s="14">
+        <f>-(Assumptions!$B$26+IF(G$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(G$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="H12" s="14">
+        <f>-(Assumptions!$B$26+IF(H$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(H$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="I12" s="14">
+        <f>-(Assumptions!$B$26+IF(I$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(I$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="J12" s="14">
+        <f>-(Assumptions!$B$26+IF(J$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(J$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="K12" s="14">
+        <f>-(Assumptions!$B$26+IF(K$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(K$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="L12" s="14">
+        <f>-(Assumptions!$B$26+IF(L$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(L$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="M12" s="14">
+        <f>-(Assumptions!$B$26+IF(M$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(M$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="N12" s="14">
+        <f>-(Assumptions!$B$26+IF(N$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(N$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="O12" s="14">
+        <f>-(Assumptions!$B$26+IF(O$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(O$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="P12" s="14">
+        <f>-(Assumptions!$B$26+IF(P$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(P$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="Q12" s="14">
+        <f>-(Assumptions!$B$26+IF(Q$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(Q$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="R12" s="14">
+        <f>-(Assumptions!$B$26+IF(R$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(R$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="S12" s="14">
+        <f>-(Assumptions!$B$26+IF(S$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(S$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="T12" s="14">
+        <f>-(Assumptions!$B$26+IF(T$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(T$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <v/>
+      </c>
+      <c r="U12" s="44">
         <f>SUM(B12:T12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="33" t="inlineStr">
+      <c r="A13" s="32" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="B13" s="16">
+      <c r="B13" s="15">
         <f>B10+B12</f>
         <v/>
       </c>
-      <c r="C13" s="16">
+      <c r="C13" s="15">
         <f>C10+C12</f>
         <v/>
       </c>
-      <c r="D13" s="16">
+      <c r="D13" s="15">
         <f>D10+D12</f>
         <v/>
       </c>
-      <c r="E13" s="16">
+      <c r="E13" s="15">
         <f>E10+E12</f>
         <v/>
       </c>
-      <c r="F13" s="16">
+      <c r="F13" s="15">
         <f>F10+F12</f>
         <v/>
       </c>
-      <c r="G13" s="16">
+      <c r="G13" s="15">
         <f>G10+G12</f>
         <v/>
       </c>
-      <c r="H13" s="16">
+      <c r="H13" s="15">
         <f>H10+H12</f>
         <v/>
       </c>
-      <c r="I13" s="16">
+      <c r="I13" s="15">
         <f>I10+I12</f>
         <v/>
       </c>
-      <c r="J13" s="16">
+      <c r="J13" s="15">
         <f>J10+J12</f>
         <v/>
       </c>
-      <c r="K13" s="16">
+      <c r="K13" s="15">
         <f>K10+K12</f>
         <v/>
       </c>
-      <c r="L13" s="16">
+      <c r="L13" s="15">
         <f>L10+L12</f>
         <v/>
       </c>
-      <c r="M13" s="16">
+      <c r="M13" s="15">
         <f>M10+M12</f>
         <v/>
       </c>
-      <c r="N13" s="16">
+      <c r="N13" s="15">
         <f>N10+N12</f>
         <v/>
       </c>
-      <c r="O13" s="16">
+      <c r="O13" s="15">
         <f>O10+O12</f>
         <v/>
       </c>
-      <c r="P13" s="16">
+      <c r="P13" s="15">
         <f>P10+P12</f>
         <v/>
       </c>
-      <c r="Q13" s="16">
+      <c r="Q13" s="15">
         <f>Q10+Q12</f>
         <v/>
       </c>
-      <c r="R13" s="16">
+      <c r="R13" s="15">
         <f>R10+R12</f>
         <v/>
       </c>
-      <c r="S13" s="16">
+      <c r="S13" s="15">
         <f>S10+S12</f>
         <v/>
       </c>
-      <c r="T13" s="16">
+      <c r="T13" s="15">
         <f>T10+T12</f>
         <v/>
       </c>
-      <c r="U13" s="45">
+      <c r="U13" s="44">
         <f>SUM(B13:T13)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="30" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>EBITDA %</t>
         </is>
@@ -2453,7 +2484,7 @@
         <f>IF(T7=0,0,T13/T7)</f>
         <v/>
       </c>
-      <c r="U14" s="46">
+      <c r="U14" s="45">
         <f>U13/U7</f>
         <v/>
       </c>
@@ -2496,716 +2527,703 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>CASHFLOW (CASH BASIS) — brand entity</t>
         </is>
       </c>
-      <c r="B1" s="27" t="n"/>
-      <c r="C1" s="27" t="n"/>
-      <c r="D1" s="27" t="n"/>
-      <c r="E1" s="27" t="n"/>
-      <c r="F1" s="27" t="n"/>
-      <c r="G1" s="27" t="n"/>
-      <c r="H1" s="27" t="n"/>
-      <c r="I1" s="27" t="n"/>
-      <c r="J1" s="27" t="n"/>
-      <c r="K1" s="27" t="n"/>
-      <c r="L1" s="27" t="n"/>
-      <c r="M1" s="27" t="n"/>
-      <c r="N1" s="27" t="n"/>
-      <c r="O1" s="27" t="n"/>
-      <c r="P1" s="27" t="n"/>
-      <c r="Q1" s="27" t="n"/>
-      <c r="R1" s="27" t="n"/>
-      <c r="S1" s="27" t="n"/>
-      <c r="T1" s="27" t="n"/>
-      <c r="U1" s="27" t="n"/>
+      <c r="B1" s="26" t="n"/>
+      <c r="C1" s="26" t="n"/>
+      <c r="D1" s="26" t="n"/>
+      <c r="E1" s="26" t="n"/>
+      <c r="F1" s="26" t="n"/>
+      <c r="G1" s="26" t="n"/>
+      <c r="H1" s="26" t="n"/>
+      <c r="I1" s="26" t="n"/>
+      <c r="J1" s="26" t="n"/>
+      <c r="K1" s="26" t="n"/>
+      <c r="L1" s="26" t="n"/>
+      <c r="M1" s="26" t="n"/>
+      <c r="N1" s="26" t="n"/>
+      <c r="O1" s="26" t="n"/>
+      <c r="P1" s="26" t="n"/>
+      <c r="Q1" s="26" t="n"/>
+      <c r="R1" s="26" t="n"/>
+      <c r="S1" s="26" t="n"/>
+      <c r="T1" s="26" t="n"/>
+      <c r="U1" s="26" t="n"/>
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="39" t="inlineStr">
+      <c r="A3" s="38" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B3" s="41" t="n">
+      <c r="B3" s="40" t="n">
         <v>46174</v>
       </c>
-      <c r="C3" s="41" t="n">
+      <c r="C3" s="40" t="n">
         <v>46204</v>
       </c>
-      <c r="D3" s="41" t="n">
+      <c r="D3" s="40" t="n">
         <v>46235</v>
       </c>
-      <c r="E3" s="41" t="n">
+      <c r="E3" s="40" t="n">
         <v>46266</v>
       </c>
-      <c r="F3" s="41" t="n">
+      <c r="F3" s="40" t="n">
         <v>46296</v>
       </c>
-      <c r="G3" s="41" t="n">
+      <c r="G3" s="40" t="n">
         <v>46327</v>
       </c>
-      <c r="H3" s="41" t="n">
+      <c r="H3" s="40" t="n">
         <v>46357</v>
       </c>
-      <c r="I3" s="41" t="n">
+      <c r="I3" s="40" t="n">
         <v>46388</v>
       </c>
-      <c r="J3" s="41" t="n">
+      <c r="J3" s="40" t="n">
         <v>46419</v>
       </c>
-      <c r="K3" s="41" t="n">
+      <c r="K3" s="40" t="n">
         <v>46447</v>
       </c>
-      <c r="L3" s="41" t="n">
+      <c r="L3" s="40" t="n">
         <v>46478</v>
       </c>
-      <c r="M3" s="41" t="n">
+      <c r="M3" s="40" t="n">
         <v>46508</v>
       </c>
-      <c r="N3" s="41" t="n">
+      <c r="N3" s="40" t="n">
         <v>46539</v>
       </c>
-      <c r="O3" s="41" t="n">
+      <c r="O3" s="40" t="n">
         <v>46569</v>
       </c>
-      <c r="P3" s="41" t="n">
+      <c r="P3" s="40" t="n">
         <v>46600</v>
       </c>
-      <c r="Q3" s="41" t="n">
+      <c r="Q3" s="40" t="n">
         <v>46631</v>
       </c>
-      <c r="R3" s="41" t="n">
+      <c r="R3" s="40" t="n">
         <v>46661</v>
       </c>
-      <c r="S3" s="41" t="n">
+      <c r="S3" s="40" t="n">
         <v>46692</v>
       </c>
-      <c r="T3" s="41" t="n">
+      <c r="T3" s="40" t="n">
         <v>46722</v>
       </c>
-      <c r="U3" s="39" t="inlineStr">
+      <c r="U3" s="38" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="30" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>Can receipts (revenue +30 days)</t>
         </is>
       </c>
-      <c r="B4" s="15" t="n">
+      <c r="B4" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="C4" s="21">
+      <c r="C4" s="20">
         <f>'P&amp;L'!B5</f>
         <v/>
       </c>
-      <c r="D4" s="21">
+      <c r="D4" s="20">
         <f>'P&amp;L'!C5</f>
         <v/>
       </c>
-      <c r="E4" s="21">
+      <c r="E4" s="20">
         <f>'P&amp;L'!D5</f>
         <v/>
       </c>
-      <c r="F4" s="21">
+      <c r="F4" s="20">
         <f>'P&amp;L'!E5</f>
         <v/>
       </c>
-      <c r="G4" s="21">
+      <c r="G4" s="20">
         <f>'P&amp;L'!F5</f>
         <v/>
       </c>
-      <c r="H4" s="21">
+      <c r="H4" s="20">
         <f>'P&amp;L'!G5</f>
         <v/>
       </c>
-      <c r="I4" s="21">
+      <c r="I4" s="20">
         <f>'P&amp;L'!H5</f>
         <v/>
       </c>
-      <c r="J4" s="21">
+      <c r="J4" s="20">
         <f>'P&amp;L'!I5</f>
         <v/>
       </c>
-      <c r="K4" s="21">
+      <c r="K4" s="20">
         <f>'P&amp;L'!J5</f>
         <v/>
       </c>
-      <c r="L4" s="21">
+      <c r="L4" s="20">
         <f>'P&amp;L'!K5</f>
         <v/>
       </c>
-      <c r="M4" s="21">
+      <c r="M4" s="20">
         <f>'P&amp;L'!L5</f>
         <v/>
       </c>
-      <c r="N4" s="21">
+      <c r="N4" s="20">
         <f>'P&amp;L'!M5</f>
         <v/>
       </c>
-      <c r="O4" s="21">
+      <c r="O4" s="20">
         <f>'P&amp;L'!N5</f>
         <v/>
       </c>
-      <c r="P4" s="21">
+      <c r="P4" s="20">
         <f>'P&amp;L'!O5</f>
         <v/>
       </c>
-      <c r="Q4" s="21">
+      <c r="Q4" s="20">
         <f>'P&amp;L'!P5</f>
         <v/>
       </c>
-      <c r="R4" s="21">
+      <c r="R4" s="20">
         <f>'P&amp;L'!Q5</f>
         <v/>
       </c>
-      <c r="S4" s="21">
+      <c r="S4" s="20">
         <f>'P&amp;L'!R5</f>
         <v/>
       </c>
-      <c r="T4" s="21">
+      <c r="T4" s="20">
         <f>'P&amp;L'!S5</f>
         <v/>
       </c>
-      <c r="U4" s="45">
+      <c r="U4" s="44">
         <f>SUM(B4:T4)</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  Bron Pro (design/brand)</t>
         </is>
       </c>
-      <c r="B5" s="15">
-        <f>-103500*Assumptions!$B$24</f>
-        <v/>
-      </c>
-      <c r="D5" s="15">
-        <f>-243800*Assumptions!$B$24</f>
-        <v/>
-      </c>
-      <c r="U5" s="45">
+      <c r="B5" s="34" t="n">
+        <v>-124200</v>
+      </c>
+      <c r="D5" s="34" t="n">
+        <v>-292560</v>
+      </c>
+      <c r="U5" s="44">
         <f>SUM(B5:T5)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="30" t="inlineStr">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  Sullwaldt printing</t>
         </is>
       </c>
-      <c r="C6" s="15">
-        <f>-91066*Assumptions!$B$24</f>
-        <v/>
-      </c>
-      <c r="F6" s="15">
-        <f>-72400*Assumptions!$B$24</f>
-        <v/>
-      </c>
-      <c r="U6" s="45">
+      <c r="C6" s="34" t="n">
+        <v>-109279</v>
+      </c>
+      <c r="F6" s="34" t="n">
+        <v>-86880</v>
+      </c>
+      <c r="U6" s="44">
         <f>SUM(B6:T6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="30" t="inlineStr">
+      <c r="A7" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  Tiny Keg cans</t>
         </is>
       </c>
-      <c r="C7" s="15">
-        <f>-405950*Assumptions!$B$24</f>
-        <v/>
-      </c>
-      <c r="E7" s="15">
-        <f>-319000*Assumptions!$B$24</f>
-        <v/>
-      </c>
-      <c r="U7" s="45">
+      <c r="C7" s="34" t="n">
+        <v>-487140</v>
+      </c>
+      <c r="E7" s="34" t="n">
+        <v>-382800</v>
+      </c>
+      <c r="U7" s="44">
         <f>SUM(B7:T7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="30" t="inlineStr">
+      <c r="A8" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  Chep pallets</t>
         </is>
       </c>
-      <c r="B8" s="15">
-        <f>-14375*Assumptions!$B$24</f>
-        <v/>
-      </c>
-      <c r="U8" s="45">
+      <c r="B8" s="34" t="n">
+        <v>-17250</v>
+      </c>
+      <c r="U8" s="44">
         <f>SUM(B8:T8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  FAL distribution</t>
         </is>
       </c>
-      <c r="C9" s="15">
-        <f>-51750*Assumptions!$B$24</f>
-        <v/>
-      </c>
-      <c r="F9" s="15">
-        <f>-28000*Assumptions!$B$24</f>
-        <v/>
-      </c>
-      <c r="U9" s="45">
+      <c r="C9" s="34" t="n">
+        <v>-62100</v>
+      </c>
+      <c r="F9" s="34" t="n">
+        <v>-33600</v>
+      </c>
+      <c r="U9" s="44">
         <f>SUM(B9:T9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="30" t="inlineStr">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  Tiny Keg production</t>
         </is>
       </c>
-      <c r="D10" s="15">
-        <f>-373350*Assumptions!$B$24</f>
-        <v/>
-      </c>
-      <c r="E10" s="15">
-        <f>-293250*Assumptions!$B$24</f>
-        <v/>
-      </c>
-      <c r="U10" s="45">
+      <c r="D10" s="34" t="n">
+        <v>-448020</v>
+      </c>
+      <c r="E10" s="34" t="n">
+        <v>-351900</v>
+      </c>
+      <c r="U10" s="44">
         <f>SUM(B10:T10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="30" t="inlineStr">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  SARS excise (launch)</t>
         </is>
       </c>
-      <c r="E11" s="15">
-        <f>-630000*Assumptions!$B$24</f>
-        <v/>
-      </c>
-      <c r="G11" s="15">
-        <f>-495571*Assumptions!$B$24</f>
-        <v/>
-      </c>
-      <c r="U11" s="45">
+      <c r="E11" s="34" t="n">
+        <v>-756000</v>
+      </c>
+      <c r="G11" s="34" t="n">
+        <v>-594685</v>
+      </c>
+      <c r="U11" s="44">
         <f>SUM(B11:T11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="A12" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  Opex (sales, ops, marketing, admin — paid monthly)</t>
         </is>
       </c>
-      <c r="B12" s="21">
+      <c r="B12" s="20">
         <f>'P&amp;L'!B12</f>
         <v/>
       </c>
-      <c r="C12" s="21">
+      <c r="C12" s="20">
         <f>'P&amp;L'!C12</f>
         <v/>
       </c>
-      <c r="D12" s="21">
+      <c r="D12" s="20">
         <f>'P&amp;L'!D12</f>
         <v/>
       </c>
-      <c r="E12" s="21">
+      <c r="E12" s="20">
         <f>'P&amp;L'!E12</f>
         <v/>
       </c>
-      <c r="F12" s="21">
+      <c r="F12" s="20">
         <f>'P&amp;L'!F12</f>
         <v/>
       </c>
-      <c r="G12" s="21">
+      <c r="G12" s="20">
         <f>'P&amp;L'!G12</f>
         <v/>
       </c>
-      <c r="H12" s="21">
+      <c r="H12" s="20">
         <f>'P&amp;L'!H12</f>
         <v/>
       </c>
-      <c r="I12" s="21">
+      <c r="I12" s="20">
         <f>'P&amp;L'!I12</f>
         <v/>
       </c>
-      <c r="J12" s="21">
+      <c r="J12" s="20">
         <f>'P&amp;L'!J12</f>
         <v/>
       </c>
-      <c r="K12" s="21">
+      <c r="K12" s="20">
         <f>'P&amp;L'!K12</f>
         <v/>
       </c>
-      <c r="L12" s="21">
+      <c r="L12" s="20">
         <f>'P&amp;L'!L12</f>
         <v/>
       </c>
-      <c r="M12" s="21">
+      <c r="M12" s="20">
         <f>'P&amp;L'!M12</f>
         <v/>
       </c>
-      <c r="N12" s="21">
+      <c r="N12" s="20">
         <f>'P&amp;L'!N12</f>
         <v/>
       </c>
-      <c r="O12" s="21">
+      <c r="O12" s="20">
         <f>'P&amp;L'!O12</f>
         <v/>
       </c>
-      <c r="P12" s="21">
+      <c r="P12" s="20">
         <f>'P&amp;L'!P12</f>
         <v/>
       </c>
-      <c r="Q12" s="21">
+      <c r="Q12" s="20">
         <f>'P&amp;L'!Q12</f>
         <v/>
       </c>
-      <c r="R12" s="21">
+      <c r="R12" s="20">
         <f>'P&amp;L'!R12</f>
         <v/>
       </c>
-      <c r="S12" s="21">
+      <c r="S12" s="20">
         <f>'P&amp;L'!S12</f>
         <v/>
       </c>
-      <c r="T12" s="21">
+      <c r="T12" s="20">
         <f>'P&amp;L'!T12</f>
         <v/>
       </c>
-      <c r="U12" s="45">
+      <c r="U12" s="44">
         <f>SUM(B12:T12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="30" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  Bottles net contribution (GM, cash in month)</t>
         </is>
       </c>
-      <c r="B13" s="21">
+      <c r="B13" s="20">
         <f>'P&amp;L'!B6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="C13" s="21">
+      <c r="C13" s="20">
         <f>'P&amp;L'!C6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="D13" s="21">
+      <c r="D13" s="20">
         <f>'P&amp;L'!D6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="E13" s="21">
+      <c r="E13" s="20">
         <f>'P&amp;L'!E6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="F13" s="21">
+      <c r="F13" s="20">
         <f>'P&amp;L'!F6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="G13" s="21">
+      <c r="G13" s="20">
         <f>'P&amp;L'!G6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="H13" s="21">
+      <c r="H13" s="20">
         <f>'P&amp;L'!H6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="I13" s="21">
+      <c r="I13" s="20">
         <f>'P&amp;L'!I6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="J13" s="21">
+      <c r="J13" s="20">
         <f>'P&amp;L'!J6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="K13" s="21">
+      <c r="K13" s="20">
         <f>'P&amp;L'!K6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="L13" s="21">
+      <c r="L13" s="20">
         <f>'P&amp;L'!L6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="M13" s="21">
+      <c r="M13" s="20">
         <f>'P&amp;L'!M6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="N13" s="21">
+      <c r="N13" s="20">
         <f>'P&amp;L'!N6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="O13" s="21">
+      <c r="O13" s="20">
         <f>'P&amp;L'!O6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="P13" s="21">
+      <c r="P13" s="20">
         <f>'P&amp;L'!P6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="Q13" s="21">
+      <c r="Q13" s="20">
         <f>'P&amp;L'!Q6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="R13" s="21">
+      <c r="R13" s="20">
         <f>'P&amp;L'!R6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="S13" s="21">
+      <c r="S13" s="20">
         <f>'P&amp;L'!S6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="T13" s="21">
+      <c r="T13" s="20">
         <f>'P&amp;L'!T6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="U13" s="45">
+      <c r="U13" s="44">
         <f>SUM(B13:T13)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="30" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  2027 recurring can COGS</t>
         </is>
       </c>
-      <c r="I14" s="15">
-        <f>-'P&amp;L'!I5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="J14" s="15">
-        <f>-'P&amp;L'!J5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="K14" s="15">
-        <f>-'P&amp;L'!K5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="L14" s="15">
-        <f>-'P&amp;L'!L5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="M14" s="15">
-        <f>-'P&amp;L'!M5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="N14" s="15">
-        <f>-'P&amp;L'!N5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="O14" s="15">
-        <f>-'P&amp;L'!O5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="P14" s="15">
-        <f>-'P&amp;L'!P5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="Q14" s="15">
-        <f>-'P&amp;L'!Q5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="R14" s="15">
-        <f>-'P&amp;L'!R5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="S14" s="15">
-        <f>-'P&amp;L'!S5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="T14" s="15">
-        <f>-'P&amp;L'!T5*Assumptions!$B$21</f>
-        <v/>
-      </c>
-      <c r="U14" s="45">
+      <c r="I14" s="14">
+        <f>-'P&amp;L'!I5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="J14" s="14">
+        <f>-'P&amp;L'!J5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="K14" s="14">
+        <f>-'P&amp;L'!K5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="L14" s="14">
+        <f>-'P&amp;L'!L5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="M14" s="14">
+        <f>-'P&amp;L'!M5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="N14" s="14">
+        <f>-'P&amp;L'!N5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="O14" s="14">
+        <f>-'P&amp;L'!O5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="P14" s="14">
+        <f>-'P&amp;L'!P5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="Q14" s="14">
+        <f>-'P&amp;L'!Q5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="R14" s="14">
+        <f>-'P&amp;L'!R5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="S14" s="14">
+        <f>-'P&amp;L'!S5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="T14" s="14">
+        <f>-'P&amp;L'!T5*Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="U14" s="44">
         <f>SUM(B14:T14)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="33" t="inlineStr">
+      <c r="A15" s="32" t="inlineStr">
         <is>
           <t>Net monthly cashflow</t>
         </is>
       </c>
-      <c r="B15" s="16">
+      <c r="B15" s="15">
         <f>SUM(B4:B14)</f>
         <v/>
       </c>
-      <c r="C15" s="16">
+      <c r="C15" s="15">
         <f>SUM(C4:C14)</f>
         <v/>
       </c>
-      <c r="D15" s="16">
+      <c r="D15" s="15">
         <f>SUM(D4:D14)</f>
         <v/>
       </c>
-      <c r="E15" s="16">
+      <c r="E15" s="15">
         <f>SUM(E4:E14)</f>
         <v/>
       </c>
-      <c r="F15" s="16">
+      <c r="F15" s="15">
         <f>SUM(F4:F14)</f>
         <v/>
       </c>
-      <c r="G15" s="16">
+      <c r="G15" s="15">
         <f>SUM(G4:G14)</f>
         <v/>
       </c>
-      <c r="H15" s="16">
+      <c r="H15" s="15">
         <f>SUM(H4:H14)</f>
         <v/>
       </c>
-      <c r="I15" s="16">
+      <c r="I15" s="15">
         <f>SUM(I4:I14)</f>
         <v/>
       </c>
-      <c r="J15" s="16">
+      <c r="J15" s="15">
         <f>SUM(J4:J14)</f>
         <v/>
       </c>
-      <c r="K15" s="16">
+      <c r="K15" s="15">
         <f>SUM(K4:K14)</f>
         <v/>
       </c>
-      <c r="L15" s="16">
+      <c r="L15" s="15">
         <f>SUM(L4:L14)</f>
         <v/>
       </c>
-      <c r="M15" s="16">
+      <c r="M15" s="15">
         <f>SUM(M4:M14)</f>
         <v/>
       </c>
-      <c r="N15" s="16">
+      <c r="N15" s="15">
         <f>SUM(N4:N14)</f>
         <v/>
       </c>
-      <c r="O15" s="16">
+      <c r="O15" s="15">
         <f>SUM(O4:O14)</f>
         <v/>
       </c>
-      <c r="P15" s="16">
+      <c r="P15" s="15">
         <f>SUM(P4:P14)</f>
         <v/>
       </c>
-      <c r="Q15" s="16">
+      <c r="Q15" s="15">
         <f>SUM(Q4:Q14)</f>
         <v/>
       </c>
-      <c r="R15" s="16">
+      <c r="R15" s="15">
         <f>SUM(R4:R14)</f>
         <v/>
       </c>
-      <c r="S15" s="16">
+      <c r="S15" s="15">
         <f>SUM(S4:S14)</f>
         <v/>
       </c>
-      <c r="T15" s="16">
+      <c r="T15" s="15">
         <f>SUM(T4:T14)</f>
         <v/>
       </c>
-      <c r="U15" s="45">
+      <c r="U15" s="44">
         <f>SUM(B15:T15)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="33" t="inlineStr">
+      <c r="A16" s="32" t="inlineStr">
         <is>
           <t>Cumulative cash position</t>
         </is>
       </c>
-      <c r="B16" s="16">
+      <c r="B16" s="15">
         <f>B15</f>
         <v/>
       </c>
-      <c r="C16" s="16">
+      <c r="C16" s="15">
         <f>B16+C15</f>
         <v/>
       </c>
-      <c r="D16" s="16">
+      <c r="D16" s="15">
         <f>C16+D15</f>
         <v/>
       </c>
-      <c r="E16" s="16">
+      <c r="E16" s="15">
         <f>D16+E15</f>
         <v/>
       </c>
-      <c r="F16" s="16">
+      <c r="F16" s="15">
         <f>E16+F15</f>
         <v/>
       </c>
-      <c r="G16" s="16">
+      <c r="G16" s="15">
         <f>F16+G15</f>
         <v/>
       </c>
-      <c r="H16" s="16">
+      <c r="H16" s="15">
         <f>G16+H15</f>
         <v/>
       </c>
-      <c r="I16" s="16">
+      <c r="I16" s="15">
         <f>H16+I15</f>
         <v/>
       </c>
-      <c r="J16" s="16">
+      <c r="J16" s="15">
         <f>I16+J15</f>
         <v/>
       </c>
-      <c r="K16" s="16">
+      <c r="K16" s="15">
         <f>J16+K15</f>
         <v/>
       </c>
-      <c r="L16" s="16">
+      <c r="L16" s="15">
         <f>K16+L15</f>
         <v/>
       </c>
-      <c r="M16" s="16">
+      <c r="M16" s="15">
         <f>L16+M15</f>
         <v/>
       </c>
-      <c r="N16" s="16">
+      <c r="N16" s="15">
         <f>M16+N15</f>
         <v/>
       </c>
-      <c r="O16" s="16">
+      <c r="O16" s="15">
         <f>N16+O15</f>
         <v/>
       </c>
-      <c r="P16" s="16">
+      <c r="P16" s="15">
         <f>O16+P15</f>
         <v/>
       </c>
-      <c r="Q16" s="16">
+      <c r="Q16" s="15">
         <f>P16+Q15</f>
         <v/>
       </c>
-      <c r="R16" s="16">
+      <c r="R16" s="15">
         <f>Q16+R15</f>
         <v/>
       </c>
-      <c r="S16" s="16">
+      <c r="S16" s="15">
         <f>R16+S15</f>
         <v/>
       </c>
-      <c r="T16" s="16">
+      <c r="T16" s="15">
         <f>S16+T15</f>
         <v/>
       </c>
@@ -3214,7 +3232,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Note: 2026 launch costs are the project model's quoted cash costs, scaled by the store factor (Assumptions!B24).</t>
+          <t>2026 launch costs per supplier quotes for the 360-store opening order and October restock.</t>
         </is>
       </c>
     </row>
@@ -3248,269 +3266,269 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>VALUATION — Doña Fuego brand entity (cans + bottles)</t>
         </is>
       </c>
-      <c r="B1" s="27" t="n"/>
-      <c r="C1" s="27" t="n"/>
-      <c r="D1" s="27" t="n"/>
-      <c r="E1" s="27" t="n"/>
+      <c r="B1" s="26" t="n"/>
+      <c r="C1" s="26" t="n"/>
+      <c r="D1" s="26" t="n"/>
+      <c r="E1" s="26" t="n"/>
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="28" t="inlineStr">
+      <c r="A3" s="27" t="inlineStr">
         <is>
           <t>Key metrics (linked to P&amp;L)</t>
         </is>
       </c>
-      <c r="B3" s="29" t="n"/>
-      <c r="C3" s="29" t="n"/>
-      <c r="D3" s="29" t="n"/>
+      <c r="B3" s="28" t="n"/>
+      <c r="C3" s="28" t="n"/>
+      <c r="D3" s="28" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="30" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>2026 (Jun–Dec) revenue</t>
         </is>
       </c>
-      <c r="B4" s="21">
+      <c r="B4" s="20">
         <f>SUM('P&amp;L'!B7:H7)</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>2026 (Jun–Dec) EBITDA</t>
         </is>
       </c>
-      <c r="B5" s="21">
+      <c r="B5" s="20">
         <f>SUM('P&amp;L'!B13:H13)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="30" t="inlineStr">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>2027 revenue</t>
         </is>
       </c>
-      <c r="B6" s="21">
+      <c r="B6" s="20">
         <f>SUM('P&amp;L'!I7:T7)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="30" t="inlineStr">
+      <c r="A7" s="29" t="inlineStr">
         <is>
           <t>2027 EBITDA</t>
         </is>
       </c>
-      <c r="B7" s="21">
+      <c r="B7" s="20">
         <f>SUM('P&amp;L'!I13:T13)</f>
         <v/>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
-      <c r="A9" s="28" t="inlineStr">
+      <c r="A9" s="27" t="inlineStr">
         <is>
           <t>Method 1: EV/EBITDA on 2027 EBITDA</t>
         </is>
       </c>
-      <c r="B9" s="29" t="inlineStr">
+      <c r="B9" s="28" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="C9" s="29" t="inlineStr">
+      <c r="C9" s="28" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="D9" s="29" t="inlineStr">
+      <c r="D9" s="28" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="30" t="inlineStr">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t>Multiple</t>
         </is>
       </c>
-      <c r="B10" s="47" t="n">
+      <c r="B10" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="C10" s="47" t="n">
+      <c r="C10" s="46" t="n">
         <v>9</v>
       </c>
-      <c r="D10" s="47" t="n">
+      <c r="D10" s="46" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="30" t="inlineStr">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="B11" s="15">
+      <c r="B11" s="14">
         <f>$B$7*B10</f>
         <v/>
       </c>
-      <c r="C11" s="15">
+      <c r="C11" s="14">
         <f>$B$7*C10</f>
         <v/>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="14">
         <f>$B$7*D10</f>
         <v/>
       </c>
     </row>
     <row r="12"/>
     <row r="13">
-      <c r="A13" s="28" t="inlineStr">
+      <c r="A13" s="27" t="inlineStr">
         <is>
           <t>Method 2: EV/Revenue on 2027 revenue</t>
         </is>
       </c>
-      <c r="B13" s="29" t="n"/>
-      <c r="C13" s="29" t="n"/>
-      <c r="D13" s="29" t="n"/>
+      <c r="B13" s="28" t="n"/>
+      <c r="C13" s="28" t="n"/>
+      <c r="D13" s="28" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="30" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>Multiple</t>
         </is>
       </c>
-      <c r="B14" s="47" t="n">
+      <c r="B14" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="C14" s="47" t="n">
+      <c r="C14" s="46" t="n">
         <v>1.5</v>
       </c>
-      <c r="D14" s="47" t="n">
+      <c r="D14" s="46" t="n">
         <v>2.5</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="30" t="inlineStr">
+      <c r="A15" s="29" t="inlineStr">
         <is>
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="B15" s="15">
+      <c r="B15" s="14">
         <f>$B$6*B14</f>
         <v/>
       </c>
-      <c r="C15" s="15">
+      <c r="C15" s="14">
         <f>$B$6*C14</f>
         <v/>
       </c>
-      <c r="D15" s="15">
+      <c r="D15" s="14">
         <f>$B$6*D14</f>
         <v/>
       </c>
     </row>
     <row r="16"/>
     <row r="17">
-      <c r="A17" s="28" t="inlineStr">
+      <c r="A17" s="27" t="inlineStr">
         <is>
           <t>Method 3: simplified DCF (EBITDA as cash proxy)</t>
         </is>
       </c>
-      <c r="B17" s="29" t="n"/>
-      <c r="C17" s="29" t="n"/>
-      <c r="D17" s="29" t="n"/>
+      <c r="B17" s="28" t="n"/>
+      <c r="C17" s="28" t="n"/>
+      <c r="D17" s="28" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="30" t="inlineStr">
+      <c r="A18" s="29" t="inlineStr">
         <is>
           <t>WACC</t>
         </is>
       </c>
-      <c r="B18" s="37" t="n">
+      <c r="B18" s="36" t="n">
         <v>0.22</v>
       </c>
-      <c r="C18" s="37" t="n">
+      <c r="C18" s="36" t="n">
         <v>0.18</v>
       </c>
-      <c r="D18" s="37" t="n">
+      <c r="D18" s="36" t="n">
         <v>0.15</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="30" t="inlineStr">
+      <c r="A19" s="29" t="inlineStr">
         <is>
           <t>Exit multiple (2027 EBITDA)</t>
         </is>
       </c>
-      <c r="B19" s="47" t="n">
+      <c r="B19" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="C19" s="47" t="n">
+      <c r="C19" s="46" t="n">
         <v>8</v>
       </c>
-      <c r="D19" s="47" t="n">
+      <c r="D19" s="46" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="30" t="inlineStr">
+      <c r="A20" s="29" t="inlineStr">
         <is>
           <t>Enterprise value (DCF)</t>
         </is>
       </c>
-      <c r="B20" s="15">
+      <c r="B20" s="14">
         <f>$B$5/(1+B18)^0.25+$B$7/(1+B18)+$B$7*B19/(1+B18)^1.5</f>
         <v/>
       </c>
-      <c r="C20" s="15">
+      <c r="C20" s="14">
         <f>$B$5/(1+C18)^0.25+$B$7/(1+C18)+$B$7*C19/(1+C18)^1.5</f>
         <v/>
       </c>
-      <c r="D20" s="15">
+      <c r="D20" s="14">
         <f>$B$5/(1+D18)^0.25+$B$7/(1+D18)+$B$7*D19/(1+D18)^1.5</f>
         <v/>
       </c>
     </row>
     <row r="21"/>
     <row r="22">
-      <c r="A22" s="33" t="inlineStr">
+      <c r="A22" s="32" t="inlineStr">
         <is>
           <t>Blended enterprise value (avg of methods)</t>
         </is>
       </c>
-      <c r="B22" s="40">
+      <c r="B22" s="39">
         <f>AVERAGE(B11,B15,B20)</f>
         <v/>
       </c>
-      <c r="C22" s="40">
+      <c r="C22" s="39">
         <f>AVERAGE(C11,C15,C20)</f>
         <v/>
       </c>
-      <c r="D22" s="40">
+      <c r="D22" s="39">
         <f>AVERAGE(D11,D15,D20)</f>
         <v/>
       </c>
     </row>
     <row r="23"/>
     <row r="24">
-      <c r="A24" s="39" t="inlineStr">
+      <c r="A24" s="38" t="inlineStr">
         <is>
           <t>Valuation guide for the raise</t>
         </is>
       </c>
-      <c r="B24" s="48" t="n">
+      <c r="B24" s="47" t="n">
         <v>15000000</v>
       </c>
-      <c r="C24" s="27" t="n"/>
-      <c r="D24" s="27" t="n"/>
+      <c r="C24" s="26" t="n"/>
+      <c r="D24" s="26" t="n"/>
       <c r="E24" s="2" t="inlineStr">
         <is>
           <t>With bottles modelled off three years of actuals, the ~R15m guide equals the blended LOW case; better-than-flat reorders, new retailers and export remain outside the model.</t>
@@ -3545,142 +3563,142 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>SUMMARY — Doña Fuego Brand Pro Forma</t>
         </is>
       </c>
-      <c r="B1" s="27" t="n"/>
+      <c r="B1" s="26" t="n"/>
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="49" t="inlineStr">
+      <c r="A3" s="48" t="inlineStr">
         <is>
           <t>Checkers listing</t>
         </is>
       </c>
-      <c r="B3" s="24">
+      <c r="B3" s="23">
         <f>Assumptions!B4&amp;" stores + Sixty60, Aug 2026"</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="49" t="inlineStr">
+      <c r="A4" s="48" t="inlineStr">
         <is>
           <t>Opening order (initial fill revenue)</t>
         </is>
       </c>
-      <c r="B4" s="21">
+      <c r="B4" s="20">
         <f>'P&amp;L'!D5</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="49" t="inlineStr">
+      <c r="A5" s="48" t="inlineStr">
         <is>
           <t>Bottle revenue (Jun 26 – Dec 27)</t>
         </is>
       </c>
-      <c r="B5" s="21">
+      <c r="B5" s="20">
         <f>'P&amp;L'!U6</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="39" t="inlineStr">
+      <c r="A6" s="38" t="inlineStr">
         <is>
           <t>Total revenue, cans + bottles (Jun 26 – Dec 27)</t>
         </is>
       </c>
-      <c r="B6" s="45">
+      <c r="B6" s="44">
         <f>'P&amp;L'!U7</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="39" t="inlineStr">
+      <c r="A7" s="38" t="inlineStr">
         <is>
           <t>Total EBITDA (Jun 26 – Dec 27)</t>
         </is>
       </c>
-      <c r="B7" s="45">
+      <c r="B7" s="44">
         <f>'P&amp;L'!U13</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="49" t="inlineStr">
+      <c r="A8" s="48" t="inlineStr">
         <is>
           <t>EBITDA margin</t>
         </is>
       </c>
-      <c r="B8" s="25">
+      <c r="B8" s="24">
         <f>'P&amp;L'!U14</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="29" t="inlineStr">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>Peak funding need</t>
         </is>
       </c>
-      <c r="B9" s="45">
+      <c r="B9" s="44">
         <f>MIN(Cashflow!B16:T16)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="49" t="inlineStr">
+      <c r="A10" s="48" t="inlineStr">
         <is>
           <t>Ending cash (Dec 27)</t>
         </is>
       </c>
-      <c r="B10" s="21">
+      <c r="B10" s="20">
         <f>Cashflow!T16</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="49" t="inlineStr">
+      <c r="A11" s="48" t="inlineStr">
         <is>
           <t>Blended valuation — low</t>
         </is>
       </c>
-      <c r="B11" s="21">
+      <c r="B11" s="20">
         <f>Valuation!B22</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="49" t="inlineStr">
+      <c r="A12" s="48" t="inlineStr">
         <is>
           <t>Blended valuation — base</t>
         </is>
       </c>
-      <c r="B12" s="21">
+      <c r="B12" s="20">
         <f>Valuation!C22</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="49" t="inlineStr">
+      <c r="A13" s="48" t="inlineStr">
         <is>
           <t>Blended valuation — high</t>
         </is>
       </c>
-      <c r="B13" s="21">
+      <c r="B13" s="20">
         <f>Valuation!D22</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="39" t="inlineStr">
+      <c r="A14" s="38" t="inlineStr">
         <is>
           <t>Valuation guide</t>
         </is>
       </c>
-      <c r="B14" s="45">
+      <c r="B14" s="44">
         <f>Valuation!B24</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Bottle gross margin 50% per management
EBITDA R3.27m (19.7%), peak funding R1.60m, end cash R2.57m; blended
valuation R11.0m/R15.8m/R22.4m — the ~R15m guide sits just below the
blended base case. Charts, tables and copy carry the figures.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hyws6xeXfxtGdqZV2paNDe
</commit_message>
<xml_diff>
--- a/site/downloads/Dona-Fuego-Brand-Pro-Forma.xlsx
+++ b/site/downloads/Dona-Fuego-Brand-Pro-Forma.xlsx
@@ -1385,11 +1385,11 @@
         </is>
       </c>
       <c r="B22" s="33" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>PLACEHOLDER matching cans — awaiting bottle cost data from management</t>
+          <t>Per management — direct and retail bottle sales</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adopt Dona's updated inputs; cost of sales improves with scale
- COGS build per management: tequila 18%, wet goods 10%, packaging 13.5%,
  co-pack 12.04%, distribution 4%, excise 18.5% = 76% in Year 1
- Economies of scale: Year 2 cost of sales 66%, Year 3 60% (workbook
  inputs); can gross margin 24% -> 34% -> 40% on the same volumes, with a
  2028 run-rate line on the Valuation sheet
- Opex per management: R105k/month from September 2026 (legal & admin nil)
- Bottles: 2027 growth 30%, gross margin 45%
- Results: revenue R17.12m, EBITDA R3.94m (23.0%), peak funding R1.41m,
  end cash R3.58m; blended valuation R14.0m/R20.0m/R28.0m with the ~R15m
  guide just above the low case
- Unit economics table, P&L, valuation, charts and copy updated

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hyws6xeXfxtGdqZV2paNDe
</commit_message>
<xml_diff>
--- a/site/downloads/Dona-Fuego-Brand-Pro-Forma.xlsx
+++ b/site/downloads/Dona-Fuego-Brand-Pro-Forma.xlsx
@@ -144,7 +144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -182,6 +182,7 @@
     <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="12" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -560,7 +561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -781,7 +782,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>Can COGS build (% of revenue)</t>
+          <t>Can COGS build — Year 1 (% of revenue)</t>
         </is>
       </c>
       <c r="B18" s="28" t="n"/>
@@ -790,7 +791,7 @@
     <row r="19">
       <c r="A19" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Tequila (supply agreement)</t>
+          <t xml:space="preserve">  Tequila (allocation)</t>
         </is>
       </c>
       <c r="B19" s="36" t="n">
@@ -805,167 +806,201 @@
     <row r="20">
       <c r="A20" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Packaging (cans, printing, pallets)</t>
+          <t xml:space="preserve">  Additional wet goods</t>
         </is>
       </c>
       <c r="B20" s="36" t="n">
-        <v>0.16</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Co-pack production</t>
+          <t xml:space="preserve">  Packaging (cans, printing, pallets)</t>
         </is>
       </c>
       <c r="B21" s="36" t="n">
-        <v>0.12</v>
+        <v>0.135</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Distribution (FAL)</t>
+          <t xml:space="preserve">  Co-pack production</t>
         </is>
       </c>
       <c r="B22" s="36" t="n">
-        <v>0.04</v>
+        <v>0.1204</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SARS Excise</t>
+          <t xml:space="preserve">  Distribution (Chep + provlog)</t>
         </is>
       </c>
       <c r="B23" s="36" t="n">
-        <v>0.2</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="32" t="inlineStr">
         <is>
-          <t>Total can COGS ratio</t>
-        </is>
-      </c>
-      <c r="B24" s="12">
-        <f>SUM(B19:B23)</f>
-        <v/>
+          <t xml:space="preserve">  SARS Excise</t>
+        </is>
+      </c>
+      <c r="B24" s="36" t="n">
+        <v>0.185</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>Operating costs — sales, operations &amp; distribution (monthly)</t>
-        </is>
-      </c>
-      <c r="B25" s="28" t="n"/>
+          <t>Year 1 can COGS ratio</t>
+        </is>
+      </c>
+      <c r="B25" s="37">
+        <f>SUM(B19:B24)</f>
+        <v/>
+      </c>
       <c r="C25" s="28" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="29" t="inlineStr">
         <is>
-          <t>Legal &amp; admin</t>
-        </is>
-      </c>
-      <c r="B26" s="34" t="n">
-        <v>10000</v>
+          <t>Year 2 can COGS ratio</t>
+        </is>
+      </c>
+      <c r="B26" s="33" t="n">
+        <v>0.66</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>From June 2026</t>
+          <t>Economies of scale: 10 points off Year 1 on volume-based input and co-pack pricing</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="29" t="inlineStr">
         <is>
-          <t>Sales &amp; key accounts (1 FTE)</t>
-        </is>
-      </c>
-      <c r="B27" s="37" t="n">
-        <v>40000</v>
+          <t>Year 3 can COGS ratio</t>
+        </is>
+      </c>
+      <c r="B27" s="33" t="n">
+        <v>0.6</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>MANAGEMENT ESTIMATE, from July 2026 — supports founder-led sales</t>
+          <t>A further 6 points at scale; applied to the 2028 run-rate</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="29" t="inlineStr">
         <is>
-          <t>Operations &amp; merchandising coordinator</t>
-        </is>
-      </c>
-      <c r="B28" s="37" t="n">
-        <v>18000</v>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>MANAGEMENT ESTIMATE, from July 2026 — shared resource with distillery</t>
+          <t>Operating costs — sales, operations &amp; distribution (monthly)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="29" t="inlineStr">
         <is>
-          <t>Trade marketing &amp; promotions</t>
-        </is>
-      </c>
-      <c r="B29" s="37" t="n">
-        <v>25000</v>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>MANAGEMENT ESTIMATE, from August 2026 — in-store support</t>
-        </is>
+          <t>Legal &amp; admin</t>
+        </is>
+      </c>
+      <c r="B29" s="34" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="29" t="inlineStr">
         <is>
-          <t>Brand marketing</t>
-        </is>
-      </c>
-      <c r="B30" s="37" t="n">
-        <v>25000</v>
+          <t>Sales &amp; key accounts (1 FTE)</t>
+        </is>
+      </c>
+      <c r="B30" s="38" t="n">
+        <v>40000</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>MANAGEMENT ESTIMATE, from August 2026 — always-on consumer brand building</t>
+          <t>From September 2026 — supports founder-led sales</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="29" t="inlineStr">
         <is>
-          <t>Warehousing &amp; insurance</t>
-        </is>
-      </c>
-      <c r="B31" s="37" t="n">
-        <v>12000</v>
+          <t>Operations &amp; merchandising coordinator</t>
+        </is>
+      </c>
+      <c r="B31" s="38" t="n">
+        <v>15000</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>MANAGEMENT ESTIMATE, from August 2026</t>
+          <t>From September 2026 — shared resource with distillery</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="32" t="inlineStr">
         <is>
+          <t>Trade marketing &amp; promotions</t>
+        </is>
+      </c>
+      <c r="B32" s="38" t="n">
+        <v>25000</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>From September 2026 — in-store support</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Brand marketing</t>
+        </is>
+      </c>
+      <c r="B33" s="38" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>From September 2026 — always-on consumer brand building</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Warehousing &amp; insurance</t>
+        </is>
+      </c>
+      <c r="B34" s="38" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>From September 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
           <t>Steady-state opex total</t>
         </is>
       </c>
-      <c r="B32" s="14">
-        <f>SUM(B26:B31)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33"/>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="B35" s="14">
+        <f>SUM(B29:B34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36"/>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>Legend: blue = input (edit these) · black = formula · green = link to another sheet · yellow = key assumptions to sense-check</t>
         </is>
@@ -1016,33 +1051,33 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="38" t="inlineStr">
+      <c r="A3" s="39" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B3" s="38" t="inlineStr">
+      <c r="B3" s="39" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="C3" s="38" t="inlineStr">
+      <c r="C3" s="39" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D3" s="38" t="inlineStr">
+      <c r="D3" s="39" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="E3" s="38" t="inlineStr">
+      <c r="E3" s="39" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr"/>
-      <c r="G3" s="38" t="inlineStr">
+      <c r="G3" s="39" t="inlineStr">
         <is>
           <t>2027 (proj)</t>
         </is>
@@ -1305,23 +1340,23 @@
           <t>Annual total</t>
         </is>
       </c>
-      <c r="B16" s="39">
+      <c r="B16" s="40">
         <f>SUM(B4:B15)</f>
         <v/>
       </c>
-      <c r="C16" s="39">
+      <c r="C16" s="40">
         <f>SUM(C4:C15)</f>
         <v/>
       </c>
-      <c r="D16" s="39">
+      <c r="D16" s="40">
         <f>SUM(D4:D15)</f>
         <v/>
       </c>
-      <c r="E16" s="39">
+      <c r="E16" s="40">
         <f>SUM(E4:E15)</f>
         <v/>
       </c>
-      <c r="G16" s="39">
+      <c r="G16" s="40">
         <f>SUM(G4:G15)</f>
         <v/>
       </c>
@@ -1359,11 +1394,11 @@
         </is>
       </c>
       <c r="B20" s="33" t="n">
-        <v>0.05</v>
+        <v>0.3</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>CONSERVATIVE vs +89% (2025) and +4.4% YTD (2026)</t>
+          <t>Per management; against +89% actual growth in 2025</t>
         </is>
       </c>
     </row>
@@ -1385,7 +1420,7 @@
         </is>
       </c>
       <c r="B22" s="33" t="n">
-        <v>0.5</v>
+        <v>0.45</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
@@ -1467,69 +1502,69 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="38" t="inlineStr">
+      <c r="A3" s="39" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B3" s="40" t="n">
+      <c r="B3" s="41" t="n">
         <v>46174</v>
       </c>
-      <c r="C3" s="40" t="n">
+      <c r="C3" s="41" t="n">
         <v>46204</v>
       </c>
-      <c r="D3" s="40" t="n">
+      <c r="D3" s="41" t="n">
         <v>46235</v>
       </c>
-      <c r="E3" s="40" t="n">
+      <c r="E3" s="41" t="n">
         <v>46266</v>
       </c>
-      <c r="F3" s="40" t="n">
+      <c r="F3" s="41" t="n">
         <v>46296</v>
       </c>
-      <c r="G3" s="40" t="n">
+      <c r="G3" s="41" t="n">
         <v>46327</v>
       </c>
-      <c r="H3" s="40" t="n">
+      <c r="H3" s="41" t="n">
         <v>46357</v>
       </c>
-      <c r="I3" s="40" t="n">
+      <c r="I3" s="41" t="n">
         <v>46388</v>
       </c>
-      <c r="J3" s="40" t="n">
+      <c r="J3" s="41" t="n">
         <v>46419</v>
       </c>
-      <c r="K3" s="40" t="n">
+      <c r="K3" s="41" t="n">
         <v>46447</v>
       </c>
-      <c r="L3" s="40" t="n">
+      <c r="L3" s="41" t="n">
         <v>46478</v>
       </c>
-      <c r="M3" s="40" t="n">
+      <c r="M3" s="41" t="n">
         <v>46508</v>
       </c>
-      <c r="N3" s="40" t="n">
+      <c r="N3" s="41" t="n">
         <v>46539</v>
       </c>
-      <c r="O3" s="40" t="n">
+      <c r="O3" s="41" t="n">
         <v>46569</v>
       </c>
-      <c r="P3" s="40" t="n">
+      <c r="P3" s="41" t="n">
         <v>46600</v>
       </c>
-      <c r="Q3" s="40" t="n">
+      <c r="Q3" s="41" t="n">
         <v>46631</v>
       </c>
-      <c r="R3" s="40" t="n">
+      <c r="R3" s="41" t="n">
         <v>46661</v>
       </c>
-      <c r="S3" s="40" t="n">
+      <c r="S3" s="41" t="n">
         <v>46692</v>
       </c>
-      <c r="T3" s="40" t="n">
+      <c r="T3" s="41" t="n">
         <v>46722</v>
       </c>
-      <c r="U3" s="38" t="inlineStr">
+      <c r="U3" s="39" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -1541,80 +1576,80 @@
           <t>Cases delivered (cans)</t>
         </is>
       </c>
-      <c r="B4" s="41" t="n">
+      <c r="B4" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="C4" s="41" t="n">
+      <c r="C4" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="42">
+      <c r="D4" s="43">
         <f>Assumptions!B7</f>
         <v/>
       </c>
-      <c r="E4" s="41" t="n">
+      <c r="E4" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="42">
+      <c r="F4" s="43">
         <f>Assumptions!B8</f>
         <v/>
       </c>
-      <c r="G4" s="42">
+      <c r="G4" s="43">
         <f>IF(OR(MONTH(G3)&gt;=10,MONTH(G3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
         <v/>
       </c>
-      <c r="H4" s="42">
+      <c r="H4" s="43">
         <f>IF(OR(MONTH(H3)&gt;=10,MONTH(H3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
         <v/>
       </c>
-      <c r="I4" s="42">
+      <c r="I4" s="43">
         <f>IF(OR(MONTH(I3)&gt;=10,MONTH(I3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
         <v/>
       </c>
-      <c r="J4" s="42">
+      <c r="J4" s="43">
         <f>IF(OR(MONTH(J3)&gt;=10,MONTH(J3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
         <v/>
       </c>
-      <c r="K4" s="42">
+      <c r="K4" s="43">
         <f>IF(OR(MONTH(K3)&gt;=10,MONTH(K3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
         <v/>
       </c>
-      <c r="L4" s="42">
+      <c r="L4" s="43">
         <f>IF(OR(MONTH(L3)&gt;=10,MONTH(L3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
         <v/>
       </c>
-      <c r="M4" s="42">
+      <c r="M4" s="43">
         <f>IF(OR(MONTH(M3)&gt;=10,MONTH(M3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
         <v/>
       </c>
-      <c r="N4" s="42">
+      <c r="N4" s="43">
         <f>IF(OR(MONTH(N3)&gt;=10,MONTH(N3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
         <v/>
       </c>
-      <c r="O4" s="42">
+      <c r="O4" s="43">
         <f>IF(OR(MONTH(O3)&gt;=10,MONTH(O3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
         <v/>
       </c>
-      <c r="P4" s="42">
+      <c r="P4" s="43">
         <f>IF(OR(MONTH(P3)&gt;=10,MONTH(P3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
         <v/>
       </c>
-      <c r="Q4" s="42">
+      <c r="Q4" s="43">
         <f>IF(OR(MONTH(Q3)&gt;=10,MONTH(Q3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
         <v/>
       </c>
-      <c r="R4" s="42">
+      <c r="R4" s="43">
         <f>IF(OR(MONTH(R3)&gt;=10,MONTH(R3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
         <v/>
       </c>
-      <c r="S4" s="42">
+      <c r="S4" s="43">
         <f>IF(OR(MONTH(S3)&gt;=10,MONTH(S3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
         <v/>
       </c>
-      <c r="T4" s="42">
+      <c r="T4" s="43">
         <f>IF(OR(MONTH(T3)&gt;=10,MONTH(T3)&lt;=3),Assumptions!$B$14,Assumptions!$B$15)</f>
         <v/>
       </c>
-      <c r="U4" s="43">
+      <c r="U4" s="44">
         <f>SUM(B4:T4)</f>
         <v/>
       </c>
@@ -1701,7 +1736,7 @@
         <f>T4*Assumptions!$B$16</f>
         <v/>
       </c>
-      <c r="U5" s="44">
+      <c r="U5" s="45">
         <f>SUM(B5:T5)</f>
         <v/>
       </c>
@@ -1788,7 +1823,7 @@
         <f>Bottles!G15</f>
         <v/>
       </c>
-      <c r="U6" s="44">
+      <c r="U6" s="45">
         <f>SUM(B6:T6)</f>
         <v/>
       </c>
@@ -1875,7 +1910,7 @@
         <f>T5+T6</f>
         <v/>
       </c>
-      <c r="U7" s="44">
+      <c r="U7" s="45">
         <f>SUM(B7:T7)</f>
         <v/>
       </c>
@@ -1887,82 +1922,82 @@
         </is>
       </c>
       <c r="B8" s="14">
-        <f>-B5*Assumptions!$B$24</f>
+        <f>-B5*IF(YEAR(B3)=2026,Assumptions!$B$25,Assumptions!$B$26)</f>
         <v/>
       </c>
       <c r="C8" s="14">
-        <f>-C5*Assumptions!$B$24</f>
+        <f>-C5*IF(YEAR(C3)=2026,Assumptions!$B$25,Assumptions!$B$26)</f>
         <v/>
       </c>
       <c r="D8" s="14">
-        <f>-D5*Assumptions!$B$24</f>
+        <f>-D5*IF(YEAR(D3)=2026,Assumptions!$B$25,Assumptions!$B$26)</f>
         <v/>
       </c>
       <c r="E8" s="14">
-        <f>-E5*Assumptions!$B$24</f>
+        <f>-E5*IF(YEAR(E3)=2026,Assumptions!$B$25,Assumptions!$B$26)</f>
         <v/>
       </c>
       <c r="F8" s="14">
-        <f>-F5*Assumptions!$B$24</f>
+        <f>-F5*IF(YEAR(F3)=2026,Assumptions!$B$25,Assumptions!$B$26)</f>
         <v/>
       </c>
       <c r="G8" s="14">
-        <f>-G5*Assumptions!$B$24</f>
+        <f>-G5*IF(YEAR(G3)=2026,Assumptions!$B$25,Assumptions!$B$26)</f>
         <v/>
       </c>
       <c r="H8" s="14">
-        <f>-H5*Assumptions!$B$24</f>
+        <f>-H5*IF(YEAR(H3)=2026,Assumptions!$B$25,Assumptions!$B$26)</f>
         <v/>
       </c>
       <c r="I8" s="14">
-        <f>-I5*Assumptions!$B$24</f>
+        <f>-I5*IF(YEAR(I3)=2026,Assumptions!$B$25,Assumptions!$B$26)</f>
         <v/>
       </c>
       <c r="J8" s="14">
-        <f>-J5*Assumptions!$B$24</f>
+        <f>-J5*IF(YEAR(J3)=2026,Assumptions!$B$25,Assumptions!$B$26)</f>
         <v/>
       </c>
       <c r="K8" s="14">
-        <f>-K5*Assumptions!$B$24</f>
+        <f>-K5*IF(YEAR(K3)=2026,Assumptions!$B$25,Assumptions!$B$26)</f>
         <v/>
       </c>
       <c r="L8" s="14">
-        <f>-L5*Assumptions!$B$24</f>
+        <f>-L5*IF(YEAR(L3)=2026,Assumptions!$B$25,Assumptions!$B$26)</f>
         <v/>
       </c>
       <c r="M8" s="14">
-        <f>-M5*Assumptions!$B$24</f>
+        <f>-M5*IF(YEAR(M3)=2026,Assumptions!$B$25,Assumptions!$B$26)</f>
         <v/>
       </c>
       <c r="N8" s="14">
-        <f>-N5*Assumptions!$B$24</f>
+        <f>-N5*IF(YEAR(N3)=2026,Assumptions!$B$25,Assumptions!$B$26)</f>
         <v/>
       </c>
       <c r="O8" s="14">
-        <f>-O5*Assumptions!$B$24</f>
+        <f>-O5*IF(YEAR(O3)=2026,Assumptions!$B$25,Assumptions!$B$26)</f>
         <v/>
       </c>
       <c r="P8" s="14">
-        <f>-P5*Assumptions!$B$24</f>
+        <f>-P5*IF(YEAR(P3)=2026,Assumptions!$B$25,Assumptions!$B$26)</f>
         <v/>
       </c>
       <c r="Q8" s="14">
-        <f>-Q5*Assumptions!$B$24</f>
+        <f>-Q5*IF(YEAR(Q3)=2026,Assumptions!$B$25,Assumptions!$B$26)</f>
         <v/>
       </c>
       <c r="R8" s="14">
-        <f>-R5*Assumptions!$B$24</f>
+        <f>-R5*IF(YEAR(R3)=2026,Assumptions!$B$25,Assumptions!$B$26)</f>
         <v/>
       </c>
       <c r="S8" s="14">
-        <f>-S5*Assumptions!$B$24</f>
+        <f>-S5*IF(YEAR(S3)=2026,Assumptions!$B$25,Assumptions!$B$26)</f>
         <v/>
       </c>
       <c r="T8" s="14">
-        <f>-T5*Assumptions!$B$24</f>
-        <v/>
-      </c>
-      <c r="U8" s="44">
+        <f>-T5*IF(YEAR(T3)=2026,Assumptions!$B$25,Assumptions!$B$26)</f>
+        <v/>
+      </c>
+      <c r="U8" s="45">
         <f>SUM(B8:T8)</f>
         <v/>
       </c>
@@ -2049,7 +2084,7 @@
         <f>-T6*(1-Bottles!$B$22)</f>
         <v/>
       </c>
-      <c r="U9" s="44">
+      <c r="U9" s="45">
         <f>SUM(B9:T9)</f>
         <v/>
       </c>
@@ -2136,7 +2171,7 @@
         <f>T7+T8+T9</f>
         <v/>
       </c>
-      <c r="U10" s="44">
+      <c r="U10" s="45">
         <f>SUM(B10:T10)</f>
         <v/>
       </c>
@@ -2223,7 +2258,7 @@
         <f>IF(T7=0,0,T10/T7)</f>
         <v/>
       </c>
-      <c r="U11" s="45">
+      <c r="U11" s="46">
         <f>U10/U7</f>
         <v/>
       </c>
@@ -2235,82 +2270,82 @@
         </is>
       </c>
       <c r="B12" s="14">
-        <f>-(Assumptions!$B$26+IF(B$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(B$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <f>-(Assumptions!$B$29+IF(B$3&gt;=DATE(2026,9,1),SUM(Assumptions!$B$30:$B$34),0))</f>
         <v/>
       </c>
       <c r="C12" s="14">
-        <f>-(Assumptions!$B$26+IF(C$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(C$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <f>-(Assumptions!$B$29+IF(C$3&gt;=DATE(2026,9,1),SUM(Assumptions!$B$30:$B$34),0))</f>
         <v/>
       </c>
       <c r="D12" s="14">
-        <f>-(Assumptions!$B$26+IF(D$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(D$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <f>-(Assumptions!$B$29+IF(D$3&gt;=DATE(2026,9,1),SUM(Assumptions!$B$30:$B$34),0))</f>
         <v/>
       </c>
       <c r="E12" s="14">
-        <f>-(Assumptions!$B$26+IF(E$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(E$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <f>-(Assumptions!$B$29+IF(E$3&gt;=DATE(2026,9,1),SUM(Assumptions!$B$30:$B$34),0))</f>
         <v/>
       </c>
       <c r="F12" s="14">
-        <f>-(Assumptions!$B$26+IF(F$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(F$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <f>-(Assumptions!$B$29+IF(F$3&gt;=DATE(2026,9,1),SUM(Assumptions!$B$30:$B$34),0))</f>
         <v/>
       </c>
       <c r="G12" s="14">
-        <f>-(Assumptions!$B$26+IF(G$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(G$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <f>-(Assumptions!$B$29+IF(G$3&gt;=DATE(2026,9,1),SUM(Assumptions!$B$30:$B$34),0))</f>
         <v/>
       </c>
       <c r="H12" s="14">
-        <f>-(Assumptions!$B$26+IF(H$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(H$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <f>-(Assumptions!$B$29+IF(H$3&gt;=DATE(2026,9,1),SUM(Assumptions!$B$30:$B$34),0))</f>
         <v/>
       </c>
       <c r="I12" s="14">
-        <f>-(Assumptions!$B$26+IF(I$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(I$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <f>-(Assumptions!$B$29+IF(I$3&gt;=DATE(2026,9,1),SUM(Assumptions!$B$30:$B$34),0))</f>
         <v/>
       </c>
       <c r="J12" s="14">
-        <f>-(Assumptions!$B$26+IF(J$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(J$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <f>-(Assumptions!$B$29+IF(J$3&gt;=DATE(2026,9,1),SUM(Assumptions!$B$30:$B$34),0))</f>
         <v/>
       </c>
       <c r="K12" s="14">
-        <f>-(Assumptions!$B$26+IF(K$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(K$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <f>-(Assumptions!$B$29+IF(K$3&gt;=DATE(2026,9,1),SUM(Assumptions!$B$30:$B$34),0))</f>
         <v/>
       </c>
       <c r="L12" s="14">
-        <f>-(Assumptions!$B$26+IF(L$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(L$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <f>-(Assumptions!$B$29+IF(L$3&gt;=DATE(2026,9,1),SUM(Assumptions!$B$30:$B$34),0))</f>
         <v/>
       </c>
       <c r="M12" s="14">
-        <f>-(Assumptions!$B$26+IF(M$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(M$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <f>-(Assumptions!$B$29+IF(M$3&gt;=DATE(2026,9,1),SUM(Assumptions!$B$30:$B$34),0))</f>
         <v/>
       </c>
       <c r="N12" s="14">
-        <f>-(Assumptions!$B$26+IF(N$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(N$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <f>-(Assumptions!$B$29+IF(N$3&gt;=DATE(2026,9,1),SUM(Assumptions!$B$30:$B$34),0))</f>
         <v/>
       </c>
       <c r="O12" s="14">
-        <f>-(Assumptions!$B$26+IF(O$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(O$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <f>-(Assumptions!$B$29+IF(O$3&gt;=DATE(2026,9,1),SUM(Assumptions!$B$30:$B$34),0))</f>
         <v/>
       </c>
       <c r="P12" s="14">
-        <f>-(Assumptions!$B$26+IF(P$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(P$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <f>-(Assumptions!$B$29+IF(P$3&gt;=DATE(2026,9,1),SUM(Assumptions!$B$30:$B$34),0))</f>
         <v/>
       </c>
       <c r="Q12" s="14">
-        <f>-(Assumptions!$B$26+IF(Q$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(Q$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <f>-(Assumptions!$B$29+IF(Q$3&gt;=DATE(2026,9,1),SUM(Assumptions!$B$30:$B$34),0))</f>
         <v/>
       </c>
       <c r="R12" s="14">
-        <f>-(Assumptions!$B$26+IF(R$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(R$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <f>-(Assumptions!$B$29+IF(R$3&gt;=DATE(2026,9,1),SUM(Assumptions!$B$30:$B$34),0))</f>
         <v/>
       </c>
       <c r="S12" s="14">
-        <f>-(Assumptions!$B$26+IF(S$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(S$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
+        <f>-(Assumptions!$B$29+IF(S$3&gt;=DATE(2026,9,1),SUM(Assumptions!$B$30:$B$34),0))</f>
         <v/>
       </c>
       <c r="T12" s="14">
-        <f>-(Assumptions!$B$26+IF(T$3&gt;=DATE(2026,7,1),Assumptions!$B$27+Assumptions!$B$28,0)+IF(T$3&gt;=DATE(2026,8,1),Assumptions!$B$29+Assumptions!$B$30+Assumptions!$B$31,0))</f>
-        <v/>
-      </c>
-      <c r="U12" s="44">
+        <f>-(Assumptions!$B$29+IF(T$3&gt;=DATE(2026,9,1),SUM(Assumptions!$B$30:$B$34),0))</f>
+        <v/>
+      </c>
+      <c r="U12" s="45">
         <f>SUM(B12:T12)</f>
         <v/>
       </c>
@@ -2397,7 +2432,7 @@
         <f>T10+T12</f>
         <v/>
       </c>
-      <c r="U13" s="44">
+      <c r="U13" s="45">
         <f>SUM(B13:T13)</f>
         <v/>
       </c>
@@ -2484,7 +2519,7 @@
         <f>IF(T7=0,0,T13/T7)</f>
         <v/>
       </c>
-      <c r="U14" s="45">
+      <c r="U14" s="46">
         <f>U13/U7</f>
         <v/>
       </c>
@@ -2555,69 +2590,69 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="38" t="inlineStr">
+      <c r="A3" s="39" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B3" s="40" t="n">
+      <c r="B3" s="41" t="n">
         <v>46174</v>
       </c>
-      <c r="C3" s="40" t="n">
+      <c r="C3" s="41" t="n">
         <v>46204</v>
       </c>
-      <c r="D3" s="40" t="n">
+      <c r="D3" s="41" t="n">
         <v>46235</v>
       </c>
-      <c r="E3" s="40" t="n">
+      <c r="E3" s="41" t="n">
         <v>46266</v>
       </c>
-      <c r="F3" s="40" t="n">
+      <c r="F3" s="41" t="n">
         <v>46296</v>
       </c>
-      <c r="G3" s="40" t="n">
+      <c r="G3" s="41" t="n">
         <v>46327</v>
       </c>
-      <c r="H3" s="40" t="n">
+      <c r="H3" s="41" t="n">
         <v>46357</v>
       </c>
-      <c r="I3" s="40" t="n">
+      <c r="I3" s="41" t="n">
         <v>46388</v>
       </c>
-      <c r="J3" s="40" t="n">
+      <c r="J3" s="41" t="n">
         <v>46419</v>
       </c>
-      <c r="K3" s="40" t="n">
+      <c r="K3" s="41" t="n">
         <v>46447</v>
       </c>
-      <c r="L3" s="40" t="n">
+      <c r="L3" s="41" t="n">
         <v>46478</v>
       </c>
-      <c r="M3" s="40" t="n">
+      <c r="M3" s="41" t="n">
         <v>46508</v>
       </c>
-      <c r="N3" s="40" t="n">
+      <c r="N3" s="41" t="n">
         <v>46539</v>
       </c>
-      <c r="O3" s="40" t="n">
+      <c r="O3" s="41" t="n">
         <v>46569</v>
       </c>
-      <c r="P3" s="40" t="n">
+      <c r="P3" s="41" t="n">
         <v>46600</v>
       </c>
-      <c r="Q3" s="40" t="n">
+      <c r="Q3" s="41" t="n">
         <v>46631</v>
       </c>
-      <c r="R3" s="40" t="n">
+      <c r="R3" s="41" t="n">
         <v>46661</v>
       </c>
-      <c r="S3" s="40" t="n">
+      <c r="S3" s="41" t="n">
         <v>46692</v>
       </c>
-      <c r="T3" s="40" t="n">
+      <c r="T3" s="41" t="n">
         <v>46722</v>
       </c>
-      <c r="U3" s="38" t="inlineStr">
+      <c r="U3" s="39" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -2704,7 +2739,7 @@
         <f>'P&amp;L'!S5</f>
         <v/>
       </c>
-      <c r="U4" s="44">
+      <c r="U4" s="45">
         <f>SUM(B4:T4)</f>
         <v/>
       </c>
@@ -2721,7 +2756,7 @@
       <c r="D5" s="34" t="n">
         <v>-292560</v>
       </c>
-      <c r="U5" s="44">
+      <c r="U5" s="45">
         <f>SUM(B5:T5)</f>
         <v/>
       </c>
@@ -2738,7 +2773,7 @@
       <c r="F6" s="34" t="n">
         <v>-86880</v>
       </c>
-      <c r="U6" s="44">
+      <c r="U6" s="45">
         <f>SUM(B6:T6)</f>
         <v/>
       </c>
@@ -2755,7 +2790,7 @@
       <c r="E7" s="34" t="n">
         <v>-382800</v>
       </c>
-      <c r="U7" s="44">
+      <c r="U7" s="45">
         <f>SUM(B7:T7)</f>
         <v/>
       </c>
@@ -2769,7 +2804,7 @@
       <c r="B8" s="34" t="n">
         <v>-17250</v>
       </c>
-      <c r="U8" s="44">
+      <c r="U8" s="45">
         <f>SUM(B8:T8)</f>
         <v/>
       </c>
@@ -2786,7 +2821,7 @@
       <c r="F9" s="34" t="n">
         <v>-33600</v>
       </c>
-      <c r="U9" s="44">
+      <c r="U9" s="45">
         <f>SUM(B9:T9)</f>
         <v/>
       </c>
@@ -2803,7 +2838,7 @@
       <c r="E10" s="34" t="n">
         <v>-351900</v>
       </c>
-      <c r="U10" s="44">
+      <c r="U10" s="45">
         <f>SUM(B10:T10)</f>
         <v/>
       </c>
@@ -2820,7 +2855,7 @@
       <c r="G11" s="34" t="n">
         <v>-594685</v>
       </c>
-      <c r="U11" s="44">
+      <c r="U11" s="45">
         <f>SUM(B11:T11)</f>
         <v/>
       </c>
@@ -2907,7 +2942,7 @@
         <f>'P&amp;L'!T12</f>
         <v/>
       </c>
-      <c r="U12" s="44">
+      <c r="U12" s="45">
         <f>SUM(B12:T12)</f>
         <v/>
       </c>
@@ -2994,7 +3029,7 @@
         <f>'P&amp;L'!T6*Bottles!$B$22</f>
         <v/>
       </c>
-      <c r="U13" s="44">
+      <c r="U13" s="45">
         <f>SUM(B13:T13)</f>
         <v/>
       </c>
@@ -3006,54 +3041,54 @@
         </is>
       </c>
       <c r="I14" s="14">
-        <f>-'P&amp;L'!I5*Assumptions!$B$24</f>
+        <f>-'P&amp;L'!I5*Assumptions!$B$26</f>
         <v/>
       </c>
       <c r="J14" s="14">
-        <f>-'P&amp;L'!J5*Assumptions!$B$24</f>
+        <f>-'P&amp;L'!J5*Assumptions!$B$26</f>
         <v/>
       </c>
       <c r="K14" s="14">
-        <f>-'P&amp;L'!K5*Assumptions!$B$24</f>
+        <f>-'P&amp;L'!K5*Assumptions!$B$26</f>
         <v/>
       </c>
       <c r="L14" s="14">
-        <f>-'P&amp;L'!L5*Assumptions!$B$24</f>
+        <f>-'P&amp;L'!L5*Assumptions!$B$26</f>
         <v/>
       </c>
       <c r="M14" s="14">
-        <f>-'P&amp;L'!M5*Assumptions!$B$24</f>
+        <f>-'P&amp;L'!M5*Assumptions!$B$26</f>
         <v/>
       </c>
       <c r="N14" s="14">
-        <f>-'P&amp;L'!N5*Assumptions!$B$24</f>
+        <f>-'P&amp;L'!N5*Assumptions!$B$26</f>
         <v/>
       </c>
       <c r="O14" s="14">
-        <f>-'P&amp;L'!O5*Assumptions!$B$24</f>
+        <f>-'P&amp;L'!O5*Assumptions!$B$26</f>
         <v/>
       </c>
       <c r="P14" s="14">
-        <f>-'P&amp;L'!P5*Assumptions!$B$24</f>
+        <f>-'P&amp;L'!P5*Assumptions!$B$26</f>
         <v/>
       </c>
       <c r="Q14" s="14">
-        <f>-'P&amp;L'!Q5*Assumptions!$B$24</f>
+        <f>-'P&amp;L'!Q5*Assumptions!$B$26</f>
         <v/>
       </c>
       <c r="R14" s="14">
-        <f>-'P&amp;L'!R5*Assumptions!$B$24</f>
+        <f>-'P&amp;L'!R5*Assumptions!$B$26</f>
         <v/>
       </c>
       <c r="S14" s="14">
-        <f>-'P&amp;L'!S5*Assumptions!$B$24</f>
+        <f>-'P&amp;L'!S5*Assumptions!$B$26</f>
         <v/>
       </c>
       <c r="T14" s="14">
-        <f>-'P&amp;L'!T5*Assumptions!$B$24</f>
-        <v/>
-      </c>
-      <c r="U14" s="44">
+        <f>-'P&amp;L'!T5*Assumptions!$B$26</f>
+        <v/>
+      </c>
+      <c r="U14" s="45">
         <f>SUM(B14:T14)</f>
         <v/>
       </c>
@@ -3140,7 +3175,7 @@
         <f>SUM(T4:T14)</f>
         <v/>
       </c>
-      <c r="U15" s="44">
+      <c r="U15" s="45">
         <f>SUM(B15:T15)</f>
         <v/>
       </c>
@@ -3255,7 +3290,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -3360,13 +3395,13 @@
           <t>Multiple</t>
         </is>
       </c>
-      <c r="B10" s="46" t="n">
+      <c r="B10" s="47" t="n">
         <v>6</v>
       </c>
-      <c r="C10" s="46" t="n">
+      <c r="C10" s="47" t="n">
         <v>9</v>
       </c>
-      <c r="D10" s="46" t="n">
+      <c r="D10" s="47" t="n">
         <v>12</v>
       </c>
     </row>
@@ -3406,13 +3441,13 @@
           <t>Multiple</t>
         </is>
       </c>
-      <c r="B14" s="46" t="n">
+      <c r="B14" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="C14" s="46" t="n">
+      <c r="C14" s="47" t="n">
         <v>1.5</v>
       </c>
-      <c r="D14" s="46" t="n">
+      <c r="D14" s="47" t="n">
         <v>2.5</v>
       </c>
     </row>
@@ -3468,13 +3503,13 @@
           <t>Exit multiple (2027 EBITDA)</t>
         </is>
       </c>
-      <c r="B19" s="46" t="n">
+      <c r="B19" s="47" t="n">
         <v>6</v>
       </c>
-      <c r="C19" s="46" t="n">
+      <c r="C19" s="47" t="n">
         <v>8</v>
       </c>
-      <c r="D19" s="46" t="n">
+      <c r="D19" s="47" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3504,40 +3539,75 @@
           <t>Blended enterprise value (avg of methods)</t>
         </is>
       </c>
-      <c r="B22" s="39">
+      <c r="B22" s="40">
         <f>AVERAGE(B11,B15,B20)</f>
         <v/>
       </c>
-      <c r="C22" s="39">
+      <c r="C22" s="40">
         <f>AVERAGE(C11,C15,C20)</f>
         <v/>
       </c>
-      <c r="D22" s="39">
+      <c r="D22" s="40">
         <f>AVERAGE(D11,D15,D20)</f>
         <v/>
       </c>
     </row>
     <row r="23"/>
     <row r="24">
-      <c r="A24" s="38" t="inlineStr">
+      <c r="A24" s="39" t="inlineStr">
         <is>
           <t>Valuation guide for the raise</t>
         </is>
       </c>
-      <c r="B24" s="47" t="n">
+      <c r="B24" s="48" t="n">
         <v>15000000</v>
       </c>
       <c r="C24" s="26" t="n"/>
       <c r="D24" s="26" t="n"/>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>With bottles modelled off three years of actuals, the ~R15m guide equals the blended LOW case; better-than-flat reorders, new retailers and export remain outside the model.</t>
+          <t>Cost of sales improves from 76% in Year 1 to 66% in Year 2 and 60% in Year 3 as volume-based input and co-pack pricing steps down.</t>
         </is>
       </c>
     </row>
     <row r="25"/>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>2028 run-rate at Year-3 COGS</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Revenue (2027 held flat)</t>
+        </is>
+      </c>
+      <c r="B27" s="20">
+        <f>$B$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>EBITDA at Year-3 can COGS</t>
+        </is>
+      </c>
+      <c r="B28" s="14">
+        <f>SUM('P&amp;L'!I5:T5)*(1-Assumptions!$B$27)+SUM('P&amp;L'!I6:T6)*Bottles!$B$22+SUM('P&amp;L'!I12:T12)</f>
+        <v/>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Scale savings carried to Year 3; volumes held flat — the operating leverage in the plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="29"/>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>Same three methods and multiples as the tequila project model, applied to brand-entity economics.</t>
         </is>
@@ -3572,7 +3642,7 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="48" t="inlineStr">
+      <c r="A3" s="49" t="inlineStr">
         <is>
           <t>Checkers listing</t>
         </is>
@@ -3583,7 +3653,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="48" t="inlineStr">
+      <c r="A4" s="49" t="inlineStr">
         <is>
           <t>Opening order (initial fill revenue)</t>
         </is>
@@ -3594,7 +3664,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="48" t="inlineStr">
+      <c r="A5" s="49" t="inlineStr">
         <is>
           <t>Bottle revenue (Jun 26 – Dec 27)</t>
         </is>
@@ -3605,29 +3675,29 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="38" t="inlineStr">
+      <c r="A6" s="39" t="inlineStr">
         <is>
           <t>Total revenue, cans + bottles (Jun 26 – Dec 27)</t>
         </is>
       </c>
-      <c r="B6" s="44">
+      <c r="B6" s="45">
         <f>'P&amp;L'!U7</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="38" t="inlineStr">
+      <c r="A7" s="39" t="inlineStr">
         <is>
           <t>Total EBITDA (Jun 26 – Dec 27)</t>
         </is>
       </c>
-      <c r="B7" s="44">
+      <c r="B7" s="45">
         <f>'P&amp;L'!U13</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="48" t="inlineStr">
+      <c r="A8" s="49" t="inlineStr">
         <is>
           <t>EBITDA margin</t>
         </is>
@@ -3643,13 +3713,13 @@
           <t>Peak funding need</t>
         </is>
       </c>
-      <c r="B9" s="44">
+      <c r="B9" s="45">
         <f>MIN(Cashflow!B16:T16)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="48" t="inlineStr">
+      <c r="A10" s="49" t="inlineStr">
         <is>
           <t>Ending cash (Dec 27)</t>
         </is>
@@ -3660,7 +3730,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="48" t="inlineStr">
+      <c r="A11" s="49" t="inlineStr">
         <is>
           <t>Blended valuation — low</t>
         </is>
@@ -3671,7 +3741,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="48" t="inlineStr">
+      <c r="A12" s="49" t="inlineStr">
         <is>
           <t>Blended valuation — base</t>
         </is>
@@ -3682,7 +3752,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="48" t="inlineStr">
+      <c r="A13" s="49" t="inlineStr">
         <is>
           <t>Blended valuation — high</t>
         </is>
@@ -3693,12 +3763,12 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="38" t="inlineStr">
+      <c r="A14" s="39" t="inlineStr">
         <is>
           <t>Valuation guide</t>
         </is>
       </c>
-      <c r="B14" s="44">
+      <c r="B14" s="45">
         <f>Valuation!B24</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Price cans at R744 per case ex VAT
Wholesale price corrected to the ex-VAT figure (R855.60 incl VAT), which
flows through revenue, margins, cash and valuation:
- Opening order R2.41m ex VAT (3,240 cases); revenue R15.45m to Dec 27
- EBITDA R3.44m (22.3%); peak funding R1.41m; end cash R2.67m
- Blended valuation R12.4m/R17.7m/R24.8m, ~R15m guide between low and base
- Unit economics, P&L, valuation, charts, stats and copy restated; revenue
  labelled ex VAT throughout

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hyws6xeXfxtGdqZV2paNDe
</commit_message>
<xml_diff>
--- a/site/downloads/Dona-Fuego-Brand-Pro-Forma.xlsx
+++ b/site/downloads/Dona-Fuego-Brand-Pro-Forma.xlsx
@@ -154,11 +154,11 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="17" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -179,11 +179,11 @@
     <xf numFmtId="3" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="10" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="7" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="12" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="17" fontId="10" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -755,15 +755,15 @@
     <row r="16">
       <c r="A16" s="29" t="inlineStr">
         <is>
-          <t>Wholesale price per case (R)</t>
+          <t>Wholesale price per case, ex VAT (R)</t>
         </is>
       </c>
       <c r="B16" s="34" t="n">
-        <v>847.04</v>
+        <v>744</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>R169 4-pack / R49 unit retail</t>
+          <t>24-unit case; R855.60 incl VAT</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
           <t>Legal &amp; admin</t>
         </is>
       </c>
-      <c r="B29" s="34" t="n">
+      <c r="B29" s="38" t="n">
         <v>0</v>
       </c>
     </row>
@@ -918,7 +918,7 @@
           <t>Sales &amp; key accounts (1 FTE)</t>
         </is>
       </c>
-      <c r="B30" s="38" t="n">
+      <c r="B30" s="34" t="n">
         <v>40000</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -933,7 +933,7 @@
           <t>Operations &amp; merchandising coordinator</t>
         </is>
       </c>
-      <c r="B31" s="38" t="n">
+      <c r="B31" s="34" t="n">
         <v>15000</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -948,7 +948,7 @@
           <t>Trade marketing &amp; promotions</t>
         </is>
       </c>
-      <c r="B32" s="38" t="n">
+      <c r="B32" s="34" t="n">
         <v>25000</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -963,7 +963,7 @@
           <t>Brand marketing</t>
         </is>
       </c>
-      <c r="B33" s="38" t="n">
+      <c r="B33" s="34" t="n">
         <v>15000</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -978,7 +978,7 @@
           <t>Warehousing &amp; insurance</t>
         </is>
       </c>
-      <c r="B34" s="38" t="n">
+      <c r="B34" s="34" t="n">
         <v>10000</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1089,13 +1089,13 @@
           <t>January</t>
         </is>
       </c>
-      <c r="C4" s="34" t="n">
+      <c r="C4" s="38" t="n">
         <v>87354</v>
       </c>
-      <c r="D4" s="34" t="n">
+      <c r="D4" s="38" t="n">
         <v>107377.8</v>
       </c>
-      <c r="E4" s="34" t="n">
+      <c r="E4" s="38" t="n">
         <v>185865.3</v>
       </c>
       <c r="G4" s="14">
@@ -1109,13 +1109,13 @@
           <t>February</t>
         </is>
       </c>
-      <c r="C5" s="34" t="n">
+      <c r="C5" s="38" t="n">
         <v>7728</v>
       </c>
-      <c r="D5" s="34" t="n">
+      <c r="D5" s="38" t="n">
         <v>46920</v>
       </c>
-      <c r="E5" s="34" t="n">
+      <c r="E5" s="38" t="n">
         <v>209857.2</v>
       </c>
       <c r="G5" s="14">
@@ -1129,10 +1129,10 @@
           <t>March</t>
         </is>
       </c>
-      <c r="D6" s="34" t="n">
+      <c r="D6" s="38" t="n">
         <v>126617.4</v>
       </c>
-      <c r="E6" s="34" t="n">
+      <c r="E6" s="38" t="n">
         <v>260918.59</v>
       </c>
       <c r="G6" s="14">
@@ -1146,13 +1146,13 @@
           <t>April</t>
         </is>
       </c>
-      <c r="C7" s="34" t="n">
+      <c r="C7" s="38" t="n">
         <v>21931.51</v>
       </c>
-      <c r="D7" s="34" t="n">
+      <c r="D7" s="38" t="n">
         <v>663918</v>
       </c>
-      <c r="E7" s="34" t="n">
+      <c r="E7" s="38" t="n">
         <v>470561.32</v>
       </c>
       <c r="G7" s="14">
@@ -1166,13 +1166,13 @@
           <t>May</t>
         </is>
       </c>
-      <c r="C8" s="34" t="n">
+      <c r="C8" s="38" t="n">
         <v>1895.8</v>
       </c>
-      <c r="D8" s="34" t="n">
+      <c r="D8" s="38" t="n">
         <v>168670.5</v>
       </c>
-      <c r="E8" s="34" t="n">
+      <c r="E8" s="38" t="n">
         <v>167687.8</v>
       </c>
       <c r="G8" s="14">
@@ -1186,13 +1186,13 @@
           <t>June</t>
         </is>
       </c>
-      <c r="C9" s="34" t="n">
+      <c r="C9" s="38" t="n">
         <v>68533.21000000001</v>
       </c>
-      <c r="D9" s="34" t="n">
+      <c r="D9" s="38" t="n">
         <v>98574.11</v>
       </c>
-      <c r="E9" s="34" t="n">
+      <c r="E9" s="38" t="n">
         <v>60059.82</v>
       </c>
       <c r="G9" s="14">
@@ -1206,13 +1206,13 @@
           <t>July</t>
         </is>
       </c>
-      <c r="C10" s="34" t="n">
+      <c r="C10" s="38" t="n">
         <v>36027.3</v>
       </c>
-      <c r="D10" s="34" t="n">
+      <c r="D10" s="38" t="n">
         <v>266641.05</v>
       </c>
-      <c r="E10" s="34" t="n">
+      <c r="E10" s="38" t="n">
         <v>188654.34</v>
       </c>
       <c r="G10" s="14">
@@ -1226,10 +1226,10 @@
           <t>August</t>
         </is>
       </c>
-      <c r="C11" s="34" t="n">
+      <c r="C11" s="38" t="n">
         <v>5796</v>
       </c>
-      <c r="D11" s="34" t="n">
+      <c r="D11" s="38" t="n">
         <v>44441.56</v>
       </c>
       <c r="E11" s="14">
@@ -1247,13 +1247,13 @@
           <t>September</t>
         </is>
       </c>
-      <c r="B12" s="34" t="n">
+      <c r="B12" s="38" t="n">
         <v>1334</v>
       </c>
-      <c r="C12" s="34" t="n">
+      <c r="C12" s="38" t="n">
         <v>46252.59</v>
       </c>
-      <c r="D12" s="34" t="n">
+      <c r="D12" s="38" t="n">
         <v>65847.11</v>
       </c>
       <c r="E12" s="14">
@@ -1271,13 +1271,13 @@
           <t>October</t>
         </is>
       </c>
-      <c r="B13" s="34" t="n">
+      <c r="B13" s="38" t="n">
         <v>2894</v>
       </c>
-      <c r="C13" s="34" t="n">
+      <c r="C13" s="38" t="n">
         <v>530949.8100000001</v>
       </c>
-      <c r="D13" s="34" t="n">
+      <c r="D13" s="38" t="n">
         <v>63268.38</v>
       </c>
       <c r="E13" s="14">
@@ -1295,10 +1295,10 @@
           <t>November</t>
         </is>
       </c>
-      <c r="C14" s="34" t="n">
+      <c r="C14" s="38" t="n">
         <v>81964.75</v>
       </c>
-      <c r="D14" s="34" t="n">
+      <c r="D14" s="38" t="n">
         <v>257848.55</v>
       </c>
       <c r="E14" s="14">
@@ -1316,13 +1316,13 @@
           <t>December</t>
         </is>
       </c>
-      <c r="B15" s="34" t="n">
+      <c r="B15" s="38" t="n">
         <v>21919</v>
       </c>
-      <c r="C15" s="34" t="n">
+      <c r="C15" s="38" t="n">
         <v>138333.09</v>
       </c>
-      <c r="D15" s="34" t="n">
+      <c r="D15" s="38" t="n">
         <v>35332.6</v>
       </c>
       <c r="E15" s="14">
@@ -2750,10 +2750,10 @@
           <t xml:space="preserve">  Bron Pro (design/brand)</t>
         </is>
       </c>
-      <c r="B5" s="34" t="n">
+      <c r="B5" s="38" t="n">
         <v>-124200</v>
       </c>
-      <c r="D5" s="34" t="n">
+      <c r="D5" s="38" t="n">
         <v>-292560</v>
       </c>
       <c r="U5" s="45">
@@ -2767,10 +2767,10 @@
           <t xml:space="preserve">  Sullwaldt printing</t>
         </is>
       </c>
-      <c r="C6" s="34" t="n">
+      <c r="C6" s="38" t="n">
         <v>-109279</v>
       </c>
-      <c r="F6" s="34" t="n">
+      <c r="F6" s="38" t="n">
         <v>-86880</v>
       </c>
       <c r="U6" s="45">
@@ -2784,10 +2784,10 @@
           <t xml:space="preserve">  Tiny Keg cans</t>
         </is>
       </c>
-      <c r="C7" s="34" t="n">
+      <c r="C7" s="38" t="n">
         <v>-487140</v>
       </c>
-      <c r="E7" s="34" t="n">
+      <c r="E7" s="38" t="n">
         <v>-382800</v>
       </c>
       <c r="U7" s="45">
@@ -2801,7 +2801,7 @@
           <t xml:space="preserve">  Chep pallets</t>
         </is>
       </c>
-      <c r="B8" s="34" t="n">
+      <c r="B8" s="38" t="n">
         <v>-17250</v>
       </c>
       <c r="U8" s="45">
@@ -2815,10 +2815,10 @@
           <t xml:space="preserve">  FAL distribution</t>
         </is>
       </c>
-      <c r="C9" s="34" t="n">
+      <c r="C9" s="38" t="n">
         <v>-62100</v>
       </c>
-      <c r="F9" s="34" t="n">
+      <c r="F9" s="38" t="n">
         <v>-33600</v>
       </c>
       <c r="U9" s="45">
@@ -2832,10 +2832,10 @@
           <t xml:space="preserve">  Tiny Keg production</t>
         </is>
       </c>
-      <c r="D10" s="34" t="n">
+      <c r="D10" s="38" t="n">
         <v>-448020</v>
       </c>
-      <c r="E10" s="34" t="n">
+      <c r="E10" s="38" t="n">
         <v>-351900</v>
       </c>
       <c r="U10" s="45">
@@ -2849,10 +2849,10 @@
           <t xml:space="preserve">  SARS excise (launch)</t>
         </is>
       </c>
-      <c r="E11" s="34" t="n">
+      <c r="E11" s="38" t="n">
         <v>-756000</v>
       </c>
-      <c r="G11" s="34" t="n">
+      <c r="G11" s="38" t="n">
         <v>-594685</v>
       </c>
       <c r="U11" s="45">

</xml_diff>